<commit_message>
Ledgr: update my-money.xlsx (2026-07-18T00:30:08.275Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -6,8 +6,10 @@
     <sheet name="Income" sheetId="1" r:id="rId1"/>
     <sheet name="Expenses" sheetId="2" r:id="rId2"/>
     <sheet name="Investments" sheetId="3" r:id="rId3"/>
-    <sheet name="Debts" sheetId="4" r:id="rId4"/>
-    <sheet name="Settings" sheetId="5" r:id="rId5"/>
+    <sheet name="Loans" sheetId="4" r:id="rId4"/>
+    <sheet name="Loan Payments" sheetId="5" r:id="rId5"/>
+    <sheet name="Debts" sheetId="6" r:id="rId6"/>
+    <sheet name="Settings" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -849,6 +851,88 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H1"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="22.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="26.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Date</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Lender</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Type</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Principal</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Interest Rate</v>
+      </c>
+      <c r="F1" t="str">
+        <v>EMI</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Tenure Months</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E1"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="22.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="26.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Date</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Lender</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Kind</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Amount</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G4"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
@@ -959,7 +1043,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B5"/>
   <cols>
@@ -988,7 +1072,7 @@
         <v>Owner</v>
       </c>
       <c r="B3" t="str">
-        <v>Demo</v>
+        <v>Sanjo</v>
       </c>
     </row>
     <row r="4">
@@ -996,7 +1080,7 @@
         <v>Username</v>
       </c>
       <c r="B4" t="str">
-        <v>demo</v>
+        <v>Galaxia</v>
       </c>
     </row>
     <row r="5">
@@ -1004,7 +1088,7 @@
         <v>PasswordHash</v>
       </c>
       <c r="B5" t="str">
-        <v>sha256:ea0bd84a1d3eedca161bd5f8545e920540186ebc95011a68299eb8f495cb0dd2</v>
+        <v>sha256:1e11cf916d3d116527ae1a9f6b50fb3a88f424ab8d22ef339d0b48b07429624f</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-18T00:35:36.541Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -851,7 +851,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -889,9 +889,35 @@
         <v>Notes</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="B2" t="str">
+        <v>SBI Home Loan</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Housing</v>
+      </c>
+      <c r="D2">
+        <v>5758624</v>
+      </c>
+      <c r="E2">
+        <v>7.3</v>
+      </c>
+      <c r="F2">
+        <v>38728</v>
+      </c>
+      <c r="G2">
+        <v>342</v>
+      </c>
+      <c r="H2" t="str">
+        <v>43716460547</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-18T00:45:47.546Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -9,7 +9,8 @@
     <sheet name="Loans" sheetId="4" r:id="rId4"/>
     <sheet name="Loan Payments" sheetId="5" r:id="rId5"/>
     <sheet name="Debts" sheetId="6" r:id="rId6"/>
-    <sheet name="Settings" sheetId="7" r:id="rId7"/>
+    <sheet name="Lists" sheetId="7" r:id="rId7"/>
+    <sheet name="Settings" sheetId="8" r:id="rId8"/>
   </sheets>
 </workbook>
 </file>
@@ -1071,7 +1072,246 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:E13"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Income Categories</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Expense Categories</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Payment Methods</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Investment Types</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Loan Types</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Salary</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Groceries</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Card</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Stocks</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Housing</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Business</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Rent / Housing</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Funds</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Car</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Freelance</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Utilities</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Bank transfer</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Real estate</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Personal</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Rental</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Transport</v>
+      </c>
+      <c r="C5" t="str">
+        <v>GPay</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Gold</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Education</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Dividends / Profit</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Dining</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Other</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Sukuk / Bonds</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Gold</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Gift</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Health</v>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v>Crypto</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Other</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Other</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Education</v>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v>Business</v>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v/>
+      </c>
+      <c r="B9" t="str">
+        <v>Shopping</v>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v>Other</v>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v/>
+      </c>
+      <c r="B10" t="str">
+        <v>Travel</v>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v/>
+      </c>
+      <c r="B11" t="str">
+        <v>Family</v>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v/>
+      </c>
+      <c r="B12" t="str">
+        <v>Other</v>
+      </c>
+      <c r="C12" t="str">
+        <v/>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v/>
+      </c>
+      <c r="B13" t="str">
+        <v>Credit Card</v>
+      </c>
+      <c r="C13" t="str">
+        <v/>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E13"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B6"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="70.83203125" customWidth="1"/>
@@ -1117,9 +1357,17 @@
         <v>sha256:1e11cf916d3d116527ae1a9f6b50fb3a88f424ab8d22ef339d0b48b07429624f</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Theme</v>
+      </c>
+      <c r="B6" t="str">
+        <v>dark</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-18T01:44:34.111Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -405,7 +405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E2"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-26</v>
+        <v>2026-07-01</v>
       </c>
       <c r="B2" t="str">
         <v>Monthly salary</v>
@@ -442,66 +442,15 @@
         <v>Salary</v>
       </c>
       <c r="D2">
-        <v>14500</v>
+        <v>115000</v>
       </c>
       <c r="E2" t="str">
-        <v>June payroll</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>2026-07-04</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Freelance web project</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Freelance</v>
-      </c>
-      <c r="D3">
-        <v>2800</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Client: design studio</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>2026-07-09</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Fund distribution</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Dividends / Profit</v>
-      </c>
-      <c r="D4">
-        <v>650</v>
-      </c>
-      <c r="E4" t="str">
-        <v>SNB Capital fund</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>2026-07-26</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Monthly salary</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Salary</v>
-      </c>
-      <c r="D5">
-        <v>145000</v>
-      </c>
-      <c r="E5" t="str">
         <v>July payroll</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-18T01:45:06.571Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -457,7 +457,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E1"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -483,179 +483,9 @@
         <v>Payment Method</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>2026-06-30</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Rent / Housing</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Apartment rent - July</v>
-      </c>
-      <c r="D2">
-        <v>3500</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Bank transfer</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>2026-07-02</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Groceries</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Panda supermarket</v>
-      </c>
-      <c r="D3">
-        <v>420</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Card</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>2026-07-05</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Transport</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Petrol</v>
-      </c>
-      <c r="D4">
-        <v>180</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Apple Pay / STC Pay</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>2026-07-07</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Dining</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Dinner with family</v>
-      </c>
-      <c r="D5">
-        <v>260</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Card</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>2026-07-11</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Utilities</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Electricity bill</v>
-      </c>
-      <c r="D6">
-        <v>310</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Bank transfer</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>2026-07-14</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Groceries</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Tamimi Markets</v>
-      </c>
-      <c r="D7">
-        <v>385</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Card</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>2026-06-27</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Health</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Pharmacy</v>
-      </c>
-      <c r="D8">
-        <v>120</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Cash</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>2026-06-19</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Shopping</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Clothes - Riyadh Park</v>
-      </c>
-      <c r="D9">
-        <v>540</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Card</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>2026-05-17</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Travel</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Weekend trip - AlUla</v>
-      </c>
-      <c r="D10">
-        <v>1450</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Card</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>2026-05-01</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Rent / Housing</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Apartment rent - May</v>
-      </c>
-      <c r="D11">
-        <v>3500</v>
-      </c>
-      <c r="E11" t="str">
-        <v>Bank transfer</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-18T01:46:59.470Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -457,7 +457,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -483,9 +483,26 @@
         <v>Payment Method</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>2026-07-17</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Recharge</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Amma</v>
+      </c>
+      <c r="D2">
+        <v>211</v>
+      </c>
+      <c r="E2" t="str">
+        <v>GPay</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -851,7 +868,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -1081,9 +1098,26 @@
         <v/>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v/>
+      </c>
+      <c r="B14" t="str">
+        <v>Recharge</v>
+      </c>
+      <c r="C14" t="str">
+        <v/>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E14"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-18T01:47:59.611Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -457,7 +457,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E1"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -483,26 +483,9 @@
         <v>Payment Method</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>2026-07-17</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Recharge</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Amma</v>
-      </c>
-      <c r="D2">
-        <v>211</v>
-      </c>
-      <c r="E2" t="str">
-        <v>GPay</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -756,7 +739,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -859,16 +842,39 @@
         <v>Fully settled</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>2026-07-13</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Jomisha</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Given</v>
+      </c>
+      <c r="D5">
+        <v>5000</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E13"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -1098,26 +1104,9 @@
         <v/>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v/>
-      </c>
-      <c r="B14" t="str">
-        <v>Recharge</v>
-      </c>
-      <c r="C14" t="str">
-        <v/>
-      </c>
-      <c r="D14" t="str">
-        <v/>
-      </c>
-      <c r="E14" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E13"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-18T01:48:10.601Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -739,7 +739,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G2"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -775,99 +775,30 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-05-09</v>
+        <v>2026-07-13</v>
       </c>
       <c r="B2" t="str">
-        <v>Khalid (friend)</v>
+        <v>Jomisha</v>
       </c>
       <c r="C2" t="str">
         <v>Given</v>
       </c>
       <c r="D2">
-        <v>2000</v>
+        <v>5000</v>
       </c>
       <c r="E2">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-08-31</v>
+        <v/>
       </c>
       <c r="G2" t="str">
-        <v>Helped with car repair</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>2026-03-14</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Brother</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Taken</v>
-      </c>
-      <c r="D3">
-        <v>5000</v>
-      </c>
-      <c r="E3">
-        <v>1000</v>
-      </c>
-      <c r="F3" t="str">
-        <v>2026-12-30</v>
-      </c>
-      <c r="G3" t="str">
-        <v>Borrowed for furniture</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>2026-05-31</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Colleague Omar</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Given</v>
-      </c>
-      <c r="D4">
-        <v>800</v>
-      </c>
-      <c r="E4">
-        <v>800</v>
-      </c>
-      <c r="F4" t="str">
-        <v/>
-      </c>
-      <c r="G4" t="str">
-        <v>Fully settled</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>2026-07-13</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Jomisha</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Given</v>
-      </c>
-      <c r="D5">
-        <v>5000</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5" t="str">
-        <v/>
-      </c>
-      <c r="G5" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-18T11:35:02.727Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -457,7 +457,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -483,9 +483,26 @@
         <v>Payment Method</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>2026-07-18</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Gst</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Gast filing fee</v>
+      </c>
+      <c r="D2">
+        <v>500</v>
+      </c>
+      <c r="E2" t="str">
+        <v>GPay</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -805,7 +822,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -1035,9 +1052,26 @@
         <v/>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v/>
+      </c>
+      <c r="B14" t="str">
+        <v>Gst</v>
+      </c>
+      <c r="C14" t="str">
+        <v/>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E14"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-18T11:58:19.035Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -509,7 +509,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F1"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -539,109 +539,9 @@
         <v>Notes</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>2025-03-09</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Al Rajhi Bank shares</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Stocks</v>
-      </c>
-      <c r="D2">
-        <v>15000</v>
-      </c>
-      <c r="E2">
-        <v>17250</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Tadawul: 1120</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>2025-06-01</v>
-      </c>
-      <c r="B3" t="str">
-        <v>SNB Capital equity fund</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Funds</v>
-      </c>
-      <c r="D3">
-        <v>20000</v>
-      </c>
-      <c r="E3">
-        <v>21100</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Monthly SIP</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>2025-09-14</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Gold bars (50g)</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Gold</v>
-      </c>
-      <c r="D4">
-        <v>12500</v>
-      </c>
-      <c r="E4">
-        <v>14200</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Kept in bank locker</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>2026-01-04</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Sukuk - Gov 2029</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Sukuk / Bonds</v>
-      </c>
-      <c r="D5">
-        <v>25000</v>
-      </c>
-      <c r="E5">
-        <v>25400</v>
-      </c>
-      <c r="F5" t="str">
-        <v>4.1% profit rate</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>2026-04-19</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Aramco shares</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Stocks</v>
-      </c>
-      <c r="D6">
-        <v>10000</v>
-      </c>
-      <c r="E6">
-        <v>9650</v>
-      </c>
-      <c r="F6" t="str">
-        <v>Tadawul: 2222</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-18T12:01:39.359Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -405,7 +405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -442,15 +442,32 @@
         <v>Salary</v>
       </c>
       <c r="D2">
-        <v>115000</v>
+        <v>113175</v>
       </c>
       <c r="E2" t="str">
         <v>July payroll</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B3" t="str">
+        <v>perdim and allowance</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Allowance</v>
+      </c>
+      <c r="D3">
+        <v>105229</v>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -869,7 +886,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v/>
+        <v>Allowance</v>
       </c>
       <c r="B9" t="str">
         <v>Shopping</v>
@@ -1021,7 +1038,7 @@
         <v>PasswordHash</v>
       </c>
       <c r="B5" t="str">
-        <v>sha256:1e11cf916d3d116527ae1a9f6b50fb3a88f424ab8d22ef339d0b48b07429624f</v>
+        <v>sha256:0c627b0cccbfc96bd1b66b9dc10e3fbd23fc91d3f23a8b4506293980448eddf8</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-18T12:03:32.267Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -474,7 +474,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E4"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -517,9 +517,43 @@
         <v>GPay</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Credit Card</v>
+      </c>
+      <c r="C3" t="str">
+        <v>axis credit card</v>
+      </c>
+      <c r="D3">
+        <v>58865</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Gpay</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Credit Card</v>
+      </c>
+      <c r="C4" t="str">
+        <v>icici</v>
+      </c>
+      <c r="D4">
+        <v>17929</v>
+      </c>
+      <c r="E4" t="str">
+        <v>GPay</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-18T12:07:13.080Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -405,7 +405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -465,16 +465,33 @@
         <v/>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>2026-07-04</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Jomisha</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Other</v>
+      </c>
+      <c r="D4">
+        <v>1000</v>
+      </c>
+      <c r="E4" t="str">
+        <v>old debt repay</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E7"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -551,9 +568,60 @@
         <v>GPay</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>2026-07-03</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Family</v>
+      </c>
+      <c r="C5" t="str">
+        <v>AMMA weekly</v>
+      </c>
+      <c r="D5">
+        <v>2000</v>
+      </c>
+      <c r="E5" t="str">
+        <v>GPay</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>2026-07-03</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Family</v>
+      </c>
+      <c r="C6" t="str">
+        <v>anusha passam</v>
+      </c>
+      <c r="D6">
+        <v>2500</v>
+      </c>
+      <c r="E6" t="str">
+        <v>GPay</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>2026-07-17</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Utilities</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Amma Recharge</v>
+      </c>
+      <c r="D7">
+        <v>211</v>
+      </c>
+      <c r="E7" t="str">
+        <v>GPay</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-18T12:11:33.326Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -405,7 +405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -482,16 +482,33 @@
         <v>old debt repay</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Repayment -Shilpa</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Other</v>
+      </c>
+      <c r="D5">
+        <v>15000</v>
+      </c>
+      <c r="E5" t="str">
+        <v>old debt repay</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -619,9 +636,26 @@
         <v>GPay</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>2026-07-08</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Loan HDFC- Shibin</v>
+      </c>
+      <c r="C8" t="str">
+        <v>land loan repayment</v>
+      </c>
+      <c r="D8">
+        <v>5891</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Bank transfer</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -841,7 +875,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -1088,9 +1122,26 @@
         <v/>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v/>
+      </c>
+      <c r="B15" t="str">
+        <v>Loan HDFC- Shibin</v>
+      </c>
+      <c r="C15" t="str">
+        <v/>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E15"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-18T12:15:20.903Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -508,7 +508,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -653,16 +653,33 @@
         <v>Bank transfer</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>2026-07-05</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Utilities</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Recharge mobile</v>
+      </c>
+      <c r="D9">
+        <v>861</v>
+      </c>
+      <c r="E9" t="str">
+        <v>GPay</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F4"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -692,9 +709,69 @@
         <v>Notes</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>APY</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Funds</v>
+      </c>
+      <c r="D2">
+        <v>409</v>
+      </c>
+      <c r="E2">
+        <v>409</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Pention fund</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>2026-07-05</v>
+      </c>
+      <c r="B3" t="str">
+        <v>coin by zerodha</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Stocks</v>
+      </c>
+      <c r="D3">
+        <v>1996</v>
+      </c>
+      <c r="E3">
+        <v>1996</v>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>2026-07-05</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Coin by zerodha</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Stocks</v>
+      </c>
+      <c r="D4">
+        <v>1331</v>
+      </c>
+      <c r="E4">
+        <v>1331</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -809,7 +886,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -866,9 +943,32 @@
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Baby Antony</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Given</v>
+      </c>
+      <c r="D3">
+        <v>25000</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-18T12:15:31.354Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -508,7 +508,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -670,9 +670,26 @@
         <v>GPay</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>2026-07-09</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Utilities</v>
+      </c>
+      <c r="C10" t="str">
+        <v>recharge airtel</v>
+      </c>
+      <c r="D10">
+        <v>199</v>
+      </c>
+      <c r="E10" t="str">
+        <v>GPay</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E10"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-18T12:19:14.438Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -405,7 +405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E9"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -499,16 +499,84 @@
         <v>old debt repay</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>2026-07-09</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Divident</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Dividends / Profit</v>
+      </c>
+      <c r="D6">
+        <v>78</v>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>2026-07-10</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Tata power</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Dividends / Profit</v>
+      </c>
+      <c r="D7">
+        <v>150</v>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>2026-07-15</v>
+      </c>
+      <c r="B8" t="str">
+        <v>excide</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Dividends / Profit</v>
+      </c>
+      <c r="D8">
+        <v>50</v>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>2026-07-18</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Credit card purchase payment</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Credit card use</v>
+      </c>
+      <c r="D9">
+        <v>33105</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Icic- 6002</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -687,9 +755,26 @@
         <v>GPay</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>2026-07-09</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Family</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Weekly expense</v>
+      </c>
+      <c r="D11">
+        <v>2500</v>
+      </c>
+      <c r="E11" t="str">
+        <v>GPay</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1156,7 +1241,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v/>
+        <v>Credit card use</v>
       </c>
       <c r="B10" t="str">
         <v>Travel</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-18T14:43:36.008Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -852,7 +852,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -963,16 +963,33 @@
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>hdfc</v>
+      </c>
+      <c r="B7" t="str">
+        <v>122321311</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Savings</v>
+      </c>
+      <c r="D7">
+        <v>11075</v>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -998,9 +1015,26 @@
         <v>Reference / Notes</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="B2" t="str">
+        <v>HDFC-ALUVA</v>
+      </c>
+      <c r="C2" t="str">
+        <v>ICICI Current</v>
+      </c>
+      <c r="D2">
+        <v>1000</v>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-18T14:54:43.832Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -413,7 +413,8 @@
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
     <col min="3" max="3" width="16.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="26.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="26.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -449,6 +450,9 @@
       <c r="D2">
         <v>113175</v>
       </c>
+      <c r="E2" t="str">
+        <v>HDFC Savings</v>
+      </c>
       <c r="F2" t="str">
         <v>July payroll</v>
       </c>
@@ -466,6 +470,9 @@
       <c r="D3">
         <v>105229</v>
       </c>
+      <c r="E3" t="str">
+        <v>HDFC Savings</v>
+      </c>
       <c r="F3" t="str">
         <v/>
       </c>
@@ -483,6 +490,9 @@
       <c r="D4">
         <v>1000</v>
       </c>
+      <c r="E4" t="str">
+        <v>HDFC Savings</v>
+      </c>
       <c r="F4" t="str">
         <v>old debt repay</v>
       </c>
@@ -500,6 +510,9 @@
       <c r="D5">
         <v>15000</v>
       </c>
+      <c r="E5" t="str">
+        <v>HDFC Savings</v>
+      </c>
       <c r="F5" t="str">
         <v>old debt repay</v>
       </c>
@@ -517,6 +530,9 @@
       <c r="D6">
         <v>78</v>
       </c>
+      <c r="E6" t="str">
+        <v>HDFC Savings</v>
+      </c>
       <c r="F6" t="str">
         <v/>
       </c>
@@ -534,6 +550,9 @@
       <c r="D7">
         <v>150</v>
       </c>
+      <c r="E7" t="str">
+        <v>HDFC Savings</v>
+      </c>
       <c r="F7" t="str">
         <v/>
       </c>
@@ -551,6 +570,9 @@
       <c r="D8">
         <v>50</v>
       </c>
+      <c r="E8" t="str">
+        <v>HDFC Savings</v>
+      </c>
       <c r="F8" t="str">
         <v/>
       </c>
@@ -567,6 +589,9 @@
       </c>
       <c r="D9">
         <v>33105</v>
+      </c>
+      <c r="E9" t="str">
+        <v>HDFC Savings</v>
       </c>
       <c r="F9" t="str">
         <v>Icic- 6002</v>
@@ -650,7 +675,8 @@
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
     <col min="3" max="3" width="28.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -686,6 +712,9 @@
       <c r="D2">
         <v>500</v>
       </c>
+      <c r="E2" t="str">
+        <v>HDFC Savings</v>
+      </c>
       <c r="F2" t="str">
         <v>GPay</v>
       </c>
@@ -703,6 +732,9 @@
       <c r="D3">
         <v>58865</v>
       </c>
+      <c r="E3" t="str">
+        <v>HDFC Savings</v>
+      </c>
       <c r="F3" t="str">
         <v>Gpay</v>
       </c>
@@ -720,6 +752,9 @@
       <c r="D4">
         <v>17929</v>
       </c>
+      <c r="E4" t="str">
+        <v>HDFC Savings</v>
+      </c>
       <c r="F4" t="str">
         <v>GPay</v>
       </c>
@@ -737,6 +772,9 @@
       <c r="D5">
         <v>2000</v>
       </c>
+      <c r="E5" t="str">
+        <v>HDFC Savings</v>
+      </c>
       <c r="F5" t="str">
         <v>GPay</v>
       </c>
@@ -754,6 +792,9 @@
       <c r="D6">
         <v>2500</v>
       </c>
+      <c r="E6" t="str">
+        <v>HDFC Savings</v>
+      </c>
       <c r="F6" t="str">
         <v>GPay</v>
       </c>
@@ -771,6 +812,9 @@
       <c r="D7">
         <v>211</v>
       </c>
+      <c r="E7" t="str">
+        <v>HDFC Savings</v>
+      </c>
       <c r="F7" t="str">
         <v>GPay</v>
       </c>
@@ -788,6 +832,9 @@
       <c r="D8">
         <v>5891</v>
       </c>
+      <c r="E8" t="str">
+        <v>HDFC Savings</v>
+      </c>
       <c r="F8" t="str">
         <v>Bank transfer</v>
       </c>
@@ -805,6 +852,9 @@
       <c r="D9">
         <v>861</v>
       </c>
+      <c r="E9" t="str">
+        <v>HDFC Savings</v>
+      </c>
       <c r="F9" t="str">
         <v>GPay</v>
       </c>
@@ -822,6 +872,9 @@
       <c r="D10">
         <v>199</v>
       </c>
+      <c r="E10" t="str">
+        <v>HDFC Savings</v>
+      </c>
       <c r="F10" t="str">
         <v>GPay</v>
       </c>
@@ -838,6 +891,9 @@
       </c>
       <c r="D11">
         <v>2500</v>
+      </c>
+      <c r="E11" t="str">
+        <v>HDFC Savings</v>
       </c>
       <c r="F11" t="str">
         <v>GPay</v>
@@ -852,7 +908,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -980,16 +1036,33 @@
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>HDFR</v>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
+        <v>Savings</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E1"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -1015,26 +1088,9 @@
         <v>Reference / Notes</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>2026-07-02</v>
-      </c>
-      <c r="B2" t="str">
-        <v>HDFC-ALUVA</v>
-      </c>
-      <c r="C2" t="str">
-        <v>ICICI Current</v>
-      </c>
-      <c r="D2">
-        <v>1000</v>
-      </c>
-      <c r="E2" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-18T15:50:48.913Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -5,14 +5,12 @@
   <sheets>
     <sheet name="Income" sheetId="1" r:id="rId1"/>
     <sheet name="Expenses" sheetId="2" r:id="rId2"/>
-    <sheet name="Banks" sheetId="3" r:id="rId3"/>
-    <sheet name="Transfers" sheetId="4" r:id="rId4"/>
-    <sheet name="Investments" sheetId="5" r:id="rId5"/>
-    <sheet name="Loans" sheetId="6" r:id="rId6"/>
-    <sheet name="Loan Payments" sheetId="7" r:id="rId7"/>
-    <sheet name="Debts" sheetId="8" r:id="rId8"/>
-    <sheet name="Lists" sheetId="9" r:id="rId9"/>
-    <sheet name="Settings" sheetId="10" r:id="rId10"/>
+    <sheet name="Investments" sheetId="3" r:id="rId3"/>
+    <sheet name="Loans" sheetId="4" r:id="rId4"/>
+    <sheet name="Loan Payments" sheetId="5" r:id="rId5"/>
+    <sheet name="Debts" sheetId="6" r:id="rId6"/>
+    <sheet name="Lists" sheetId="7" r:id="rId7"/>
+    <sheet name="Settings" sheetId="8" r:id="rId8"/>
   </sheets>
 </workbook>
 </file>
@@ -407,14 +405,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:E9"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
     <col min="3" max="3" width="16.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="26.83203125" customWidth="1"/>
+    <col min="5" max="5" width="26.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -431,9 +428,6 @@
         <v>Amount</v>
       </c>
       <c r="E1" t="str">
-        <v>Bank</v>
-      </c>
-      <c r="F1" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -448,12 +442,9 @@
         <v>Salary</v>
       </c>
       <c r="D2">
-        <v>113175</v>
+        <v>113</v>
       </c>
       <c r="E2" t="str">
-        <v>HDFC Savings</v>
-      </c>
-      <c r="F2" t="str">
         <v>July payroll</v>
       </c>
     </row>
@@ -468,12 +459,9 @@
         <v>Allowance</v>
       </c>
       <c r="D3">
-        <v>105229</v>
+        <v>105</v>
       </c>
       <c r="E3" t="str">
-        <v>HDFC Savings</v>
-      </c>
-      <c r="F3" t="str">
         <v/>
       </c>
     </row>
@@ -491,9 +479,6 @@
         <v>1000</v>
       </c>
       <c r="E4" t="str">
-        <v>HDFC Savings</v>
-      </c>
-      <c r="F4" t="str">
         <v>old debt repay</v>
       </c>
     </row>
@@ -511,9 +496,6 @@
         <v>15000</v>
       </c>
       <c r="E5" t="str">
-        <v>HDFC Savings</v>
-      </c>
-      <c r="F5" t="str">
         <v>old debt repay</v>
       </c>
     </row>
@@ -531,9 +513,6 @@
         <v>78</v>
       </c>
       <c r="E6" t="str">
-        <v>HDFC Savings</v>
-      </c>
-      <c r="F6" t="str">
         <v/>
       </c>
     </row>
@@ -551,9 +530,6 @@
         <v>150</v>
       </c>
       <c r="E7" t="str">
-        <v>HDFC Savings</v>
-      </c>
-      <c r="F7" t="str">
         <v/>
       </c>
     </row>
@@ -571,9 +547,6 @@
         <v>50</v>
       </c>
       <c r="E8" t="str">
-        <v>HDFC Savings</v>
-      </c>
-      <c r="F8" t="str">
         <v/>
       </c>
     </row>
@@ -591,92 +564,25 @@
         <v>33105</v>
       </c>
       <c r="E9" t="str">
-        <v>HDFC Savings</v>
-      </c>
-      <c r="F9" t="str">
         <v>Icic- 6002</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F9"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B6"/>
-  <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="70.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Key</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Value</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Currency</v>
-      </c>
-      <c r="B2" t="str">
-        <v>INR</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Owner</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Sanjo</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Username</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Galaxia</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>PasswordHash</v>
-      </c>
-      <c r="B5" t="str">
-        <v>sha256:0c627b0cccbfc96bd1b66b9dc10e3fbd23fc91d3f23a8b4506293980448eddf8</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Theme</v>
-      </c>
-      <c r="B6" t="str">
-        <v>dark</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:E11"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
     <col min="3" max="3" width="28.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -693,9 +599,6 @@
         <v>Amount</v>
       </c>
       <c r="E1" t="str">
-        <v>Bank</v>
-      </c>
-      <c r="F1" t="str">
         <v>Payment Method</v>
       </c>
     </row>
@@ -713,9 +616,6 @@
         <v>500</v>
       </c>
       <c r="E2" t="str">
-        <v>HDFC Savings</v>
-      </c>
-      <c r="F2" t="str">
         <v>GPay</v>
       </c>
     </row>
@@ -733,9 +633,6 @@
         <v>58865</v>
       </c>
       <c r="E3" t="str">
-        <v>HDFC Savings</v>
-      </c>
-      <c r="F3" t="str">
         <v>Gpay</v>
       </c>
     </row>
@@ -753,9 +650,6 @@
         <v>17929</v>
       </c>
       <c r="E4" t="str">
-        <v>HDFC Savings</v>
-      </c>
-      <c r="F4" t="str">
         <v>GPay</v>
       </c>
     </row>
@@ -773,9 +667,6 @@
         <v>2000</v>
       </c>
       <c r="E5" t="str">
-        <v>HDFC Savings</v>
-      </c>
-      <c r="F5" t="str">
         <v>GPay</v>
       </c>
     </row>
@@ -793,9 +684,6 @@
         <v>2500</v>
       </c>
       <c r="E6" t="str">
-        <v>HDFC Savings</v>
-      </c>
-      <c r="F6" t="str">
         <v>GPay</v>
       </c>
     </row>
@@ -813,9 +701,6 @@
         <v>211</v>
       </c>
       <c r="E7" t="str">
-        <v>HDFC Savings</v>
-      </c>
-      <c r="F7" t="str">
         <v>GPay</v>
       </c>
     </row>
@@ -833,9 +718,6 @@
         <v>5891</v>
       </c>
       <c r="E8" t="str">
-        <v>HDFC Savings</v>
-      </c>
-      <c r="F8" t="str">
         <v>Bank transfer</v>
       </c>
     </row>
@@ -853,9 +735,6 @@
         <v>861</v>
       </c>
       <c r="E9" t="str">
-        <v>HDFC Savings</v>
-      </c>
-      <c r="F9" t="str">
         <v>GPay</v>
       </c>
     </row>
@@ -873,9 +752,6 @@
         <v>199</v>
       </c>
       <c r="E10" t="str">
-        <v>HDFC Savings</v>
-      </c>
-      <c r="F10" t="str">
         <v>GPay</v>
       </c>
     </row>
@@ -893,209 +769,17 @@
         <v>2500</v>
       </c>
       <c r="E11" t="str">
-        <v>HDFC Savings</v>
-      </c>
-      <c r="F11" t="str">
         <v>GPay</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E8"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="28.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Bank Name</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Account Number</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Account Type</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Opening Balance</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Notes</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>HDFC Savings</v>
-      </c>
-      <c r="B2" t="str">
-        <v>1234567890</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Savings</v>
-      </c>
-      <c r="D2">
-        <v>250000</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Main account</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>ICICI Current</v>
-      </c>
-      <c r="B3" t="str">
-        <v>9876543210</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Current</v>
-      </c>
-      <c r="D3">
-        <v>150000</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Business account</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>SBI Savings</v>
-      </c>
-      <c r="B4" t="str">
-        <v>5555666677</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Savings</v>
-      </c>
-      <c r="D4">
-        <v>75000</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Secondary</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Axis Cash</v>
-      </c>
-      <c r="B5" t="str">
-        <v>1111222233</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Cash</v>
-      </c>
-      <c r="D5">
-        <v>5000</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Petty cash</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>HDFC-ALUVA</v>
-      </c>
-      <c r="B6" t="str">
-        <v>50100523900334</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Savings</v>
-      </c>
-      <c r="D6">
-        <v>11078.46</v>
-      </c>
-      <c r="E6" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>hdfc</v>
-      </c>
-      <c r="B7" t="str">
-        <v>122321311</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Savings</v>
-      </c>
-      <c r="D7">
-        <v>11075</v>
-      </c>
-      <c r="E7" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>HDFR</v>
-      </c>
-      <c r="B8" t="str">
-        <v/>
-      </c>
-      <c r="C8" t="str">
-        <v>Savings</v>
-      </c>
-      <c r="D8">
-        <v>0</v>
-      </c>
-      <c r="E8" t="str">
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="28.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Date</v>
-      </c>
-      <c r="B1" t="str">
-        <v>From Bank</v>
-      </c>
-      <c r="C1" t="str">
-        <v>To Bank</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Amount</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Reference / Notes</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F4"/>
   <cols>
@@ -1194,7 +878,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H2"/>
   <cols>
@@ -1267,7 +951,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E1"/>
   <cols>
@@ -1302,7 +986,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G3"/>
   <cols>
@@ -1391,9 +1075,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E15"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -1538,9 +1222,191 @@
         <v/>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Allowance</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Shopping</v>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v>Other</v>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Credit card use</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Travel</v>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v/>
+      </c>
+      <c r="B11" t="str">
+        <v>Family</v>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v/>
+      </c>
+      <c r="B12" t="str">
+        <v>Other</v>
+      </c>
+      <c r="C12" t="str">
+        <v/>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v/>
+      </c>
+      <c r="B13" t="str">
+        <v>Credit Card</v>
+      </c>
+      <c r="C13" t="str">
+        <v/>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v/>
+      </c>
+      <c r="B14" t="str">
+        <v>Gst</v>
+      </c>
+      <c r="C14" t="str">
+        <v/>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v/>
+      </c>
+      <c r="B15" t="str">
+        <v>Loan HDFC- Shibin</v>
+      </c>
+      <c r="C15" t="str">
+        <v/>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E15"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B6"/>
+  <cols>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="70.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Key</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Value</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Currency</v>
+      </c>
+      <c r="B2" t="str">
+        <v>INR</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Owner</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Sanjo</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Username</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Galaxia</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>PasswordHash</v>
+      </c>
+      <c r="B5" t="str">
+        <v>sha256:0c627b0cccbfc96bd1b66b9dc10e3fbd23fc91d3f23a8b4506293980448eddf8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Theme</v>
+      </c>
+      <c r="B6" t="str">
+        <v>dark</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-18T18:19:27.020Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -5,12 +5,14 @@
   <sheets>
     <sheet name="Income" sheetId="1" r:id="rId1"/>
     <sheet name="Expenses" sheetId="2" r:id="rId2"/>
-    <sheet name="Investments" sheetId="3" r:id="rId3"/>
-    <sheet name="Loans" sheetId="4" r:id="rId4"/>
-    <sheet name="Loan Payments" sheetId="5" r:id="rId5"/>
-    <sheet name="Debts" sheetId="6" r:id="rId6"/>
-    <sheet name="Lists" sheetId="7" r:id="rId7"/>
-    <sheet name="Settings" sheetId="8" r:id="rId8"/>
+    <sheet name="Banks" sheetId="3" r:id="rId3"/>
+    <sheet name="Transfers" sheetId="4" r:id="rId4"/>
+    <sheet name="Investments" sheetId="5" r:id="rId5"/>
+    <sheet name="Loans" sheetId="6" r:id="rId6"/>
+    <sheet name="Loan Payments" sheetId="7" r:id="rId7"/>
+    <sheet name="Debts" sheetId="8" r:id="rId8"/>
+    <sheet name="Lists" sheetId="9" r:id="rId9"/>
+    <sheet name="Settings" sheetId="10" r:id="rId10"/>
   </sheets>
 </workbook>
 </file>
@@ -405,13 +407,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:F9"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
     <col min="3" max="3" width="16.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="26.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="26.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -428,6 +431,9 @@
         <v>Amount</v>
       </c>
       <c r="E1" t="str">
+        <v>Bank</v>
+      </c>
+      <c r="F1" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -445,6 +451,9 @@
         <v>113</v>
       </c>
       <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
         <v>July payroll</v>
       </c>
     </row>
@@ -464,6 +473,9 @@
       <c r="E3" t="str">
         <v/>
       </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -479,6 +491,9 @@
         <v>1000</v>
       </c>
       <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
         <v>old debt repay</v>
       </c>
     </row>
@@ -496,6 +511,9 @@
         <v>15000</v>
       </c>
       <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
         <v>old debt repay</v>
       </c>
     </row>
@@ -515,6 +533,9 @@
       <c r="E6" t="str">
         <v/>
       </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -532,6 +553,9 @@
       <c r="E7" t="str">
         <v/>
       </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -549,6 +573,9 @@
       <c r="E8" t="str">
         <v/>
       </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -564,25 +591,92 @@
         <v>33105</v>
       </c>
       <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
         <v>Icic- 6002</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F9"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B6"/>
+  <cols>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="70.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Key</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Value</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Currency</v>
+      </c>
+      <c r="B2" t="str">
+        <v>INR</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Owner</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Sanjo</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Username</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Galaxia</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>PasswordHash</v>
+      </c>
+      <c r="B5" t="str">
+        <v>sha256:0c627b0cccbfc96bd1b66b9dc10e3fbd23fc91d3f23a8b4506293980448eddf8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Theme</v>
+      </c>
+      <c r="B6" t="str">
+        <v>dark</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:F11"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
     <col min="3" max="3" width="28.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -599,6 +693,9 @@
         <v>Amount</v>
       </c>
       <c r="E1" t="str">
+        <v>Bank</v>
+      </c>
+      <c r="F1" t="str">
         <v>Payment Method</v>
       </c>
     </row>
@@ -616,6 +713,9 @@
         <v>500</v>
       </c>
       <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
         <v>GPay</v>
       </c>
     </row>
@@ -633,6 +733,9 @@
         <v>58865</v>
       </c>
       <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
         <v>Gpay</v>
       </c>
     </row>
@@ -650,6 +753,9 @@
         <v>17929</v>
       </c>
       <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
         <v>GPay</v>
       </c>
     </row>
@@ -667,6 +773,9 @@
         <v>2000</v>
       </c>
       <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
         <v>GPay</v>
       </c>
     </row>
@@ -684,6 +793,9 @@
         <v>2500</v>
       </c>
       <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
         <v>GPay</v>
       </c>
     </row>
@@ -701,6 +813,9 @@
         <v>211</v>
       </c>
       <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
         <v>GPay</v>
       </c>
     </row>
@@ -718,6 +833,9 @@
         <v>5891</v>
       </c>
       <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
         <v>Bank transfer</v>
       </c>
     </row>
@@ -735,6 +853,9 @@
         <v>861</v>
       </c>
       <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
         <v>GPay</v>
       </c>
     </row>
@@ -752,6 +873,9 @@
         <v>199</v>
       </c>
       <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
         <v>GPay</v>
       </c>
     </row>
@@ -769,17 +893,107 @@
         <v>2500</v>
       </c>
       <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
         <v>GPay</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E2"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="28.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Bank Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Account Number</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Account Type</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Opening Balance</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>HDFC- Aluva</v>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v>Savings</v>
+      </c>
+      <c r="D2">
+        <v>11000</v>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E1"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="28.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Date</v>
+      </c>
+      <c r="B1" t="str">
+        <v>From Bank</v>
+      </c>
+      <c r="C1" t="str">
+        <v>To Bank</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Amount</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Reference / Notes</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F4"/>
   <cols>
@@ -878,7 +1092,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H2"/>
   <cols>
@@ -951,7 +1165,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E1"/>
   <cols>
@@ -986,7 +1200,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G3"/>
   <cols>
@@ -1075,7 +1289,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E15"/>
   <cols>
@@ -1346,67 +1560,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:E15"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B6"/>
-  <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="70.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Key</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Value</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Currency</v>
-      </c>
-      <c r="B2" t="str">
-        <v>INR</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Owner</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Sanjo</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Username</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Galaxia</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>PasswordHash</v>
-      </c>
-      <c r="B5" t="str">
-        <v>sha256:0c627b0cccbfc96bd1b66b9dc10e3fbd23fc91d3f23a8b4506293980448eddf8</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Theme</v>
-      </c>
-      <c r="B6" t="str">
-        <v>dark</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-19T05:01:49.901Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -451,7 +451,7 @@
         <v>113</v>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>HDFC- Aluva</v>
       </c>
       <c r="F2" t="str">
         <v>July payroll</v>
@@ -471,7 +471,7 @@
         <v>105</v>
       </c>
       <c r="E3" t="str">
-        <v/>
+        <v>HDFC- Aluva</v>
       </c>
       <c r="F3" t="str">
         <v/>
@@ -491,7 +491,7 @@
         <v>1000</v>
       </c>
       <c r="E4" t="str">
-        <v/>
+        <v>HDFC- Aluva</v>
       </c>
       <c r="F4" t="str">
         <v>old debt repay</v>
@@ -511,7 +511,7 @@
         <v>15000</v>
       </c>
       <c r="E5" t="str">
-        <v/>
+        <v>HDFC- Aluva</v>
       </c>
       <c r="F5" t="str">
         <v>old debt repay</v>
@@ -531,7 +531,7 @@
         <v>78</v>
       </c>
       <c r="E6" t="str">
-        <v/>
+        <v>HDFC- Aluva</v>
       </c>
       <c r="F6" t="str">
         <v/>
@@ -551,7 +551,7 @@
         <v>150</v>
       </c>
       <c r="E7" t="str">
-        <v/>
+        <v>HDFC- Aluva</v>
       </c>
       <c r="F7" t="str">
         <v/>
@@ -571,7 +571,7 @@
         <v>50</v>
       </c>
       <c r="E8" t="str">
-        <v/>
+        <v>HDFC- Aluva</v>
       </c>
       <c r="F8" t="str">
         <v/>
@@ -591,7 +591,7 @@
         <v>33105</v>
       </c>
       <c r="E9" t="str">
-        <v/>
+        <v>HDFC- Aluva</v>
       </c>
       <c r="F9" t="str">
         <v>Icic- 6002</v>
@@ -669,7 +669,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -713,7 +713,7 @@
         <v>500</v>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>HDFC- Aluva</v>
       </c>
       <c r="F2" t="str">
         <v>GPay</v>
@@ -733,7 +733,7 @@
         <v>58865</v>
       </c>
       <c r="E3" t="str">
-        <v/>
+        <v>HDFC- Aluva</v>
       </c>
       <c r="F3" t="str">
         <v>Gpay</v>
@@ -753,7 +753,7 @@
         <v>17929</v>
       </c>
       <c r="E4" t="str">
-        <v/>
+        <v>HDFC- Aluva</v>
       </c>
       <c r="F4" t="str">
         <v>GPay</v>
@@ -773,7 +773,7 @@
         <v>2000</v>
       </c>
       <c r="E5" t="str">
-        <v/>
+        <v>HDFC- Aluva</v>
       </c>
       <c r="F5" t="str">
         <v>GPay</v>
@@ -793,7 +793,7 @@
         <v>2500</v>
       </c>
       <c r="E6" t="str">
-        <v/>
+        <v>HDFC- Aluva</v>
       </c>
       <c r="F6" t="str">
         <v>GPay</v>
@@ -813,7 +813,7 @@
         <v>211</v>
       </c>
       <c r="E7" t="str">
-        <v/>
+        <v>HDFC- Aluva</v>
       </c>
       <c r="F7" t="str">
         <v>GPay</v>
@@ -833,7 +833,7 @@
         <v>5891</v>
       </c>
       <c r="E8" t="str">
-        <v/>
+        <v>HDFC- Aluva</v>
       </c>
       <c r="F8" t="str">
         <v>Bank transfer</v>
@@ -853,7 +853,7 @@
         <v>861</v>
       </c>
       <c r="E9" t="str">
-        <v/>
+        <v>HDFC- Aluva</v>
       </c>
       <c r="F9" t="str">
         <v>GPay</v>
@@ -873,7 +873,7 @@
         <v>199</v>
       </c>
       <c r="E10" t="str">
-        <v/>
+        <v>HDFC- Aluva</v>
       </c>
       <c r="F10" t="str">
         <v>GPay</v>
@@ -893,15 +893,35 @@
         <v>2500</v>
       </c>
       <c r="E11" t="str">
-        <v/>
+        <v>HDFC- Aluva</v>
       </c>
       <c r="F11" t="str">
         <v>GPay</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>2026-07-19</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Family</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Amma expense</v>
+      </c>
+      <c r="D12">
+        <v>2000</v>
+      </c>
+      <c r="E12" t="str">
+        <v>HDFC- Aluva</v>
+      </c>
+      <c r="F12" t="str">
+        <v>GPay</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F12"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-19T05:39:52.487Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -1222,7 +1222,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -1302,9 +1302,32 @@
         <v/>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>2026-07-19</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Binison</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Given</v>
+      </c>
+      <c r="D4">
+        <v>1500</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-19T06:15:58.419Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -928,7 +928,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -971,9 +971,26 @@
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>test</v>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v>Savings</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-19T06:17:01.896Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -997,7 +997,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -1023,9 +1023,26 @@
         <v>Reference / Notes</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>2026-07-19</v>
+      </c>
+      <c r="B2" t="str">
+        <v>HDFC- Aluva</v>
+      </c>
+      <c r="C2" t="str">
+        <v>test</v>
+      </c>
+      <c r="D2">
+        <v>100</v>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-19T06:37:10.316Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -959,13 +959,13 @@
         <v>HDFC- Aluva</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v>50100523900334</v>
       </c>
       <c r="C2" t="str">
         <v>Savings</v>
       </c>
       <c r="D2">
-        <v>11000</v>
+        <v>11106</v>
       </c>
       <c r="E2" t="str">
         <v/>
@@ -973,16 +973,16 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>test</v>
+        <v>HDFC- Info</v>
       </c>
       <c r="B3" t="str">
-        <v/>
+        <v>50100465194051</v>
       </c>
       <c r="C3" t="str">
         <v>Savings</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>6463</v>
       </c>
       <c r="E3" t="str">
         <v/>
@@ -997,7 +997,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E1"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -1023,26 +1023,9 @@
         <v>Reference / Notes</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>2026-07-19</v>
-      </c>
-      <c r="B2" t="str">
-        <v>HDFC- Aluva</v>
-      </c>
-      <c r="C2" t="str">
-        <v>test</v>
-      </c>
-      <c r="D2">
-        <v>100</v>
-      </c>
-      <c r="E2" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-19T09:23:03.867Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -927,7 +927,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -987,9 +987,26 @@
         <v/>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Federal-Ang</v>
+      </c>
+      <c r="B4" t="str">
+        <v>10020100375530</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Savings</v>
+      </c>
+      <c r="D4">
+        <v>18944</v>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-19T09:25:24.020Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -927,7 +927,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -1004,9 +1004,26 @@
         <v/>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>SBI</v>
+      </c>
+      <c r="B5" t="str">
+        <v>43602594069</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Savings</v>
+      </c>
+      <c r="D5">
+        <v>123024.2</v>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-19T09:37:36.713Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -470,7 +470,7 @@
         <v>105</v>
       </c>
       <c r="E3" t="str">
-        <v>HDFC- Aluva</v>
+        <v>Federal-Ang</v>
       </c>
       <c r="F3" t="str">
         <v/>
@@ -510,7 +510,7 @@
         <v>15000</v>
       </c>
       <c r="E5" t="str">
-        <v>HDFC- Aluva</v>
+        <v>Federal-Ang</v>
       </c>
       <c r="F5" t="str">
         <v>old debt repay</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-19T09:41:01.168Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -550,7 +550,7 @@
         <v>150</v>
       </c>
       <c r="E7" t="str">
-        <v>HDFC- Aluva</v>
+        <v>Federal-Ang</v>
       </c>
       <c r="F7" t="str">
         <v/>
@@ -570,7 +570,7 @@
         <v>50</v>
       </c>
       <c r="E8" t="str">
-        <v>HDFC- Aluva</v>
+        <v>Federal-Ang</v>
       </c>
       <c r="F8" t="str">
         <v/>
@@ -590,7 +590,7 @@
         <v>33105</v>
       </c>
       <c r="E9" t="str">
-        <v>HDFC- Aluva</v>
+        <v>Federal-Ang</v>
       </c>
       <c r="F9" t="str">
         <v>Icic- 6002</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-19T09:46:14.144Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -1115,7 +1115,7 @@
         <v>409</v>
       </c>
       <c r="F2" t="str">
-        <v>HDFC- Aluva</v>
+        <v>Federal-Ang</v>
       </c>
       <c r="G2" t="str">
         <v>Pention fund</v>
@@ -1138,7 +1138,7 @@
         <v>1996</v>
       </c>
       <c r="F3" t="str">
-        <v>HDFC- Aluva</v>
+        <v>Federal-Ang</v>
       </c>
       <c r="G3" t="str">
         <v/>
@@ -1161,7 +1161,7 @@
         <v>1331</v>
       </c>
       <c r="F4" t="str">
-        <v>HDFC- Aluva</v>
+        <v>Federal-Ang</v>
       </c>
       <c r="G4" t="str">
         <v/>
@@ -1370,7 +1370,7 @@
         <v>2026-08-01</v>
       </c>
       <c r="G3" t="str">
-        <v>HDFC- Aluva</v>
+        <v>Federal-Ang</v>
       </c>
       <c r="H3" t="str">
         <v/>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-20T08:42:23.200Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -712,7 +712,7 @@
         <v>500</v>
       </c>
       <c r="E2" t="str">
-        <v>HDFC- Aluva</v>
+        <v>HDFC- Info</v>
       </c>
       <c r="F2" t="str">
         <v>GPay</v>
@@ -812,7 +812,7 @@
         <v>211</v>
       </c>
       <c r="E7" t="str">
-        <v>HDFC- Aluva</v>
+        <v>Federal-Ang</v>
       </c>
       <c r="F7" t="str">
         <v>GPay</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-20T08:47:47.019Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -732,7 +732,7 @@
         <v>58865</v>
       </c>
       <c r="E3" t="str">
-        <v>HDFC- Aluva</v>
+        <v>HDFC- Info</v>
       </c>
       <c r="F3" t="str">
         <v>Gpay</v>
@@ -752,7 +752,7 @@
         <v>17929</v>
       </c>
       <c r="E4" t="str">
-        <v>HDFC- Aluva</v>
+        <v>HDFC- Info</v>
       </c>
       <c r="F4" t="str">
         <v>GPay</v>
@@ -772,7 +772,7 @@
         <v>2000</v>
       </c>
       <c r="E5" t="str">
-        <v>HDFC- Aluva</v>
+        <v>HDFC- Info</v>
       </c>
       <c r="F5" t="str">
         <v>GPay</v>
@@ -792,7 +792,7 @@
         <v>2500</v>
       </c>
       <c r="E6" t="str">
-        <v>HDFC- Aluva</v>
+        <v>HDFC- Info</v>
       </c>
       <c r="F6" t="str">
         <v>GPay</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-20T08:49:35.853Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -447,10 +447,10 @@
         <v>Salary</v>
       </c>
       <c r="D2">
-        <v>113</v>
+        <v>113175</v>
       </c>
       <c r="E2" t="str">
-        <v>HDFC- Aluva</v>
+        <v>HDFC- Info</v>
       </c>
       <c r="F2" t="str">
         <v>July payroll</v>
@@ -467,10 +467,10 @@
         <v>Allowance</v>
       </c>
       <c r="D3">
-        <v>105</v>
+        <v>105229</v>
       </c>
       <c r="E3" t="str">
-        <v>Federal-Ang</v>
+        <v>HDFC- Info</v>
       </c>
       <c r="F3" t="str">
         <v/>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-20T10:34:09.812Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -490,7 +490,7 @@
         <v>1000</v>
       </c>
       <c r="E4" t="str">
-        <v>HDFC- Aluva</v>
+        <v>HDFC- Info</v>
       </c>
       <c r="F4" t="str">
         <v>old debt repay</v>
@@ -530,7 +530,7 @@
         <v>78</v>
       </c>
       <c r="E6" t="str">
-        <v>HDFC- Aluva</v>
+        <v>Federal-Ang</v>
       </c>
       <c r="F6" t="str">
         <v/>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-20T11:22:34.211Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -668,7 +668,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -918,9 +918,29 @@
         <v>GPay</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>2026-07-20</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Family</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Hanna Passam</v>
+      </c>
+      <c r="D13">
+        <v>300</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Federal-Ang</v>
+      </c>
+      <c r="F13" t="str">
+        <v>GPay</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F13"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-20T11:27:59.423Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -729,7 +729,7 @@
         <v>axis credit card</v>
       </c>
       <c r="D3">
-        <v>58865</v>
+        <v>58864.38</v>
       </c>
       <c r="E3" t="str">
         <v>HDFC- Info</v>
@@ -749,7 +749,7 @@
         <v>icici</v>
       </c>
       <c r="D4">
-        <v>17929</v>
+        <v>17928.39</v>
       </c>
       <c r="E4" t="str">
         <v>HDFC- Info</v>
@@ -812,7 +812,7 @@
         <v>211</v>
       </c>
       <c r="E7" t="str">
-        <v>Federal-Ang</v>
+        <v>HDFC- Info</v>
       </c>
       <c r="F7" t="str">
         <v>GPay</v>
@@ -849,7 +849,7 @@
         <v>Recharge mobile</v>
       </c>
       <c r="D9">
-        <v>861</v>
+        <v>860.9</v>
       </c>
       <c r="E9" t="str">
         <v>Federal-Ang</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-20T11:29:58.063Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -406,7 +406,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -596,9 +596,29 @@
         <v>Icic- 6002</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Bank Interest SB</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Interest</v>
+      </c>
+      <c r="D10">
+        <v>158</v>
+      </c>
+      <c r="E10" t="str">
+        <v>HDFC- Info</v>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F10"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1612,7 +1632,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v/>
+        <v>Interest</v>
       </c>
       <c r="B11" t="str">
         <v>Family</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-20T12:11:50.942Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -1105,7 +1105,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:J5"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -1135,6 +1135,15 @@
         <v>Bank</v>
       </c>
       <c r="G1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Closed Date</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Closed Value</v>
+      </c>
+      <c r="J1" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -1158,6 +1167,15 @@
         <v>Federal-Ang</v>
       </c>
       <c r="G2" t="str">
+        <v>Open</v>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
         <v>Pention fund</v>
       </c>
     </row>
@@ -1181,6 +1199,15 @@
         <v>Federal-Ang</v>
       </c>
       <c r="G3" t="str">
+        <v>Open</v>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
         <v/>
       </c>
     </row>
@@ -1204,19 +1231,60 @@
         <v>Federal-Ang</v>
       </c>
       <c r="G4" t="str">
+        <v>Open</v>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>2026-07-20</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Test</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Stocks</v>
+      </c>
+      <c r="D5">
+        <v>100</v>
+      </c>
+      <c r="E5">
+        <v>100</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Federal-Ang</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Closed</v>
+      </c>
+      <c r="H5" t="str">
+        <v>2026-07-20</v>
+      </c>
+      <c r="I5">
+        <v>100</v>
+      </c>
+      <c r="J5" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:L2"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -1251,6 +1319,18 @@
         <v>Tenure Months</v>
       </c>
       <c r="H1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Closed Date</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Close Bank</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Close Amount</v>
+      </c>
+      <c r="L1" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -1277,12 +1357,24 @@
         <v>342</v>
       </c>
       <c r="H2" t="str">
+        <v>Open</v>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
         <v>43716460547</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-20T12:11:59.516Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -1105,7 +1105,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J4"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -1243,41 +1243,9 @@
         <v/>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>2026-07-20</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Test</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Stocks</v>
-      </c>
-      <c r="D5">
-        <v>100</v>
-      </c>
-      <c r="E5">
-        <v>100</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Federal-Ang</v>
-      </c>
-      <c r="G5" t="str">
-        <v>Closed</v>
-      </c>
-      <c r="H5" t="str">
-        <v>2026-07-20</v>
-      </c>
-      <c r="I5">
-        <v>100</v>
-      </c>
-      <c r="J5" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-20T15:51:01.000Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I21"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -976,38 +976,9 @@
         <v>Family</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>TXN-1019</v>
-      </c>
-      <c r="B22" t="str">
-        <v>2026-07-20</v>
-      </c>
-      <c r="C22" t="str">
-        <v>Income</v>
-      </c>
-      <c r="D22" t="str">
-        <v>Debt Settlement</v>
-      </c>
-      <c r="E22" t="str">
-        <v>Full repayment received</v>
-      </c>
-      <c r="F22">
-        <v>5000</v>
-      </c>
-      <c r="G22" t="str">
-        <v>HDFC- Info</v>
-      </c>
-      <c r="H22" t="str">
-        <v>GPay</v>
-      </c>
-      <c r="I22" t="str">
-        <v>Auto-Posted: DEBT-01 (Jomisha)</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I21"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1133,13 +1104,13 @@
         <v>6463</v>
       </c>
       <c r="F5">
-        <v>224562</v>
+        <v>219562</v>
       </c>
       <c r="G5">
         <v>84003.77</v>
       </c>
       <c r="H5">
-        <v>147021.23</v>
+        <v>142021.23</v>
       </c>
       <c r="I5" t="str">
         <v>2026-07-20</v>
@@ -1148,7 +1119,7 @@
         <v>140134.46</v>
       </c>
       <c r="K5">
-        <v>6886.77</v>
+        <v>1886.77</v>
       </c>
       <c r="L5" t="str">
         <v>Discrepancy</v>
@@ -1320,7 +1291,7 @@
         <v>5000</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="G4" t="str">
         <v>2026-07-13</v>
@@ -1329,16 +1300,16 @@
         <v>2026-07-20</v>
       </c>
       <c r="I4" t="str">
-        <v>Closed</v>
+        <v>Open</v>
       </c>
       <c r="J4" t="str">
-        <v>2026-07-20</v>
+        <v/>
       </c>
       <c r="K4" t="str">
-        <v>HDFC- Info</v>
+        <v/>
       </c>
       <c r="L4" t="str">
-        <v>TXN-1019</v>
+        <v/>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-20T15:52:53.688Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -1953,7 +1953,7 @@
         <v>Username</v>
       </c>
       <c r="B4" t="str">
-        <v/>
+        <v>Galaxia</v>
       </c>
     </row>
     <row r="5">
@@ -1961,7 +1961,7 @@
         <v>PasswordHash</v>
       </c>
       <c r="B5" t="str">
-        <v/>
+        <v>sha256:0c627b0cccbfc96bd1b66b9dc10e3fbd23fc91d3f23a8b4506293980448eddf8</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-20T21:30:43.417Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I22"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -976,9 +976,38 @@
         <v>Family</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>TXN-1019</v>
+      </c>
+      <c r="B22" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Income</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Interest</v>
+      </c>
+      <c r="E22" t="str">
+        <v>sb Interest</v>
+      </c>
+      <c r="F22">
+        <v>28</v>
+      </c>
+      <c r="G22" t="str">
+        <v>HDFC- Aluva</v>
+      </c>
+      <c r="H22" t="str">
+        <v>Other</v>
+      </c>
+      <c r="I22" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I22"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1066,13 +1095,13 @@
         <v>11106</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="G4">
         <v>5891</v>
       </c>
       <c r="H4">
-        <v>5215</v>
+        <v>5243</v>
       </c>
       <c r="I4" t="str">
         <v>2026-07-20</v>
@@ -1081,7 +1110,7 @@
         <v>5218</v>
       </c>
       <c r="K4">
-        <v>-3</v>
+        <v>25</v>
       </c>
       <c r="L4" t="str">
         <v>Discrepancy</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-20T21:31:15.604Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1005,9 +1005,38 @@
         <v/>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>TXN-1020</v>
+      </c>
+      <c r="B23" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Transfer</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Transfer</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Savings transfer</v>
+      </c>
+      <c r="F23">
+        <v>20000</v>
+      </c>
+      <c r="G23" t="str">
+        <v>HDFC- Info → HDFC- Aluva</v>
+      </c>
+      <c r="H23" t="str">
+        <v/>
+      </c>
+      <c r="I23" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I23"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1095,13 +1124,13 @@
         <v>11106</v>
       </c>
       <c r="F4">
-        <v>28</v>
+        <v>20028</v>
       </c>
       <c r="G4">
         <v>5891</v>
       </c>
       <c r="H4">
-        <v>5243</v>
+        <v>25243</v>
       </c>
       <c r="I4" t="str">
         <v>2026-07-20</v>
@@ -1110,7 +1139,7 @@
         <v>5218</v>
       </c>
       <c r="K4">
-        <v>25</v>
+        <v>20025</v>
       </c>
       <c r="L4" t="str">
         <v>Discrepancy</v>
@@ -1136,10 +1165,10 @@
         <v>219562</v>
       </c>
       <c r="G5">
-        <v>84003.77</v>
+        <v>104003.77</v>
       </c>
       <c r="H5">
-        <v>142021.23</v>
+        <v>122021.23</v>
       </c>
       <c r="I5" t="str">
         <v>2026-07-20</v>
@@ -1148,7 +1177,7 @@
         <v>140134.46</v>
       </c>
       <c r="K5">
-        <v>1886.77</v>
+        <v>-18113.23</v>
       </c>
       <c r="L5" t="str">
         <v>Discrepancy</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-20T21:34:39.259Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -1109,37 +1109,37 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ACC-01</v>
+        <v>ACC-02</v>
       </c>
       <c r="B4" t="str">
-        <v>HDFC- Aluva</v>
+        <v>HDFC- Info</v>
       </c>
       <c r="C4" t="str">
-        <v>50100523900334</v>
+        <v>50100465194051</v>
       </c>
       <c r="D4" t="str">
         <v>Savings</v>
       </c>
       <c r="E4">
-        <v>11106</v>
+        <v>6463</v>
       </c>
       <c r="F4">
-        <v>20028</v>
+        <v>219562</v>
       </c>
       <c r="G4">
-        <v>5891</v>
+        <v>104003.77</v>
       </c>
       <c r="H4">
-        <v>25243</v>
+        <v>122021.23</v>
       </c>
       <c r="I4" t="str">
         <v>2026-07-20</v>
       </c>
       <c r="J4">
-        <v>5218</v>
+        <v>140134.46</v>
       </c>
       <c r="K4">
-        <v>20025</v>
+        <v>-18113.23</v>
       </c>
       <c r="L4" t="str">
         <v>Discrepancy</v>
@@ -1147,37 +1147,37 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ACC-02</v>
+        <v>ACC-03</v>
       </c>
       <c r="B5" t="str">
-        <v>HDFC- Info</v>
+        <v>Federal-Ang</v>
       </c>
       <c r="C5" t="str">
-        <v>50100465194051</v>
+        <v>10020100375530</v>
       </c>
       <c r="D5" t="str">
         <v>Savings</v>
       </c>
       <c r="E5">
-        <v>6463</v>
+        <v>18944</v>
       </c>
       <c r="F5">
-        <v>219562</v>
+        <v>200</v>
       </c>
       <c r="G5">
-        <v>104003.77</v>
+        <v>3859.9</v>
       </c>
       <c r="H5">
-        <v>122021.23</v>
+        <v>15284.1</v>
       </c>
       <c r="I5" t="str">
         <v>2026-07-20</v>
       </c>
       <c r="J5">
-        <v>140134.46</v>
+        <v>30367.1</v>
       </c>
       <c r="K5">
-        <v>-18113.23</v>
+        <v>-15083</v>
       </c>
       <c r="L5" t="str">
         <v>Discrepancy</v>
@@ -1185,78 +1185,78 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ACC-03</v>
+        <v>ACC-04</v>
       </c>
       <c r="B6" t="str">
-        <v>Federal-Ang</v>
+        <v>SBI</v>
       </c>
       <c r="C6" t="str">
-        <v>10020100375530</v>
+        <v>43602594069</v>
       </c>
       <c r="D6" t="str">
         <v>Savings</v>
       </c>
       <c r="E6">
-        <v>18944</v>
+        <v>123024.2</v>
       </c>
       <c r="F6">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="G6">
-        <v>3859.9</v>
+        <v>0</v>
       </c>
       <c r="H6">
-        <v>15284.1</v>
+        <v>123024.2</v>
       </c>
       <c r="I6" t="str">
-        <v>2026-07-20</v>
+        <v/>
       </c>
       <c r="J6">
-        <v>30367.1</v>
+        <v>123024.2</v>
       </c>
       <c r="K6">
-        <v>-15083</v>
+        <v>0</v>
       </c>
       <c r="L6" t="str">
-        <v>Discrepancy</v>
+        <v>Reconciled</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ACC-04</v>
+        <v>ACC-01</v>
       </c>
       <c r="B7" t="str">
-        <v>SBI</v>
+        <v>HDFC- Aluva</v>
       </c>
       <c r="C7" t="str">
-        <v>43602594069</v>
+        <v>50100523900334</v>
       </c>
       <c r="D7" t="str">
         <v>Savings</v>
       </c>
       <c r="E7">
-        <v>123024.2</v>
+        <v>11078.46</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>20028</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <v>5891</v>
       </c>
       <c r="H7">
-        <v>123024.2</v>
+        <v>25215.46</v>
       </c>
       <c r="I7" t="str">
         <v/>
       </c>
-      <c r="J7">
-        <v>123024.2</v>
-      </c>
-      <c r="K7">
-        <v>0</v>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v/>
       </c>
       <c r="L7" t="str">
-        <v>Reconciled</v>
+        <v>Pending</v>
       </c>
     </row>
   </sheetData>
@@ -1268,7 +1268,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L6"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -1334,28 +1334,28 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>DEBT-01</v>
+        <v>DEBT-02</v>
       </c>
       <c r="B4" t="str">
         <v>Debt Receivable</v>
       </c>
       <c r="C4" t="str">
-        <v>Jomisha</v>
+        <v>Baby Antony</v>
       </c>
       <c r="D4" t="str">
         <v>Money Given</v>
       </c>
       <c r="E4">
-        <v>5000</v>
+        <v>25000</v>
       </c>
       <c r="F4">
-        <v>5000</v>
+        <v>25000</v>
       </c>
       <c r="G4" t="str">
-        <v>2026-07-13</v>
+        <v>2026-07-01</v>
       </c>
       <c r="H4" t="str">
-        <v>2026-07-20</v>
+        <v>2026-08-01</v>
       </c>
       <c r="I4" t="str">
         <v>Open</v>
@@ -1372,28 +1372,28 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>DEBT-02</v>
+        <v>DEBT-03</v>
       </c>
       <c r="B5" t="str">
         <v>Debt Receivable</v>
       </c>
       <c r="C5" t="str">
-        <v>Baby Antony</v>
+        <v>Binison</v>
       </c>
       <c r="D5" t="str">
         <v>Money Given</v>
       </c>
       <c r="E5">
-        <v>25000</v>
+        <v>1500</v>
       </c>
       <c r="F5">
-        <v>25000</v>
+        <v>1500</v>
       </c>
       <c r="G5" t="str">
-        <v>2026-07-01</v>
+        <v>2026-07-19</v>
       </c>
       <c r="H5" t="str">
-        <v>2026-08-01</v>
+        <v>2026-08-31</v>
       </c>
       <c r="I5" t="str">
         <v>Open</v>
@@ -1410,28 +1410,28 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>DEBT-03</v>
+        <v>LOAN-01</v>
       </c>
       <c r="B6" t="str">
-        <v>Debt Receivable</v>
+        <v>Bank Loan Payable</v>
       </c>
       <c r="C6" t="str">
-        <v>Binison</v>
+        <v>SBI Home Loan</v>
       </c>
       <c r="D6" t="str">
-        <v>Money Given</v>
+        <v>Housing Loan</v>
       </c>
       <c r="E6">
-        <v>1500</v>
+        <v>5758624</v>
       </c>
       <c r="F6">
-        <v>1500</v>
+        <v>5758624</v>
       </c>
       <c r="G6" t="str">
-        <v>2026-07-19</v>
+        <v>2026-08-14</v>
       </c>
       <c r="H6" t="str">
-        <v>2026-08-31</v>
+        <v/>
       </c>
       <c r="I6" t="str">
         <v>Open</v>
@@ -1446,47 +1446,9 @@
         <v/>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>LOAN-01</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Bank Loan Payable</v>
-      </c>
-      <c r="C7" t="str">
-        <v>SBI Home Loan</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Housing Loan</v>
-      </c>
-      <c r="E7">
-        <v>5758624</v>
-      </c>
-      <c r="F7">
-        <v>5758624</v>
-      </c>
-      <c r="G7" t="str">
-        <v>2026-08-14</v>
-      </c>
-      <c r="H7" t="str">
-        <v/>
-      </c>
-      <c r="I7" t="str">
-        <v>Open</v>
-      </c>
-      <c r="J7" t="str">
-        <v/>
-      </c>
-      <c r="K7" t="str">
-        <v/>
-      </c>
-      <c r="L7" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L6"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-20T21:38:30.952Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I24"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1034,9 +1034,38 @@
         <v/>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>TXN-1021</v>
+      </c>
+      <c r="B24" t="str">
+        <v>2026-07-13</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Debt Given</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Lent to Jomisha</v>
+      </c>
+      <c r="F24">
+        <v>5000</v>
+      </c>
+      <c r="G24" t="str">
+        <v>HDFC- Info</v>
+      </c>
+      <c r="H24" t="str">
+        <v/>
+      </c>
+      <c r="I24" t="str">
+        <v>Linked: DEBT-04 (Jomisha)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I24"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1127,10 +1156,10 @@
         <v>219562</v>
       </c>
       <c r="G4">
-        <v>104003.77</v>
+        <v>109003.77</v>
       </c>
       <c r="H4">
-        <v>122021.23</v>
+        <v>117021.23</v>
       </c>
       <c r="I4" t="str">
         <v>2026-07-20</v>
@@ -1139,7 +1168,7 @@
         <v>140134.46</v>
       </c>
       <c r="K4">
-        <v>-18113.23</v>
+        <v>-23113.23</v>
       </c>
       <c r="L4" t="str">
         <v>Discrepancy</v>
@@ -1268,7 +1297,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -1446,9 +1475,47 @@
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>DEBT-04</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Debt Receivable</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Jomisha</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Sisy</v>
+      </c>
+      <c r="E7">
+        <v>5000</v>
+      </c>
+      <c r="F7">
+        <v>5000</v>
+      </c>
+      <c r="G7" t="str">
+        <v>2026-07-13</v>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v>Open</v>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L7"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-20T21:40:45.568Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I25"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1063,9 +1063,38 @@
         <v>Linked: DEBT-04 (Jomisha)</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>TXN-1022</v>
+      </c>
+      <c r="B25" t="str">
+        <v>2026-07-19</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Debt Given</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Lent to Binison</v>
+      </c>
+      <c r="F25">
+        <v>1500</v>
+      </c>
+      <c r="G25" t="str">
+        <v>HDFC- Info</v>
+      </c>
+      <c r="H25" t="str">
+        <v/>
+      </c>
+      <c r="I25" t="str">
+        <v>Linked: DEBT-05 (Binison)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I25"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1156,10 +1185,10 @@
         <v>219562</v>
       </c>
       <c r="G4">
-        <v>109003.77</v>
+        <v>110503.77</v>
       </c>
       <c r="H4">
-        <v>117021.23</v>
+        <v>115521.23</v>
       </c>
       <c r="I4" t="str">
         <v>2026-07-20</v>
@@ -1168,7 +1197,7 @@
         <v>140134.46</v>
       </c>
       <c r="K4">
-        <v>-23113.23</v>
+        <v>-24613.23</v>
       </c>
       <c r="L4" t="str">
         <v>Discrepancy</v>
@@ -1401,28 +1430,28 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>DEBT-03</v>
+        <v>LOAN-01</v>
       </c>
       <c r="B5" t="str">
-        <v>Debt Receivable</v>
+        <v>Bank Loan Payable</v>
       </c>
       <c r="C5" t="str">
-        <v>Binison</v>
+        <v>SBI Home Loan</v>
       </c>
       <c r="D5" t="str">
-        <v>Money Given</v>
+        <v>Housing Loan</v>
       </c>
       <c r="E5">
-        <v>1500</v>
+        <v>5758624</v>
       </c>
       <c r="F5">
-        <v>1500</v>
+        <v>5758624</v>
       </c>
       <c r="G5" t="str">
-        <v>2026-07-19</v>
+        <v>2026-08-14</v>
       </c>
       <c r="H5" t="str">
-        <v>2026-08-31</v>
+        <v/>
       </c>
       <c r="I5" t="str">
         <v>Open</v>
@@ -1439,25 +1468,25 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>LOAN-01</v>
+        <v>DEBT-04</v>
       </c>
       <c r="B6" t="str">
-        <v>Bank Loan Payable</v>
+        <v>Debt Receivable</v>
       </c>
       <c r="C6" t="str">
-        <v>SBI Home Loan</v>
+        <v>Jomisha</v>
       </c>
       <c r="D6" t="str">
-        <v>Housing Loan</v>
+        <v>Sisy</v>
       </c>
       <c r="E6">
-        <v>5758624</v>
+        <v>5000</v>
       </c>
       <c r="F6">
-        <v>5758624</v>
+        <v>5000</v>
       </c>
       <c r="G6" t="str">
-        <v>2026-08-14</v>
+        <v>2026-07-13</v>
       </c>
       <c r="H6" t="str">
         <v/>
@@ -1477,28 +1506,28 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>DEBT-04</v>
+        <v>DEBT-05</v>
       </c>
       <c r="B7" t="str">
         <v>Debt Receivable</v>
       </c>
       <c r="C7" t="str">
-        <v>Jomisha</v>
+        <v>Binison</v>
       </c>
       <c r="D7" t="str">
-        <v>Sisy</v>
+        <v>Friend</v>
       </c>
       <c r="E7">
-        <v>5000</v>
+        <v>1500</v>
       </c>
       <c r="F7">
-        <v>5000</v>
+        <v>1500</v>
       </c>
       <c r="G7" t="str">
-        <v>2026-07-13</v>
+        <v>2026-07-19</v>
       </c>
       <c r="H7" t="str">
-        <v/>
+        <v>2026-08-20</v>
       </c>
       <c r="I7" t="str">
         <v>Open</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-20T21:43:08.173Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I26"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1092,9 +1092,38 @@
         <v>Linked: DEBT-05 (Binison)</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>TXN-1023</v>
+      </c>
+      <c r="B26" t="str">
+        <v>2026-07-05</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Transfer</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Transfer</v>
+      </c>
+      <c r="E26" t="str">
+        <v>EMI Savings</v>
+      </c>
+      <c r="F26">
+        <v>50000</v>
+      </c>
+      <c r="G26" t="str">
+        <v>HDFC- Info → SBI</v>
+      </c>
+      <c r="H26" t="str">
+        <v/>
+      </c>
+      <c r="I26" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I26"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1185,10 +1214,10 @@
         <v>219562</v>
       </c>
       <c r="G4">
-        <v>110503.77</v>
+        <v>160503.77</v>
       </c>
       <c r="H4">
-        <v>115521.23</v>
+        <v>65521.23</v>
       </c>
       <c r="I4" t="str">
         <v>2026-07-20</v>
@@ -1197,7 +1226,7 @@
         <v>140134.46</v>
       </c>
       <c r="K4">
-        <v>-24613.23</v>
+        <v>-74613.23</v>
       </c>
       <c r="L4" t="str">
         <v>Discrepancy</v>
@@ -1258,13 +1287,13 @@
         <v>123024.2</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>50000</v>
       </c>
       <c r="G6">
         <v>0</v>
       </c>
       <c r="H6">
-        <v>123024.2</v>
+        <v>173024.2</v>
       </c>
       <c r="I6" t="str">
         <v/>
@@ -1273,10 +1302,10 @@
         <v>123024.2</v>
       </c>
       <c r="K6">
-        <v>0</v>
+        <v>50000</v>
       </c>
       <c r="L6" t="str">
-        <v>Reconciled</v>
+        <v>Discrepancy</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-20T21:44:59.048Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -1272,66 +1272,66 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ACC-04</v>
+        <v>ACC-01</v>
       </c>
       <c r="B6" t="str">
-        <v>SBI</v>
+        <v>HDFC- Aluva</v>
       </c>
       <c r="C6" t="str">
-        <v>43602594069</v>
+        <v>50100523900334</v>
       </c>
       <c r="D6" t="str">
         <v>Savings</v>
       </c>
       <c r="E6">
-        <v>123024.2</v>
+        <v>11078.46</v>
       </c>
       <c r="F6">
-        <v>50000</v>
+        <v>20028</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>5891</v>
       </c>
       <c r="H6">
-        <v>173024.2</v>
+        <v>25215.46</v>
       </c>
       <c r="I6" t="str">
         <v/>
       </c>
-      <c r="J6">
-        <v>123024.2</v>
-      </c>
-      <c r="K6">
-        <v>50000</v>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v/>
       </c>
       <c r="L6" t="str">
-        <v>Discrepancy</v>
+        <v>Pending</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ACC-01</v>
+        <v>ACC-04</v>
       </c>
       <c r="B7" t="str">
-        <v>HDFC- Aluva</v>
+        <v>SBI</v>
       </c>
       <c r="C7" t="str">
-        <v>50100523900334</v>
+        <v>43602594069</v>
       </c>
       <c r="D7" t="str">
         <v>Savings</v>
       </c>
       <c r="E7">
-        <v>11078.46</v>
+        <v>184324.2</v>
       </c>
       <c r="F7">
-        <v>20028</v>
+        <v>50000</v>
       </c>
       <c r="G7">
-        <v>5891</v>
+        <v>0</v>
       </c>
       <c r="H7">
-        <v>25215.46</v>
+        <v>234324.2</v>
       </c>
       <c r="I7" t="str">
         <v/>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-20T21:45:34.209Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -1322,7 +1322,7 @@
         <v>Savings</v>
       </c>
       <c r="E7">
-        <v>184324.2</v>
+        <v>84324.2</v>
       </c>
       <c r="F7">
         <v>50000</v>
@@ -1331,7 +1331,7 @@
         <v>0</v>
       </c>
       <c r="H7">
-        <v>234324.2</v>
+        <v>134324.2</v>
       </c>
       <c r="I7" t="str">
         <v/>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-20T21:47:57.562Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I27"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1121,9 +1121,38 @@
         <v/>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>TXN-1024</v>
+      </c>
+      <c r="B27" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Income</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Debt Settlement</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Shilpa</v>
+      </c>
+      <c r="F27">
+        <v>15000</v>
+      </c>
+      <c r="G27" t="str">
+        <v>Federal-Ang</v>
+      </c>
+      <c r="H27" t="str">
+        <v>GPay</v>
+      </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I27"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1249,13 +1278,13 @@
         <v>18944</v>
       </c>
       <c r="F5">
-        <v>200</v>
+        <v>15200</v>
       </c>
       <c r="G5">
         <v>3859.9</v>
       </c>
       <c r="H5">
-        <v>15284.1</v>
+        <v>30284.1</v>
       </c>
       <c r="I5" t="str">
         <v>2026-07-20</v>
@@ -1264,7 +1293,7 @@
         <v>30367.1</v>
       </c>
       <c r="K5">
-        <v>-15083</v>
+        <v>-83</v>
       </c>
       <c r="L5" t="str">
         <v>Discrepancy</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-20T21:48:58.021Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I28"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1150,9 +1150,38 @@
         <v/>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>TXN-1025</v>
+      </c>
+      <c r="B28" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Investment</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Invested in APY Pension</v>
+      </c>
+      <c r="F28">
+        <v>409</v>
+      </c>
+      <c r="G28" t="str">
+        <v>Federal-Ang</v>
+      </c>
+      <c r="H28" t="str">
+        <v/>
+      </c>
+      <c r="I28" t="str">
+        <v>Linked: INV-04</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I28"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1281,10 +1310,10 @@
         <v>15200</v>
       </c>
       <c r="G5">
-        <v>3859.9</v>
+        <v>4268.9</v>
       </c>
       <c r="H5">
-        <v>30284.1</v>
+        <v>29875.1</v>
       </c>
       <c r="I5" t="str">
         <v>2026-07-20</v>
@@ -1293,7 +1322,7 @@
         <v>30367.1</v>
       </c>
       <c r="K5">
-        <v>-83</v>
+        <v>-492</v>
       </c>
       <c r="L5" t="str">
         <v>Discrepancy</v>
@@ -1675,25 +1704,25 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>INV-01</v>
+        <v>INV-02</v>
       </c>
       <c r="B4" t="str">
-        <v>APY Pension</v>
+        <v>Coin by Zerodha</v>
       </c>
       <c r="C4" t="str">
-        <v>Funds</v>
+        <v>Stocks</v>
       </c>
       <c r="D4" t="str">
-        <v>2026-07-01</v>
+        <v>2026-07-05</v>
       </c>
       <c r="E4">
-        <v>409</v>
+        <v>1996</v>
       </c>
       <c r="F4">
-        <v>409</v>
+        <v>2300</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>304</v>
       </c>
       <c r="H4" t="str">
         <v>Federal-Ang</v>
@@ -1713,7 +1742,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>INV-02</v>
+        <v>INV-03</v>
       </c>
       <c r="B5" t="str">
         <v>Coin by Zerodha</v>
@@ -1725,13 +1754,13 @@
         <v>2026-07-05</v>
       </c>
       <c r="E5">
-        <v>1996</v>
+        <v>1331</v>
       </c>
       <c r="F5">
-        <v>2300</v>
+        <v>1331</v>
       </c>
       <c r="G5">
-        <v>304</v>
+        <v>0</v>
       </c>
       <c r="H5" t="str">
         <v>Federal-Ang</v>
@@ -1751,22 +1780,22 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>INV-03</v>
+        <v>INV-04</v>
       </c>
       <c r="B6" t="str">
-        <v>Coin by Zerodha</v>
+        <v>APY Pension</v>
       </c>
       <c r="C6" t="str">
-        <v>Stocks</v>
+        <v>Funds</v>
       </c>
       <c r="D6" t="str">
-        <v>2026-07-05</v>
+        <v>2026-07-01</v>
       </c>
       <c r="E6">
-        <v>1331</v>
+        <v>409</v>
       </c>
       <c r="F6">
-        <v>1331</v>
+        <v>409</v>
       </c>
       <c r="G6">
         <v>0</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-20T22:13:01.333Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I30"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1179,9 +1179,67 @@
         <v>Linked: INV-04</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>TXN-1026</v>
+      </c>
+      <c r="B29" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Investment</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Invested in Coin by Zerodha</v>
+      </c>
+      <c r="F29">
+        <v>1331</v>
+      </c>
+      <c r="G29" t="str">
+        <v>Federal-Ang</v>
+      </c>
+      <c r="H29" t="str">
+        <v/>
+      </c>
+      <c r="I29" t="str">
+        <v>Linked: INV-05</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>TXN-1027</v>
+      </c>
+      <c r="B30" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Investment</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Invested in Coin by Zerodha</v>
+      </c>
+      <c r="F30">
+        <v>1996</v>
+      </c>
+      <c r="G30" t="str">
+        <v>Federal-Ang</v>
+      </c>
+      <c r="H30" t="str">
+        <v/>
+      </c>
+      <c r="I30" t="str">
+        <v>Linked: INV-06</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I30"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1310,10 +1368,10 @@
         <v>15200</v>
       </c>
       <c r="G5">
-        <v>4268.9</v>
+        <v>7595.9</v>
       </c>
       <c r="H5">
-        <v>29875.1</v>
+        <v>26548.1</v>
       </c>
       <c r="I5" t="str">
         <v>2026-07-20</v>
@@ -1322,7 +1380,7 @@
         <v>30367.1</v>
       </c>
       <c r="K5">
-        <v>-492</v>
+        <v>-3819</v>
       </c>
       <c r="L5" t="str">
         <v>Discrepancy</v>
@@ -1704,25 +1762,25 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>INV-02</v>
+        <v>INV-04</v>
       </c>
       <c r="B4" t="str">
-        <v>Coin by Zerodha</v>
+        <v>APY Pension</v>
       </c>
       <c r="C4" t="str">
-        <v>Stocks</v>
+        <v>Funds</v>
       </c>
       <c r="D4" t="str">
-        <v>2026-07-05</v>
+        <v>2026-07-01</v>
       </c>
       <c r="E4">
-        <v>1996</v>
+        <v>409</v>
       </c>
       <c r="F4">
-        <v>2300</v>
+        <v>409</v>
       </c>
       <c r="G4">
-        <v>304</v>
+        <v>0</v>
       </c>
       <c r="H4" t="str">
         <v>Federal-Ang</v>
@@ -1742,7 +1800,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>INV-03</v>
+        <v>INV-05</v>
       </c>
       <c r="B5" t="str">
         <v>Coin by Zerodha</v>
@@ -1751,7 +1809,7 @@
         <v>Stocks</v>
       </c>
       <c r="D5" t="str">
-        <v>2026-07-05</v>
+        <v>2026-07-01</v>
       </c>
       <c r="E5">
         <v>1331</v>
@@ -1780,22 +1838,22 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>INV-04</v>
+        <v>INV-06</v>
       </c>
       <c r="B6" t="str">
-        <v>APY Pension</v>
+        <v>Coin by Zerodha</v>
       </c>
       <c r="C6" t="str">
-        <v>Funds</v>
+        <v>Stocks</v>
       </c>
       <c r="D6" t="str">
         <v>2026-07-01</v>
       </c>
       <c r="E6">
-        <v>409</v>
+        <v>1996</v>
       </c>
       <c r="F6">
-        <v>409</v>
+        <v>1996</v>
       </c>
       <c r="G6">
         <v>0</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-20T22:16:08.894Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I32"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1237,9 +1237,67 @@
         <v>Linked: INV-06</v>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>TXN-1028</v>
+      </c>
+      <c r="B31" t="str">
+        <v>2026-07-09</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Income</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Dividends / Profit</v>
+      </c>
+      <c r="E31" t="str">
+        <v>TMPVL</v>
+      </c>
+      <c r="F31">
+        <v>78</v>
+      </c>
+      <c r="G31" t="str">
+        <v>Federal-Ang</v>
+      </c>
+      <c r="H31" t="str">
+        <v>Bank Transfer</v>
+      </c>
+      <c r="I31" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>TXN-1029</v>
+      </c>
+      <c r="B32" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Debt Given</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Lent to Baby</v>
+      </c>
+      <c r="F32">
+        <v>25000</v>
+      </c>
+      <c r="G32" t="str">
+        <v>Federal-Ang</v>
+      </c>
+      <c r="H32" t="str">
+        <v/>
+      </c>
+      <c r="I32" t="str">
+        <v>Linked: DEBT-06 (Baby)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I30"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I32"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1365,13 +1423,13 @@
         <v>18944</v>
       </c>
       <c r="F5">
-        <v>15200</v>
+        <v>15278</v>
       </c>
       <c r="G5">
-        <v>7595.9</v>
+        <v>32595.9</v>
       </c>
       <c r="H5">
-        <v>26548.1</v>
+        <v>1626.1</v>
       </c>
       <c r="I5" t="str">
         <v>2026-07-20</v>
@@ -1380,7 +1438,7 @@
         <v>30367.1</v>
       </c>
       <c r="K5">
-        <v>-3819</v>
+        <v>-28741</v>
       </c>
       <c r="L5" t="str">
         <v>Discrepancy</v>
@@ -1537,28 +1595,28 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>DEBT-02</v>
+        <v>LOAN-01</v>
       </c>
       <c r="B4" t="str">
-        <v>Debt Receivable</v>
+        <v>Bank Loan Payable</v>
       </c>
       <c r="C4" t="str">
-        <v>Baby Antony</v>
+        <v>SBI Home Loan</v>
       </c>
       <c r="D4" t="str">
-        <v>Money Given</v>
+        <v>Housing Loan</v>
       </c>
       <c r="E4">
-        <v>25000</v>
+        <v>5758624</v>
       </c>
       <c r="F4">
-        <v>25000</v>
+        <v>5758624</v>
       </c>
       <c r="G4" t="str">
-        <v>2026-07-01</v>
+        <v>2026-08-14</v>
       </c>
       <c r="H4" t="str">
-        <v>2026-08-01</v>
+        <v/>
       </c>
       <c r="I4" t="str">
         <v>Open</v>
@@ -1575,25 +1633,25 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>LOAN-01</v>
+        <v>DEBT-04</v>
       </c>
       <c r="B5" t="str">
-        <v>Bank Loan Payable</v>
+        <v>Debt Receivable</v>
       </c>
       <c r="C5" t="str">
-        <v>SBI Home Loan</v>
+        <v>Jomisha</v>
       </c>
       <c r="D5" t="str">
-        <v>Housing Loan</v>
+        <v>Sisy</v>
       </c>
       <c r="E5">
-        <v>5758624</v>
+        <v>5000</v>
       </c>
       <c r="F5">
-        <v>5758624</v>
+        <v>5000</v>
       </c>
       <c r="G5" t="str">
-        <v>2026-08-14</v>
+        <v>2026-07-13</v>
       </c>
       <c r="H5" t="str">
         <v/>
@@ -1613,28 +1671,28 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>DEBT-04</v>
+        <v>DEBT-05</v>
       </c>
       <c r="B6" t="str">
         <v>Debt Receivable</v>
       </c>
       <c r="C6" t="str">
-        <v>Jomisha</v>
+        <v>Binison</v>
       </c>
       <c r="D6" t="str">
-        <v>Sisy</v>
+        <v>Friend</v>
       </c>
       <c r="E6">
-        <v>5000</v>
+        <v>1500</v>
       </c>
       <c r="F6">
-        <v>5000</v>
+        <v>1500</v>
       </c>
       <c r="G6" t="str">
-        <v>2026-07-13</v>
+        <v>2026-07-19</v>
       </c>
       <c r="H6" t="str">
-        <v/>
+        <v>2026-08-20</v>
       </c>
       <c r="I6" t="str">
         <v>Open</v>
@@ -1651,28 +1709,28 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>DEBT-05</v>
+        <v>DEBT-06</v>
       </c>
       <c r="B7" t="str">
         <v>Debt Receivable</v>
       </c>
       <c r="C7" t="str">
-        <v>Binison</v>
+        <v>Baby</v>
       </c>
       <c r="D7" t="str">
         <v>Friend</v>
       </c>
       <c r="E7">
-        <v>1500</v>
+        <v>25000</v>
       </c>
       <c r="F7">
-        <v>1500</v>
+        <v>25000</v>
       </c>
       <c r="G7" t="str">
-        <v>2026-07-19</v>
+        <v>2026-07-01</v>
       </c>
       <c r="H7" t="str">
-        <v>2026-08-20</v>
+        <v>2026-08-01</v>
       </c>
       <c r="I7" t="str">
         <v>Open</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-20T22:18:21.384Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I33"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1295,9 +1295,38 @@
         <v>Linked: DEBT-06 (Baby)</v>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>TXN-1030</v>
+      </c>
+      <c r="B33" t="str">
+        <v>2026-07-20</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Income</v>
+      </c>
+      <c r="D33" t="str">
+        <v>For CC Payment</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Shibin Washing machine - Icici Amazon Pay</v>
+      </c>
+      <c r="F33">
+        <v>33105</v>
+      </c>
+      <c r="G33" t="str">
+        <v>Federal-Ang</v>
+      </c>
+      <c r="H33" t="str">
+        <v>Bank Transfer</v>
+      </c>
+      <c r="I33" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I33"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1423,13 +1452,13 @@
         <v>18944</v>
       </c>
       <c r="F5">
-        <v>15278</v>
+        <v>48383</v>
       </c>
       <c r="G5">
         <v>32595.9</v>
       </c>
       <c r="H5">
-        <v>1626.1</v>
+        <v>34731.1</v>
       </c>
       <c r="I5" t="str">
         <v>2026-07-20</v>
@@ -1438,7 +1467,7 @@
         <v>30367.1</v>
       </c>
       <c r="K5">
-        <v>-28741</v>
+        <v>4364</v>
       </c>
       <c r="L5" t="str">
         <v>Discrepancy</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-22T11:09:21.578Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I34"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1324,9 +1324,38 @@
         <v/>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>TXN-1031</v>
+      </c>
+      <c r="B34" t="str">
+        <v>2026-07-22</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Debt Given</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Lent to Albert</v>
+      </c>
+      <c r="F34">
+        <v>78700</v>
+      </c>
+      <c r="G34" t="str">
+        <v>SBI</v>
+      </c>
+      <c r="H34" t="str">
+        <v/>
+      </c>
+      <c r="I34" t="str">
+        <v>Linked: DEBT-07 (Albert)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I34"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1531,10 +1560,10 @@
         <v>50000</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <v>78700</v>
       </c>
       <c r="H7">
-        <v>134324.2</v>
+        <v>55624.2</v>
       </c>
       <c r="I7" t="str">
         <v/>
@@ -1558,7 +1587,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -1774,9 +1803,47 @@
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>DEBT-07</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Debt Receivable</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Albert</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Friend paid through husain ikka</v>
+      </c>
+      <c r="E8">
+        <v>78700</v>
+      </c>
+      <c r="F8">
+        <v>78700</v>
+      </c>
+      <c r="G8" t="str">
+        <v>2026-07-22</v>
+      </c>
+      <c r="H8" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="I8" t="str">
+        <v>Open</v>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L8"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-22T15:18:43.027Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I35"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1353,9 +1353,38 @@
         <v>Linked: DEBT-07 (Albert)</v>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>TXN-1032</v>
+      </c>
+      <c r="B35" t="str">
+        <v>2026-07-22</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Groceries</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Guest visit mary jincy</v>
+      </c>
+      <c r="F35">
+        <v>3000</v>
+      </c>
+      <c r="G35" t="str">
+        <v>Federal-Ang</v>
+      </c>
+      <c r="H35" t="str">
+        <v>GPay</v>
+      </c>
+      <c r="I35" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I35"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1484,10 +1513,10 @@
         <v>48383</v>
       </c>
       <c r="G5">
-        <v>32595.9</v>
+        <v>35595.9</v>
       </c>
       <c r="H5">
-        <v>34731.1</v>
+        <v>31731.1</v>
       </c>
       <c r="I5" t="str">
         <v>2026-07-20</v>
@@ -1496,7 +1525,7 @@
         <v>30367.1</v>
       </c>
       <c r="K5">
-        <v>4364</v>
+        <v>1364</v>
       </c>
       <c r="L5" t="str">
         <v>Discrepancy</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-22T18:44:28.380Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -1057,7 +1057,7 @@
         <v>HDFC- Info</v>
       </c>
       <c r="H24" t="str">
-        <v/>
+        <v>GPay</v>
       </c>
       <c r="I24" t="str">
         <v>Linked: DEBT-04 (Jomisha)</v>
@@ -1086,7 +1086,7 @@
         <v>HDFC- Info</v>
       </c>
       <c r="H25" t="str">
-        <v/>
+        <v>GPay</v>
       </c>
       <c r="I25" t="str">
         <v>Linked: DEBT-05 (Binison)</v>
@@ -1347,7 +1347,7 @@
         <v>SBI</v>
       </c>
       <c r="H34" t="str">
-        <v/>
+        <v>GPay</v>
       </c>
       <c r="I34" t="str">
         <v>Linked: DEBT-07 (Albert)</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-22T19:33:49.512Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -1289,10 +1289,10 @@
         <v>Federal-Ang</v>
       </c>
       <c r="H32" t="str">
-        <v/>
+        <v>GPay</v>
       </c>
       <c r="I32" t="str">
-        <v>Linked: DEBT-06 (Baby)</v>
+        <v/>
       </c>
     </row>
     <row r="33">

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-24T11:25:51.694Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -500,7 +500,7 @@
         <v>Perdiem and allowance</v>
       </c>
       <c r="F5">
-        <v>105229</v>
+        <v>95229</v>
       </c>
       <c r="G5" t="str">
         <v>HDFC- Info</v>
@@ -509,7 +509,7 @@
         <v>Direct Credit</v>
       </c>
       <c r="I5" t="str">
-        <v>Allowance</v>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -1472,13 +1472,13 @@
         <v>6463</v>
       </c>
       <c r="F4">
-        <v>219562</v>
+        <v>209562</v>
       </c>
       <c r="G4">
         <v>160503.77</v>
       </c>
       <c r="H4">
-        <v>65521.23</v>
+        <v>55521.23</v>
       </c>
       <c r="I4" t="str">
         <v>2026-07-20</v>
@@ -1487,7 +1487,7 @@
         <v>140134.46</v>
       </c>
       <c r="K4">
-        <v>-74613.23</v>
+        <v>-84613.23</v>
       </c>
       <c r="L4" t="str">
         <v>Discrepancy</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-24T11:26:02.271Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -471,7 +471,7 @@
         <v>Monthly salary</v>
       </c>
       <c r="F4">
-        <v>113175</v>
+        <v>13175</v>
       </c>
       <c r="G4" t="str">
         <v>HDFC- Info</v>
@@ -480,7 +480,7 @@
         <v>Direct Credit</v>
       </c>
       <c r="I4" t="str">
-        <v>July Payroll</v>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -1472,13 +1472,13 @@
         <v>6463</v>
       </c>
       <c r="F4">
-        <v>209562</v>
+        <v>109562</v>
       </c>
       <c r="G4">
         <v>160503.77</v>
       </c>
       <c r="H4">
-        <v>55521.23</v>
+        <v>-44478.77</v>
       </c>
       <c r="I4" t="str">
         <v>2026-07-20</v>
@@ -1487,7 +1487,7 @@
         <v>140134.46</v>
       </c>
       <c r="K4">
-        <v>-84613.23</v>
+        <v>-184613.23</v>
       </c>
       <c r="L4" t="str">
         <v>Discrepancy</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-24T18:07:40.920Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -471,7 +471,7 @@
         <v>Monthly salary</v>
       </c>
       <c r="F4">
-        <v>13175</v>
+        <v>113175</v>
       </c>
       <c r="G4" t="str">
         <v>HDFC- Info</v>
@@ -1472,13 +1472,13 @@
         <v>6463</v>
       </c>
       <c r="F4">
-        <v>109562</v>
+        <v>209562</v>
       </c>
       <c r="G4">
         <v>160503.77</v>
       </c>
       <c r="H4">
-        <v>-44478.77</v>
+        <v>55521.23</v>
       </c>
       <c r="I4" t="str">
         <v>2026-07-20</v>
@@ -1487,7 +1487,7 @@
         <v>140134.46</v>
       </c>
       <c r="K4">
-        <v>-184613.23</v>
+        <v>-84613.23</v>
       </c>
       <c r="L4" t="str">
         <v>Discrepancy</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-24T18:07:58.962Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -500,7 +500,7 @@
         <v>Perdiem and allowance</v>
       </c>
       <c r="F5">
-        <v>95229</v>
+        <v>105229</v>
       </c>
       <c r="G5" t="str">
         <v>HDFC- Info</v>
@@ -1472,13 +1472,13 @@
         <v>6463</v>
       </c>
       <c r="F4">
-        <v>209562</v>
+        <v>219562</v>
       </c>
       <c r="G4">
         <v>160503.77</v>
       </c>
       <c r="H4">
-        <v>55521.23</v>
+        <v>65521.23</v>
       </c>
       <c r="I4" t="str">
         <v>2026-07-20</v>
@@ -1487,7 +1487,7 @@
         <v>140134.46</v>
       </c>
       <c r="K4">
-        <v>-84613.23</v>
+        <v>-74613.23</v>
       </c>
       <c r="L4" t="str">
         <v>Discrepancy</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-07-31T09:58:54.712Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -1421,7 +1421,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:M7"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -1435,6 +1435,7 @@
     <col min="10" max="10" width="16.83203125" customWidth="1"/>
     <col min="11" max="11" width="12.83203125" customWidth="1"/>
     <col min="12" max="12" width="18.83203125" customWidth="1"/>
+    <col min="13" max="13" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1484,6 +1485,9 @@
       <c r="L3" t="str">
         <v>Reconciliation Status</v>
       </c>
+      <c r="M3" t="str">
+        <v>Main Account</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -1522,6 +1526,9 @@
       <c r="L4" t="str">
         <v>Discrepancy</v>
       </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -1560,6 +1567,9 @@
       <c r="L5" t="str">
         <v>Discrepancy</v>
       </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -1598,6 +1608,9 @@
       <c r="L6" t="str">
         <v>Pending</v>
       </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -1636,17 +1649,20 @@
       <c r="L7" t="str">
         <v>Pending</v>
       </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q8"/>
+  <dimension ref="A1:R8"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -1729,6 +1745,9 @@
       <c r="Q3" t="str">
         <v>Auto-Posted Txn Ref</v>
       </c>
+      <c r="R3" t="str">
+        <v>Main Account</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -1782,6 +1801,9 @@
       <c r="Q4" t="str">
         <v/>
       </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -1835,6 +1857,9 @@
       <c r="Q5" t="str">
         <v/>
       </c>
+      <c r="R5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -1888,6 +1913,9 @@
       <c r="Q6" t="str">
         <v/>
       </c>
+      <c r="R6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -1941,6 +1969,9 @@
       <c r="Q7" t="str">
         <v/>
       </c>
+      <c r="R7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -1994,17 +2025,20 @@
       <c r="Q8" t="str">
         <v/>
       </c>
+      <c r="R8" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R8"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:M6"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -2067,6 +2101,9 @@
       <c r="L3" t="str">
         <v>Auto-Posted Txn Ref</v>
       </c>
+      <c r="M3" t="str">
+        <v>Main Account</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -2105,6 +2142,9 @@
       <c r="L4" t="str">
         <v/>
       </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -2143,6 +2183,9 @@
       <c r="L5" t="str">
         <v/>
       </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -2181,17 +2224,20 @@
       <c r="L6" t="str">
         <v/>
       </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F46"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -2313,30 +2359,30 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>12001</v>
+        <v>11101</v>
       </c>
       <c r="B8" t="str">
-        <v>APY Pension</v>
+        <v>Cash Account</v>
       </c>
       <c r="C8" t="str">
         <v>Asset</v>
       </c>
       <c r="D8" t="str">
-        <v>Investments</v>
+        <v>Cash &amp; Bank</v>
       </c>
       <c r="E8" t="str">
-        <v>Pension</v>
+        <v>Cash</v>
       </c>
       <c r="F8" t="str">
-        <v>apy</v>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>12002</v>
+        <v>12001</v>
       </c>
       <c r="B9" t="str">
-        <v>Zerodha Coin</v>
+        <v>APY Pension</v>
       </c>
       <c r="C9" t="str">
         <v>Asset</v>
@@ -2345,18 +2391,18 @@
         <v>Investments</v>
       </c>
       <c r="E9" t="str">
-        <v>Mutual Funds / Stocks</v>
+        <v>Pension</v>
       </c>
       <c r="F9" t="str">
-        <v>zerodha,coin</v>
+        <v>apy</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>12099</v>
+        <v>12002</v>
       </c>
       <c r="B10" t="str">
-        <v>Other Investments</v>
+        <v>Zerodha Coin</v>
       </c>
       <c r="C10" t="str">
         <v>Asset</v>
@@ -2365,158 +2411,158 @@
         <v>Investments</v>
       </c>
       <c r="E10" t="str">
-        <v>General</v>
+        <v>Mutual Funds / Stocks</v>
       </c>
       <c r="F10" t="str">
-        <v>nps,ppf,fd,deposit</v>
+        <v>zerodha,coin</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>13001</v>
+        <v>12099</v>
       </c>
       <c r="B11" t="str">
-        <v>Loans Given (Receivables)</v>
+        <v>Other Investments</v>
       </c>
       <c r="C11" t="str">
         <v>Asset</v>
       </c>
       <c r="D11" t="str">
-        <v>Receivables</v>
+        <v>Investments</v>
       </c>
       <c r="E11" t="str">
-        <v>Personal Loans Given</v>
+        <v>General</v>
       </c>
       <c r="F11" t="str">
-        <v>lent,jomisha,binison,albert</v>
+        <v>nps,ppf,fd,deposit</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>21001</v>
+        <v>13001</v>
       </c>
       <c r="B12" t="str">
-        <v>SBI Home Loan</v>
+        <v>Loans Given (Receivables)</v>
       </c>
       <c r="C12" t="str">
-        <v>Liability</v>
+        <v>Asset</v>
       </c>
       <c r="D12" t="str">
-        <v>Bank Loans</v>
+        <v>Receivables</v>
       </c>
       <c r="E12" t="str">
-        <v>Housing Loan</v>
+        <v>Personal Loans Given</v>
       </c>
       <c r="F12" t="str">
-        <v>home loan,housing loan</v>
+        <v>lent,jomisha,binison,albert</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>22001</v>
+        <v>21001</v>
       </c>
       <c r="B13" t="str">
-        <v>Personal Borrowings</v>
+        <v>SBI Home Loan</v>
       </c>
       <c r="C13" t="str">
         <v>Liability</v>
       </c>
       <c r="D13" t="str">
-        <v>Debts Payable</v>
+        <v>Bank Loans</v>
       </c>
       <c r="E13" t="str">
-        <v>From People</v>
+        <v>Housing Loan</v>
       </c>
       <c r="F13" t="str">
-        <v>borrowed</v>
+        <v>home loan,housing loan</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>23001</v>
+        <v>22001</v>
       </c>
       <c r="B14" t="str">
-        <v>Credit Card Payable</v>
+        <v>Personal Borrowings</v>
       </c>
       <c r="C14" t="str">
         <v>Liability</v>
       </c>
       <c r="D14" t="str">
-        <v>Credit Cards</v>
+        <v>Debts Payable</v>
       </c>
       <c r="E14" t="str">
-        <v>ICICI Amazon Pay</v>
+        <v>From People</v>
       </c>
       <c r="F14" t="str">
-        <v>icici amazon</v>
+        <v>borrowed</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>30001</v>
+        <v>23001</v>
       </c>
       <c r="B15" t="str">
-        <v>Opening Balances / Net Worth</v>
+        <v>Credit Card Payable</v>
       </c>
       <c r="C15" t="str">
-        <v>Equity</v>
+        <v>Liability</v>
       </c>
       <c r="D15" t="str">
-        <v>Capital</v>
+        <v>Credit Cards</v>
       </c>
       <c r="E15" t="str">
-        <v>Opening Balance</v>
+        <v>ICICI Amazon Pay</v>
       </c>
       <c r="F15" t="str">
-        <v/>
+        <v>icici amazon</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>41001</v>
+        <v>30001</v>
       </c>
       <c r="B16" t="str">
-        <v>Salary</v>
+        <v>Opening Balances / Net Worth</v>
       </c>
       <c r="C16" t="str">
-        <v>Income</v>
+        <v>Equity</v>
       </c>
       <c r="D16" t="str">
-        <v>Employment</v>
+        <v>Capital</v>
       </c>
       <c r="E16" t="str">
-        <v>Monthly Salary</v>
+        <v>Opening Balance</v>
       </c>
       <c r="F16" t="str">
-        <v>salary,sal cr,infopark</v>
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>41002</v>
+        <v>41001</v>
       </c>
       <c r="B17" t="str">
-        <v>Business Income</v>
+        <v>Salary</v>
       </c>
       <c r="C17" t="str">
         <v>Income</v>
       </c>
       <c r="D17" t="str">
-        <v>Business</v>
+        <v>Employment</v>
       </c>
       <c r="E17" t="str">
-        <v>General</v>
+        <v>Monthly Salary</v>
       </c>
       <c r="F17" t="str">
-        <v>business</v>
+        <v>salary,sal cr,infopark</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>41003</v>
+        <v>41002</v>
       </c>
       <c r="B18" t="str">
-        <v>Freelance Income</v>
+        <v>Business Income</v>
       </c>
       <c r="C18" t="str">
         <v>Income</v>
@@ -2525,38 +2571,38 @@
         <v>Business</v>
       </c>
       <c r="E18" t="str">
-        <v>Freelance</v>
+        <v>General</v>
       </c>
       <c r="F18" t="str">
-        <v>freelance</v>
+        <v>business</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>42001</v>
+        <v>41003</v>
       </c>
       <c r="B19" t="str">
-        <v>Interest Income</v>
+        <v>Freelance Income</v>
       </c>
       <c r="C19" t="str">
         <v>Income</v>
       </c>
       <c r="D19" t="str">
-        <v>Investment Income</v>
+        <v>Business</v>
       </c>
       <c r="E19" t="str">
-        <v>Bank / FD Interest</v>
+        <v>Freelance</v>
       </c>
       <c r="F19" t="str">
-        <v>interest,int.pd,sbint,sb int</v>
+        <v>freelance</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>42002</v>
+        <v>42001</v>
       </c>
       <c r="B20" t="str">
-        <v>Dividend Income</v>
+        <v>Interest Income</v>
       </c>
       <c r="C20" t="str">
         <v>Income</v>
@@ -2565,38 +2611,38 @@
         <v>Investment Income</v>
       </c>
       <c r="E20" t="str">
-        <v>Dividends</v>
+        <v>Bank / FD Interest</v>
       </c>
       <c r="F20" t="str">
-        <v>dividend,div,achcr</v>
+        <v>interest,int.pd,sbint,sb int</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>43001</v>
+        <v>42002</v>
       </c>
       <c r="B21" t="str">
-        <v>Rental Income</v>
+        <v>Dividend Income</v>
       </c>
       <c r="C21" t="str">
         <v>Income</v>
       </c>
       <c r="D21" t="str">
-        <v>Other Income</v>
+        <v>Investment Income</v>
       </c>
       <c r="E21" t="str">
-        <v>Rent Received</v>
+        <v>Dividends</v>
       </c>
       <c r="F21" t="str">
-        <v>rent received</v>
+        <v>dividend,div,achcr</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>43002</v>
+        <v>43001</v>
       </c>
       <c r="B22" t="str">
-        <v>Gifts &amp; Allowance</v>
+        <v>Rental Income</v>
       </c>
       <c r="C22" t="str">
         <v>Income</v>
@@ -2605,18 +2651,18 @@
         <v>Other Income</v>
       </c>
       <c r="E22" t="str">
-        <v>Gifts</v>
+        <v>Rent Received</v>
       </c>
       <c r="F22" t="str">
-        <v>gift received</v>
+        <v>rent received</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>43003</v>
+        <v>43002</v>
       </c>
       <c r="B23" t="str">
-        <v>Debt Settlement Received</v>
+        <v>Gifts &amp; Allowance</v>
       </c>
       <c r="C23" t="str">
         <v>Income</v>
@@ -2625,18 +2671,18 @@
         <v>Other Income</v>
       </c>
       <c r="E23" t="str">
-        <v>Loan Repaid to You</v>
+        <v>Gifts</v>
       </c>
       <c r="F23" t="str">
-        <v>repayment</v>
+        <v>gift received</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>49999</v>
+        <v>43003</v>
       </c>
       <c r="B24" t="str">
-        <v>Other Income</v>
+        <v>Debt Settlement Received</v>
       </c>
       <c r="C24" t="str">
         <v>Income</v>
@@ -2645,38 +2691,38 @@
         <v>Other Income</v>
       </c>
       <c r="E24" t="str">
-        <v>Miscellaneous</v>
+        <v>Loan Repaid to You</v>
       </c>
       <c r="F24" t="str">
-        <v/>
+        <v>repayment</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>51001</v>
+        <v>49999</v>
       </c>
       <c r="B25" t="str">
-        <v>Rent / Housing</v>
+        <v>Other Income</v>
       </c>
       <c r="C25" t="str">
-        <v>Expense</v>
+        <v>Income</v>
       </c>
       <c r="D25" t="str">
-        <v>Household</v>
+        <v>Other Income</v>
       </c>
       <c r="E25" t="str">
-        <v>Rent &amp; Maintenance</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="F25" t="str">
-        <v>rent,maintenance</v>
+        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>51002</v>
+        <v>51001</v>
       </c>
       <c r="B26" t="str">
-        <v>Utilities - Electricity &amp; Water</v>
+        <v>Rent / Housing</v>
       </c>
       <c r="C26" t="str">
         <v>Expense</v>
@@ -2685,18 +2731,18 @@
         <v>Household</v>
       </c>
       <c r="E26" t="str">
-        <v>Electricity / Water</v>
+        <v>Rent &amp; Maintenance</v>
       </c>
       <c r="F26" t="str">
-        <v>kseb,electricity,water bill</v>
+        <v>rent,maintenance</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>51003</v>
+        <v>51002</v>
       </c>
       <c r="B27" t="str">
-        <v>Utilities - Internet &amp; Mobile</v>
+        <v>Utilities - Electricity &amp; Water</v>
       </c>
       <c r="C27" t="str">
         <v>Expense</v>
@@ -2705,18 +2751,18 @@
         <v>Household</v>
       </c>
       <c r="E27" t="str">
-        <v>Recharge / Broadband</v>
+        <v>Electricity / Water</v>
       </c>
       <c r="F27" t="str">
-        <v>recharge,airtel,jio,bsnl,broadband,wifi</v>
+        <v>kseb,electricity,water bill</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>51004</v>
+        <v>51003</v>
       </c>
       <c r="B28" t="str">
-        <v>Gas / LPG</v>
+        <v>Utilities - Internet &amp; Mobile</v>
       </c>
       <c r="C28" t="str">
         <v>Expense</v>
@@ -2725,18 +2771,18 @@
         <v>Household</v>
       </c>
       <c r="E28" t="str">
-        <v>Cooking Gas</v>
+        <v>Recharge / Broadband</v>
       </c>
       <c r="F28" t="str">
-        <v>lpg,indane,gas</v>
+        <v>recharge,airtel,jio,bsnl,broadband,wifi</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>51005</v>
+        <v>51004</v>
       </c>
       <c r="B29" t="str">
-        <v>Household Appliances</v>
+        <v>Gas / LPG</v>
       </c>
       <c r="C29" t="str">
         <v>Expense</v>
@@ -2745,38 +2791,38 @@
         <v>Household</v>
       </c>
       <c r="E29" t="str">
-        <v>Appliances &amp; Repairs</v>
+        <v>Cooking Gas</v>
       </c>
       <c r="F29" t="str">
-        <v>washing machine,appliance,repair</v>
+        <v>lpg,indane,gas</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>52001</v>
+        <v>51005</v>
       </c>
       <c r="B30" t="str">
-        <v>Groceries</v>
+        <v>Household Appliances</v>
       </c>
       <c r="C30" t="str">
         <v>Expense</v>
       </c>
       <c r="D30" t="str">
-        <v>Food</v>
+        <v>Household</v>
       </c>
       <c r="E30" t="str">
-        <v>Provisions</v>
+        <v>Appliances &amp; Repairs</v>
       </c>
       <c r="F30" t="str">
-        <v>grocery,supermarket,mart,bigbasket,blinkit,zepto,dmart</v>
+        <v>washing machine,appliance,repair</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>52002</v>
+        <v>52001</v>
       </c>
       <c r="B31" t="str">
-        <v>Dining Out</v>
+        <v>Groceries</v>
       </c>
       <c r="C31" t="str">
         <v>Expense</v>
@@ -2785,38 +2831,38 @@
         <v>Food</v>
       </c>
       <c r="E31" t="str">
-        <v>Restaurants &amp; Delivery</v>
+        <v>Provisions</v>
       </c>
       <c r="F31" t="str">
-        <v>swiggy,zomato,restaurant,hotel,cafe</v>
+        <v>grocery,supermarket,mart,bigbasket,blinkit,zepto,dmart</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>53001</v>
+        <v>52002</v>
       </c>
       <c r="B32" t="str">
-        <v>Transport &amp; Fuel</v>
+        <v>Dining Out</v>
       </c>
       <c r="C32" t="str">
         <v>Expense</v>
       </c>
       <c r="D32" t="str">
-        <v>Transport</v>
+        <v>Food</v>
       </c>
       <c r="E32" t="str">
-        <v>Fuel / Taxi / Toll</v>
+        <v>Restaurants &amp; Delivery</v>
       </c>
       <c r="F32" t="str">
-        <v>uber,ola,rapido,petrol,fuel,hpcl,bpcl,fastag</v>
+        <v>swiggy,zomato,restaurant,hotel,cafe</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>53002</v>
+        <v>53001</v>
       </c>
       <c r="B33" t="str">
-        <v>Travel</v>
+        <v>Transport &amp; Fuel</v>
       </c>
       <c r="C33" t="str">
         <v>Expense</v>
@@ -2825,38 +2871,38 @@
         <v>Transport</v>
       </c>
       <c r="E33" t="str">
-        <v>Trips &amp; Tickets</v>
+        <v>Fuel / Taxi / Toll</v>
       </c>
       <c r="F33" t="str">
-        <v>irctc,makemytrip,redbus,indigo</v>
+        <v>uber,ola,rapido,petrol,fuel,hpcl,bpcl,fastag</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>54001</v>
+        <v>53002</v>
       </c>
       <c r="B34" t="str">
-        <v>Family Support</v>
+        <v>Travel</v>
       </c>
       <c r="C34" t="str">
         <v>Expense</v>
       </c>
       <c r="D34" t="str">
-        <v>Family &amp; Personal</v>
+        <v>Transport</v>
       </c>
       <c r="E34" t="str">
-        <v>Family / Amma</v>
+        <v>Trips &amp; Tickets</v>
       </c>
       <c r="F34" t="str">
-        <v>amma,family</v>
+        <v>irctc,makemytrip,redbus,indigo</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>54002</v>
+        <v>54001</v>
       </c>
       <c r="B35" t="str">
-        <v>Health &amp; Medical</v>
+        <v>Family Support</v>
       </c>
       <c r="C35" t="str">
         <v>Expense</v>
@@ -2865,18 +2911,18 @@
         <v>Family &amp; Personal</v>
       </c>
       <c r="E35" t="str">
-        <v>Pharmacy / Hospital</v>
+        <v>Family / Amma</v>
       </c>
       <c r="F35" t="str">
-        <v>pharmacy,medical,hospital,clinic</v>
+        <v>amma,family</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>54003</v>
+        <v>54002</v>
       </c>
       <c r="B36" t="str">
-        <v>Education</v>
+        <v>Health &amp; Medical</v>
       </c>
       <c r="C36" t="str">
         <v>Expense</v>
@@ -2885,18 +2931,18 @@
         <v>Family &amp; Personal</v>
       </c>
       <c r="E36" t="str">
-        <v>Fees &amp; Courses</v>
+        <v>Pharmacy / Hospital</v>
       </c>
       <c r="F36" t="str">
-        <v>school,college,course,tuition</v>
+        <v>pharmacy,medical,hospital,clinic</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>54004</v>
+        <v>54003</v>
       </c>
       <c r="B37" t="str">
-        <v>Shopping</v>
+        <v>Education</v>
       </c>
       <c r="C37" t="str">
         <v>Expense</v>
@@ -2905,18 +2951,18 @@
         <v>Family &amp; Personal</v>
       </c>
       <c r="E37" t="str">
-        <v>Online &amp; Retail</v>
+        <v>Fees &amp; Courses</v>
       </c>
       <c r="F37" t="str">
-        <v>amazon,flipkart,myntra,ajio</v>
+        <v>school,college,course,tuition</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>54005</v>
+        <v>54004</v>
       </c>
       <c r="B38" t="str">
-        <v>Gifts &amp; Functions</v>
+        <v>Shopping</v>
       </c>
       <c r="C38" t="str">
         <v>Expense</v>
@@ -2925,38 +2971,38 @@
         <v>Family &amp; Personal</v>
       </c>
       <c r="E38" t="str">
-        <v>Guests &amp; Gifts</v>
+        <v>Online &amp; Retail</v>
       </c>
       <c r="F38" t="str">
-        <v>guest,marriage,function</v>
+        <v>amazon,flipkart,myntra,ajio</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>55001</v>
+        <v>54005</v>
       </c>
       <c r="B39" t="str">
-        <v>Loan EMI / Repayment</v>
+        <v>Gifts &amp; Functions</v>
       </c>
       <c r="C39" t="str">
         <v>Expense</v>
       </c>
       <c r="D39" t="str">
-        <v>Financial</v>
+        <v>Family &amp; Personal</v>
       </c>
       <c r="E39" t="str">
-        <v>EMIs</v>
+        <v>Guests &amp; Gifts</v>
       </c>
       <c r="F39" t="str">
-        <v>emi,loan repay</v>
+        <v>guest,marriage,function</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>55002</v>
+        <v>55001</v>
       </c>
       <c r="B40" t="str">
-        <v>Credit Card Payment</v>
+        <v>Loan EMI / Repayment</v>
       </c>
       <c r="C40" t="str">
         <v>Expense</v>
@@ -2965,18 +3011,18 @@
         <v>Financial</v>
       </c>
       <c r="E40" t="str">
-        <v>Card Bills</v>
+        <v>EMIs</v>
       </c>
       <c r="F40" t="str">
-        <v>cc payment,card payment</v>
+        <v>emi,loan repay</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>55003</v>
+        <v>55002</v>
       </c>
       <c r="B41" t="str">
-        <v>Investment Contribution</v>
+        <v>Credit Card Payment</v>
       </c>
       <c r="C41" t="str">
         <v>Expense</v>
@@ -2985,18 +3031,18 @@
         <v>Financial</v>
       </c>
       <c r="E41" t="str">
-        <v>SIP / Deposits</v>
+        <v>Card Bills</v>
       </c>
       <c r="F41" t="str">
-        <v>sip</v>
+        <v>cc payment,card payment</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>55004</v>
+        <v>55003</v>
       </c>
       <c r="B42" t="str">
-        <v>Debt Given (Lent Out)</v>
+        <v>Investment Contribution</v>
       </c>
       <c r="C42" t="str">
         <v>Expense</v>
@@ -3005,18 +3051,18 @@
         <v>Financial</v>
       </c>
       <c r="E42" t="str">
-        <v>Money Lent</v>
+        <v>SIP / Deposits</v>
       </c>
       <c r="F42" t="str">
-        <v>lent to</v>
+        <v>sip</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>55005</v>
+        <v>55004</v>
       </c>
       <c r="B43" t="str">
-        <v>Taxes &amp; GST</v>
+        <v>Debt Given (Lent Out)</v>
       </c>
       <c r="C43" t="str">
         <v>Expense</v>
@@ -3025,18 +3071,18 @@
         <v>Financial</v>
       </c>
       <c r="E43" t="str">
-        <v>GST / Filing</v>
+        <v>Money Lent</v>
       </c>
       <c r="F43" t="str">
-        <v>gst,filing fee,tax</v>
+        <v>lent to</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>55006</v>
+        <v>55005</v>
       </c>
       <c r="B44" t="str">
-        <v>Insurance</v>
+        <v>Taxes &amp; GST</v>
       </c>
       <c r="C44" t="str">
         <v>Expense</v>
@@ -3045,35 +3091,55 @@
         <v>Financial</v>
       </c>
       <c r="E44" t="str">
-        <v>Premiums</v>
+        <v>GST / Filing</v>
       </c>
       <c r="F44" t="str">
-        <v>insurance,lic,premium</v>
+        <v>gst,filing fee,tax</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
+        <v>55006</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Insurance</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Financial</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Premiums</v>
+      </c>
+      <c r="F45" t="str">
+        <v>insurance,lic,premium</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
         <v>59999</v>
       </c>
-      <c r="B45" t="str">
+      <c r="B46" t="str">
         <v>Other Expenses</v>
       </c>
-      <c r="C45" t="str">
-        <v>Expense</v>
-      </c>
-      <c r="D45" t="str">
+      <c r="C46" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D46" t="str">
         <v>Other</v>
       </c>
-      <c r="E45" t="str">
+      <c r="E46" t="str">
         <v>Miscellaneous</v>
       </c>
-      <c r="F45" t="str">
+      <c r="F46" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F45"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F46"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-15T19:24:40.239Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:K36"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -414,6 +414,8 @@
     <col min="7" max="7" width="20.83203125" customWidth="1"/>
     <col min="8" max="8" width="15.83203125" customWidth="1"/>
     <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
+    <col min="11" max="11" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -454,6 +456,12 @@
       <c r="I3" t="str">
         <v>Linked Entity Ref</v>
       </c>
+      <c r="J3" t="str">
+        <v>COA Account</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Bank Reference</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -483,6 +491,12 @@
       <c r="I4" t="str">
         <v>July Payroll</v>
       </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -512,6 +526,12 @@
       <c r="I5" t="str">
         <v>Allowance</v>
       </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -541,6 +561,12 @@
       <c r="I6" t="str">
         <v>Interest</v>
       </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -570,6 +596,12 @@
       <c r="I7" t="str">
         <v>CC Payment</v>
       </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -599,6 +631,12 @@
       <c r="I8" t="str">
         <v>CC Payment</v>
       </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -628,6 +666,12 @@
       <c r="I9" t="str">
         <v>Family</v>
       </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -657,6 +701,12 @@
       <c r="I10" t="str">
         <v>Family</v>
       </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -686,6 +736,12 @@
       <c r="I11" t="str">
         <v>Old debt repay</v>
       </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -715,6 +771,12 @@
       <c r="I12" t="str">
         <v>Utilities</v>
       </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -744,6 +806,12 @@
       <c r="I13" t="str">
         <v>Loan HDFC- Shibin</v>
       </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -773,6 +841,12 @@
       <c r="I14" t="str">
         <v>Dividend</v>
       </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -802,6 +876,12 @@
       <c r="I15" t="str">
         <v>Utilities</v>
       </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -831,6 +911,12 @@
       <c r="I16" t="str">
         <v>Family</v>
       </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -860,6 +946,12 @@
       <c r="I17" t="str">
         <v>Dividend</v>
       </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+      <c r="K17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -889,6 +981,12 @@
       <c r="I18" t="str">
         <v>Utilities</v>
       </c>
+      <c r="J18" t="str">
+        <v/>
+      </c>
+      <c r="K18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -918,6 +1016,12 @@
       <c r="I19" t="str">
         <v>GST Filing</v>
       </c>
+      <c r="J19" t="str">
+        <v/>
+      </c>
+      <c r="K19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -947,6 +1051,12 @@
       <c r="I20" t="str">
         <v>Family</v>
       </c>
+      <c r="J20" t="str">
+        <v/>
+      </c>
+      <c r="K20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -976,6 +1086,12 @@
       <c r="I21" t="str">
         <v>Family</v>
       </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
+      <c r="K21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -1005,6 +1121,12 @@
       <c r="I22" t="str">
         <v/>
       </c>
+      <c r="J22" t="str">
+        <v/>
+      </c>
+      <c r="K22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -1034,6 +1156,12 @@
       <c r="I23" t="str">
         <v/>
       </c>
+      <c r="J23" t="str">
+        <v/>
+      </c>
+      <c r="K23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -1063,6 +1191,12 @@
       <c r="I24" t="str">
         <v>Linked: DEBT-04 (Jomisha)</v>
       </c>
+      <c r="J24" t="str">
+        <v/>
+      </c>
+      <c r="K24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -1092,6 +1226,12 @@
       <c r="I25" t="str">
         <v>Linked: DEBT-05 (Binison)</v>
       </c>
+      <c r="J25" t="str">
+        <v/>
+      </c>
+      <c r="K25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -1121,6 +1261,12 @@
       <c r="I26" t="str">
         <v/>
       </c>
+      <c r="J26" t="str">
+        <v/>
+      </c>
+      <c r="K26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -1150,6 +1296,12 @@
       <c r="I27" t="str">
         <v/>
       </c>
+      <c r="J27" t="str">
+        <v/>
+      </c>
+      <c r="K27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -1179,6 +1331,12 @@
       <c r="I28" t="str">
         <v>Linked: INV-04</v>
       </c>
+      <c r="J28" t="str">
+        <v/>
+      </c>
+      <c r="K28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -1208,6 +1366,12 @@
       <c r="I29" t="str">
         <v>Linked: INV-05</v>
       </c>
+      <c r="J29" t="str">
+        <v/>
+      </c>
+      <c r="K29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -1237,6 +1401,12 @@
       <c r="I30" t="str">
         <v>Linked: INV-06</v>
       </c>
+      <c r="J30" t="str">
+        <v/>
+      </c>
+      <c r="K30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -1266,6 +1436,12 @@
       <c r="I31" t="str">
         <v/>
       </c>
+      <c r="J31" t="str">
+        <v/>
+      </c>
+      <c r="K31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -1295,6 +1471,12 @@
       <c r="I32" t="str">
         <v>Linked: DEBT-06 (Baby)</v>
       </c>
+      <c r="J32" t="str">
+        <v/>
+      </c>
+      <c r="K32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -1324,6 +1506,12 @@
       <c r="I33" t="str">
         <v/>
       </c>
+      <c r="J33" t="str">
+        <v/>
+      </c>
+      <c r="K33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -1353,6 +1541,12 @@
       <c r="I34" t="str">
         <v>Linked: DEBT-07 (Albert)</v>
       </c>
+      <c r="J34" t="str">
+        <v/>
+      </c>
+      <c r="K34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -1382,6 +1576,12 @@
       <c r="I35" t="str">
         <v/>
       </c>
+      <c r="J35" t="str">
+        <v/>
+      </c>
+      <c r="K35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -1411,10 +1611,16 @@
       <c r="I36" t="str">
         <v/>
       </c>
+      <c r="J36" t="str">
+        <v/>
+      </c>
+      <c r="K36" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K36"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3493,7 +3699,7 @@
         <v>Theme</v>
       </c>
       <c r="B6" t="str">
-        <v>dark</v>
+        <v>light</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-15T19:54:27.652Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:K37"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1618,9 +1618,44 @@
         <v/>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>TXN-1034</v>
+      </c>
+      <c r="B37" t="str">
+        <v>2026-07-08</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Family Support</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Payment to amma</v>
+      </c>
+      <c r="F37">
+        <v>1000</v>
+      </c>
+      <c r="G37" t="str">
+        <v>Federal-Ang</v>
+      </c>
+      <c r="H37" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="I37" t="str">
+        <v>Import: ACC_STATEMENT_XXXXX5530_23JUN2026_23JUL2026_1784733785805439.pdf (SECURED).pdf</v>
+      </c>
+      <c r="J37" t="str">
+        <v>54001</v>
+      </c>
+      <c r="K37" t="str">
+        <v>S20829825</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K37"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1756,10 +1791,10 @@
         <v>48383</v>
       </c>
       <c r="G5">
-        <v>38595.9</v>
+        <v>39595.9</v>
       </c>
       <c r="H5">
-        <v>28731.1</v>
+        <v>27731.1</v>
       </c>
       <c r="I5" t="str">
         <v>2026-07-20</v>
@@ -1768,7 +1803,7 @@
         <v>30367.1</v>
       </c>
       <c r="K5">
-        <v>-1636</v>
+        <v>-2636</v>
       </c>
       <c r="L5" t="str">
         <v>Discrepancy</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-15T20:00:19.133Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:K38"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1653,9 +1653,44 @@
         <v>S20829825</v>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>TXN-1035</v>
+      </c>
+      <c r="B38" t="str">
+        <v>2026-07-16</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Income</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Debt Settlement</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Receipt of loan amount</v>
+      </c>
+      <c r="F38">
+        <v>925</v>
+      </c>
+      <c r="G38" t="str">
+        <v>Federal-Ang</v>
+      </c>
+      <c r="H38" t="str">
+        <v>GPay</v>
+      </c>
+      <c r="I38" t="str">
+        <v>Payment: DEBT-04 (Jomisha)</v>
+      </c>
+      <c r="J38" t="str">
+        <v/>
+      </c>
+      <c r="K38" t="str">
+        <v>S10292193</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K38"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1788,13 +1823,13 @@
         <v>18944</v>
       </c>
       <c r="F5">
-        <v>48383</v>
+        <v>49308</v>
       </c>
       <c r="G5">
         <v>39595.9</v>
       </c>
       <c r="H5">
-        <v>27731.1</v>
+        <v>28656.1</v>
       </c>
       <c r="I5" t="str">
         <v>2026-07-20</v>
@@ -1803,7 +1838,7 @@
         <v>30367.1</v>
       </c>
       <c r="K5">
-        <v>-2636</v>
+        <v>-1711</v>
       </c>
       <c r="L5" t="str">
         <v>Discrepancy</v>
@@ -2007,22 +2042,22 @@
         <v>5758624</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>7.3</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>340</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>40136.64</v>
       </c>
       <c r="I4">
-        <v>5758624</v>
+        <v>13646457.6</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>5758624</v>
+        <v>13646457.6</v>
       </c>
       <c r="L4" t="str">
         <v>2026-08-14</v>
@@ -2043,7 +2078,7 @@
         <v/>
       </c>
       <c r="R4" t="str">
-        <v/>
+        <v>21001</v>
       </c>
     </row>
     <row r="5">
@@ -2075,10 +2110,10 @@
         <v>5000</v>
       </c>
       <c r="J5">
-        <v>0</v>
+        <v>925</v>
       </c>
       <c r="K5">
-        <v>5000</v>
+        <v>4075</v>
       </c>
       <c r="L5" t="str">
         <v>2026-07-13</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-15T20:03:34.021Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K38"/>
+  <dimension ref="A1:K39"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1688,9 +1688,44 @@
         <v>S10292193</v>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>TXN-1036</v>
+      </c>
+      <c r="B39" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Income</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Gifts &amp; Allowance</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Old payment</v>
+      </c>
+      <c r="F39">
+        <v>60000</v>
+      </c>
+      <c r="G39" t="str">
+        <v>Federal-Ang</v>
+      </c>
+      <c r="H39" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="I39" t="str">
+        <v>Import: ACC_STATEMENT_XXXXX5530_23JUN2026_23JUL2026_1784733785805439.pdf (SECURED).pdf</v>
+      </c>
+      <c r="J39" t="str">
+        <v>43002</v>
+      </c>
+      <c r="K39" t="str">
+        <v>S7318245</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K39"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1823,13 +1858,13 @@
         <v>18944</v>
       </c>
       <c r="F5">
-        <v>49308</v>
+        <v>109308</v>
       </c>
       <c r="G5">
         <v>39595.9</v>
       </c>
       <c r="H5">
-        <v>28656.1</v>
+        <v>88656.1</v>
       </c>
       <c r="I5" t="str">
         <v>2026-07-20</v>
@@ -1838,7 +1873,7 @@
         <v>30367.1</v>
       </c>
       <c r="K5">
-        <v>-1711</v>
+        <v>58289</v>
       </c>
       <c r="L5" t="str">
         <v>Discrepancy</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-15T20:50:32.527Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:K38"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -745,31 +745,31 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>TXN-1009</v>
+        <v>TXN-1010</v>
       </c>
       <c r="B12" t="str">
-        <v>2026-07-05</v>
+        <v>2026-07-08</v>
       </c>
       <c r="C12" t="str">
         <v>Expense</v>
       </c>
       <c r="D12" t="str">
-        <v>Utilities</v>
+        <v>Loan Repayment</v>
       </c>
       <c r="E12" t="str">
-        <v>Recharge mobile</v>
+        <v>Land loan repayment</v>
       </c>
       <c r="F12">
-        <v>860.9</v>
+        <v>5891</v>
       </c>
       <c r="G12" t="str">
-        <v>Federal-Ang</v>
+        <v>HDFC- Aluva</v>
       </c>
       <c r="H12" t="str">
-        <v>GPay</v>
+        <v>Bank Transfer</v>
       </c>
       <c r="I12" t="str">
-        <v>Utilities</v>
+        <v>Loan HDFC- Shibin</v>
       </c>
       <c r="J12" t="str">
         <v/>
@@ -780,31 +780,31 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>TXN-1010</v>
+        <v>TXN-1011</v>
       </c>
       <c r="B13" t="str">
-        <v>2026-07-08</v>
+        <v>2026-07-09</v>
       </c>
       <c r="C13" t="str">
-        <v>Expense</v>
+        <v>Income</v>
       </c>
       <c r="D13" t="str">
-        <v>Loan Repayment</v>
+        <v>Dividends / Profit</v>
       </c>
       <c r="E13" t="str">
-        <v>Land loan repayment</v>
+        <v>Dividend - Tata Power</v>
       </c>
       <c r="F13">
-        <v>5891</v>
+        <v>150</v>
       </c>
       <c r="G13" t="str">
-        <v>HDFC- Aluva</v>
+        <v>Federal-Ang</v>
       </c>
       <c r="H13" t="str">
-        <v>Bank Transfer</v>
+        <v>Direct Credit</v>
       </c>
       <c r="I13" t="str">
-        <v>Loan HDFC- Shibin</v>
+        <v>Dividend</v>
       </c>
       <c r="J13" t="str">
         <v/>
@@ -815,31 +815,31 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>TXN-1011</v>
+        <v>TXN-1012</v>
       </c>
       <c r="B14" t="str">
         <v>2026-07-09</v>
       </c>
       <c r="C14" t="str">
-        <v>Income</v>
+        <v>Expense</v>
       </c>
       <c r="D14" t="str">
-        <v>Dividends / Profit</v>
+        <v>Utilities</v>
       </c>
       <c r="E14" t="str">
-        <v>Dividend - Tata Power</v>
+        <v>Recharge airtel</v>
       </c>
       <c r="F14">
-        <v>150</v>
+        <v>199</v>
       </c>
       <c r="G14" t="str">
         <v>Federal-Ang</v>
       </c>
       <c r="H14" t="str">
-        <v>Direct Credit</v>
+        <v>GPay</v>
       </c>
       <c r="I14" t="str">
-        <v>Dividend</v>
+        <v>Utilities</v>
       </c>
       <c r="J14" t="str">
         <v/>
@@ -850,7 +850,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>TXN-1012</v>
+        <v>TXN-1013</v>
       </c>
       <c r="B15" t="str">
         <v>2026-07-09</v>
@@ -859,13 +859,13 @@
         <v>Expense</v>
       </c>
       <c r="D15" t="str">
-        <v>Utilities</v>
+        <v>Family</v>
       </c>
       <c r="E15" t="str">
-        <v>Recharge airtel</v>
+        <v>Weekly expense</v>
       </c>
       <c r="F15">
-        <v>199</v>
+        <v>2500</v>
       </c>
       <c r="G15" t="str">
         <v>Federal-Ang</v>
@@ -874,7 +874,7 @@
         <v>GPay</v>
       </c>
       <c r="I15" t="str">
-        <v>Utilities</v>
+        <v>Family</v>
       </c>
       <c r="J15" t="str">
         <v/>
@@ -885,31 +885,31 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>TXN-1013</v>
+        <v>TXN-1014</v>
       </c>
       <c r="B16" t="str">
-        <v>2026-07-09</v>
+        <v>2026-07-10</v>
       </c>
       <c r="C16" t="str">
-        <v>Expense</v>
+        <v>Income</v>
       </c>
       <c r="D16" t="str">
-        <v>Family</v>
+        <v>Dividends / Profit</v>
       </c>
       <c r="E16" t="str">
-        <v>Weekly expense</v>
+        <v>Dividend - Excide</v>
       </c>
       <c r="F16">
-        <v>2500</v>
+        <v>50</v>
       </c>
       <c r="G16" t="str">
         <v>Federal-Ang</v>
       </c>
       <c r="H16" t="str">
-        <v>GPay</v>
+        <v>Direct Credit</v>
       </c>
       <c r="I16" t="str">
-        <v>Family</v>
+        <v>Dividend</v>
       </c>
       <c r="J16" t="str">
         <v/>
@@ -920,31 +920,31 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>TXN-1014</v>
+        <v>TXN-1015</v>
       </c>
       <c r="B17" t="str">
-        <v>2026-07-10</v>
+        <v>2026-07-17</v>
       </c>
       <c r="C17" t="str">
-        <v>Income</v>
+        <v>Expense</v>
       </c>
       <c r="D17" t="str">
-        <v>Dividends / Profit</v>
+        <v>Utilities</v>
       </c>
       <c r="E17" t="str">
-        <v>Dividend - Excide</v>
+        <v>Amma Recharge</v>
       </c>
       <c r="F17">
-        <v>50</v>
+        <v>211</v>
       </c>
       <c r="G17" t="str">
-        <v>Federal-Ang</v>
+        <v>HDFC- Info</v>
       </c>
       <c r="H17" t="str">
-        <v>Direct Credit</v>
+        <v>GPay</v>
       </c>
       <c r="I17" t="str">
-        <v>Dividend</v>
+        <v>Utilities</v>
       </c>
       <c r="J17" t="str">
         <v/>
@@ -955,22 +955,22 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>TXN-1015</v>
+        <v>TXN-1016</v>
       </c>
       <c r="B18" t="str">
-        <v>2026-07-17</v>
+        <v>2026-07-18</v>
       </c>
       <c r="C18" t="str">
         <v>Expense</v>
       </c>
       <c r="D18" t="str">
-        <v>Utilities</v>
+        <v>GST</v>
       </c>
       <c r="E18" t="str">
-        <v>Amma Recharge</v>
+        <v>Gast filing fee</v>
       </c>
       <c r="F18">
-        <v>211</v>
+        <v>500</v>
       </c>
       <c r="G18" t="str">
         <v>HDFC- Info</v>
@@ -979,7 +979,7 @@
         <v>GPay</v>
       </c>
       <c r="I18" t="str">
-        <v>Utilities</v>
+        <v>GST Filing</v>
       </c>
       <c r="J18" t="str">
         <v/>
@@ -990,22 +990,22 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>TXN-1016</v>
+        <v>TXN-1017</v>
       </c>
       <c r="B19" t="str">
-        <v>2026-07-18</v>
+        <v>2026-07-19</v>
       </c>
       <c r="C19" t="str">
         <v>Expense</v>
       </c>
       <c r="D19" t="str">
-        <v>GST</v>
+        <v>Family</v>
       </c>
       <c r="E19" t="str">
-        <v>Gast filing fee</v>
+        <v>Amma expense</v>
       </c>
       <c r="F19">
-        <v>500</v>
+        <v>2000</v>
       </c>
       <c r="G19" t="str">
         <v>HDFC- Info</v>
@@ -1014,7 +1014,7 @@
         <v>GPay</v>
       </c>
       <c r="I19" t="str">
-        <v>GST Filing</v>
+        <v>Family</v>
       </c>
       <c r="J19" t="str">
         <v/>
@@ -1025,10 +1025,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>TXN-1017</v>
+        <v>TXN-1018</v>
       </c>
       <c r="B20" t="str">
-        <v>2026-07-19</v>
+        <v>2026-07-20</v>
       </c>
       <c r="C20" t="str">
         <v>Expense</v>
@@ -1037,13 +1037,13 @@
         <v>Family</v>
       </c>
       <c r="E20" t="str">
-        <v>Amma expense</v>
+        <v>Hanna Passam</v>
       </c>
       <c r="F20">
-        <v>2000</v>
+        <v>300</v>
       </c>
       <c r="G20" t="str">
-        <v>HDFC- Info</v>
+        <v>Federal-Ang</v>
       </c>
       <c r="H20" t="str">
         <v>GPay</v>
@@ -1060,31 +1060,31 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>TXN-1018</v>
+        <v>TXN-1019</v>
       </c>
       <c r="B21" t="str">
-        <v>2026-07-20</v>
+        <v>2026-07-01</v>
       </c>
       <c r="C21" t="str">
-        <v>Expense</v>
+        <v>Income</v>
       </c>
       <c r="D21" t="str">
-        <v>Family</v>
+        <v>Interest</v>
       </c>
       <c r="E21" t="str">
-        <v>Hanna Passam</v>
+        <v>sb Interest</v>
       </c>
       <c r="F21">
-        <v>300</v>
+        <v>28</v>
       </c>
       <c r="G21" t="str">
-        <v>Federal-Ang</v>
+        <v>HDFC- Aluva</v>
       </c>
       <c r="H21" t="str">
-        <v>GPay</v>
+        <v>Other</v>
       </c>
       <c r="I21" t="str">
-        <v>Family</v>
+        <v/>
       </c>
       <c r="J21" t="str">
         <v/>
@@ -1095,28 +1095,28 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>TXN-1019</v>
+        <v>TXN-1020</v>
       </c>
       <c r="B22" t="str">
         <v>2026-07-01</v>
       </c>
       <c r="C22" t="str">
-        <v>Income</v>
+        <v>Transfer</v>
       </c>
       <c r="D22" t="str">
-        <v>Interest</v>
+        <v>Transfer</v>
       </c>
       <c r="E22" t="str">
-        <v>sb Interest</v>
+        <v>Savings transfer</v>
       </c>
       <c r="F22">
-        <v>28</v>
+        <v>20000</v>
       </c>
       <c r="G22" t="str">
-        <v>HDFC- Aluva</v>
+        <v>HDFC- Info → HDFC- Aluva</v>
       </c>
       <c r="H22" t="str">
-        <v>Other</v>
+        <v/>
       </c>
       <c r="I22" t="str">
         <v/>
@@ -1130,31 +1130,31 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>TXN-1020</v>
+        <v>TXN-1021</v>
       </c>
       <c r="B23" t="str">
-        <v>2026-07-01</v>
+        <v>2026-07-13</v>
       </c>
       <c r="C23" t="str">
-        <v>Transfer</v>
+        <v>Expense</v>
       </c>
       <c r="D23" t="str">
-        <v>Transfer</v>
+        <v>Debt Given</v>
       </c>
       <c r="E23" t="str">
-        <v>Savings transfer</v>
+        <v>Lent to Jomisha</v>
       </c>
       <c r="F23">
-        <v>20000</v>
+        <v>5000</v>
       </c>
       <c r="G23" t="str">
-        <v>HDFC- Info → HDFC- Aluva</v>
+        <v>HDFC- Info</v>
       </c>
       <c r="H23" t="str">
-        <v/>
+        <v>GPay</v>
       </c>
       <c r="I23" t="str">
-        <v/>
+        <v>Linked: DEBT-04 (Jomisha)</v>
       </c>
       <c r="J23" t="str">
         <v/>
@@ -1165,10 +1165,10 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>TXN-1021</v>
+        <v>TXN-1022</v>
       </c>
       <c r="B24" t="str">
-        <v>2026-07-13</v>
+        <v>2026-07-19</v>
       </c>
       <c r="C24" t="str">
         <v>Expense</v>
@@ -1177,10 +1177,10 @@
         <v>Debt Given</v>
       </c>
       <c r="E24" t="str">
-        <v>Lent to Jomisha</v>
+        <v>Lent to Binison</v>
       </c>
       <c r="F24">
-        <v>5000</v>
+        <v>1500</v>
       </c>
       <c r="G24" t="str">
         <v>HDFC- Info</v>
@@ -1189,7 +1189,7 @@
         <v>GPay</v>
       </c>
       <c r="I24" t="str">
-        <v>Linked: DEBT-04 (Jomisha)</v>
+        <v>Linked: DEBT-05 (Binison)</v>
       </c>
       <c r="J24" t="str">
         <v/>
@@ -1200,31 +1200,31 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>TXN-1022</v>
+        <v>TXN-1023</v>
       </c>
       <c r="B25" t="str">
-        <v>2026-07-19</v>
+        <v>2026-07-05</v>
       </c>
       <c r="C25" t="str">
-        <v>Expense</v>
+        <v>Transfer</v>
       </c>
       <c r="D25" t="str">
-        <v>Debt Given</v>
+        <v>Transfer</v>
       </c>
       <c r="E25" t="str">
-        <v>Lent to Binison</v>
+        <v>EMI Savings</v>
       </c>
       <c r="F25">
-        <v>1500</v>
+        <v>50000</v>
       </c>
       <c r="G25" t="str">
-        <v>HDFC- Info</v>
+        <v>HDFC- Info → SBI</v>
       </c>
       <c r="H25" t="str">
-        <v>GPay</v>
+        <v/>
       </c>
       <c r="I25" t="str">
-        <v>Linked: DEBT-05 (Binison)</v>
+        <v/>
       </c>
       <c r="J25" t="str">
         <v/>
@@ -1235,28 +1235,28 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>TXN-1023</v>
+        <v>TXN-1024</v>
       </c>
       <c r="B26" t="str">
-        <v>2026-07-05</v>
+        <v>2026-07-01</v>
       </c>
       <c r="C26" t="str">
-        <v>Transfer</v>
+        <v>Income</v>
       </c>
       <c r="D26" t="str">
-        <v>Transfer</v>
+        <v>Debt Settlement</v>
       </c>
       <c r="E26" t="str">
-        <v>EMI Savings</v>
+        <v>Shilpa</v>
       </c>
       <c r="F26">
-        <v>50000</v>
+        <v>15000</v>
       </c>
       <c r="G26" t="str">
-        <v>HDFC- Info → SBI</v>
+        <v>Federal-Ang</v>
       </c>
       <c r="H26" t="str">
-        <v/>
+        <v>GPay</v>
       </c>
       <c r="I26" t="str">
         <v/>
@@ -1270,31 +1270,31 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>TXN-1024</v>
+        <v>TXN-1025</v>
       </c>
       <c r="B27" t="str">
         <v>2026-07-01</v>
       </c>
       <c r="C27" t="str">
-        <v>Income</v>
+        <v>Expense</v>
       </c>
       <c r="D27" t="str">
-        <v>Debt Settlement</v>
+        <v>Investment</v>
       </c>
       <c r="E27" t="str">
-        <v>Shilpa</v>
+        <v>Invested in APY Pension</v>
       </c>
       <c r="F27">
-        <v>15000</v>
+        <v>409</v>
       </c>
       <c r="G27" t="str">
         <v>Federal-Ang</v>
       </c>
       <c r="H27" t="str">
-        <v>GPay</v>
+        <v/>
       </c>
       <c r="I27" t="str">
-        <v/>
+        <v>Linked: INV-04</v>
       </c>
       <c r="J27" t="str">
         <v/>
@@ -1305,7 +1305,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>TXN-1025</v>
+        <v>TXN-1026</v>
       </c>
       <c r="B28" t="str">
         <v>2026-07-01</v>
@@ -1317,10 +1317,10 @@
         <v>Investment</v>
       </c>
       <c r="E28" t="str">
-        <v>Invested in APY Pension</v>
+        <v>Invested in Coin by Zerodha</v>
       </c>
       <c r="F28">
-        <v>409</v>
+        <v>1331</v>
       </c>
       <c r="G28" t="str">
         <v>Federal-Ang</v>
@@ -1329,7 +1329,7 @@
         <v/>
       </c>
       <c r="I28" t="str">
-        <v>Linked: INV-04</v>
+        <v>Linked: INV-05</v>
       </c>
       <c r="J28" t="str">
         <v/>
@@ -1340,7 +1340,7 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>TXN-1026</v>
+        <v>TXN-1027</v>
       </c>
       <c r="B29" t="str">
         <v>2026-07-01</v>
@@ -1355,7 +1355,7 @@
         <v>Invested in Coin by Zerodha</v>
       </c>
       <c r="F29">
-        <v>1331</v>
+        <v>1996</v>
       </c>
       <c r="G29" t="str">
         <v>Federal-Ang</v>
@@ -1364,7 +1364,7 @@
         <v/>
       </c>
       <c r="I29" t="str">
-        <v>Linked: INV-05</v>
+        <v>Linked: INV-06</v>
       </c>
       <c r="J29" t="str">
         <v/>
@@ -1375,31 +1375,31 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>TXN-1027</v>
+        <v>TXN-1028</v>
       </c>
       <c r="B30" t="str">
-        <v>2026-07-01</v>
+        <v>2026-07-09</v>
       </c>
       <c r="C30" t="str">
-        <v>Expense</v>
+        <v>Income</v>
       </c>
       <c r="D30" t="str">
-        <v>Investment</v>
+        <v>Dividends / Profit</v>
       </c>
       <c r="E30" t="str">
-        <v>Invested in Coin by Zerodha</v>
+        <v>TMPVL</v>
       </c>
       <c r="F30">
-        <v>1996</v>
+        <v>78</v>
       </c>
       <c r="G30" t="str">
         <v>Federal-Ang</v>
       </c>
       <c r="H30" t="str">
-        <v/>
+        <v>Bank Transfer</v>
       </c>
       <c r="I30" t="str">
-        <v>Linked: INV-06</v>
+        <v/>
       </c>
       <c r="J30" t="str">
         <v/>
@@ -1410,31 +1410,31 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>TXN-1028</v>
+        <v>TXN-1029</v>
       </c>
       <c r="B31" t="str">
-        <v>2026-07-09</v>
+        <v>2026-07-01</v>
       </c>
       <c r="C31" t="str">
-        <v>Income</v>
+        <v>Expense</v>
       </c>
       <c r="D31" t="str">
-        <v>Dividends / Profit</v>
+        <v>Debt Given</v>
       </c>
       <c r="E31" t="str">
-        <v>TMPVL</v>
+        <v>Lent to Baby</v>
       </c>
       <c r="F31">
-        <v>78</v>
+        <v>25000</v>
       </c>
       <c r="G31" t="str">
         <v>Federal-Ang</v>
       </c>
       <c r="H31" t="str">
-        <v>Bank Transfer</v>
+        <v/>
       </c>
       <c r="I31" t="str">
-        <v/>
+        <v>Linked: DEBT-06 (Baby)</v>
       </c>
       <c r="J31" t="str">
         <v/>
@@ -1445,31 +1445,31 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>TXN-1029</v>
+        <v>TXN-1030</v>
       </c>
       <c r="B32" t="str">
-        <v>2026-07-01</v>
+        <v>2026-07-20</v>
       </c>
       <c r="C32" t="str">
-        <v>Expense</v>
+        <v>Income</v>
       </c>
       <c r="D32" t="str">
-        <v>Debt Given</v>
+        <v>For CC Payment</v>
       </c>
       <c r="E32" t="str">
-        <v>Lent to Baby</v>
+        <v>Shibin Washing machine - Icici Amazon Pay</v>
       </c>
       <c r="F32">
-        <v>25000</v>
+        <v>33105</v>
       </c>
       <c r="G32" t="str">
         <v>Federal-Ang</v>
       </c>
       <c r="H32" t="str">
-        <v/>
+        <v>Bank Transfer</v>
       </c>
       <c r="I32" t="str">
-        <v>Linked: DEBT-06 (Baby)</v>
+        <v/>
       </c>
       <c r="J32" t="str">
         <v/>
@@ -1480,31 +1480,31 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>TXN-1030</v>
+        <v>TXN-1031</v>
       </c>
       <c r="B33" t="str">
-        <v>2026-07-20</v>
+        <v>2026-07-22</v>
       </c>
       <c r="C33" t="str">
-        <v>Income</v>
+        <v>Expense</v>
       </c>
       <c r="D33" t="str">
-        <v>For CC Payment</v>
+        <v>Debt Given</v>
       </c>
       <c r="E33" t="str">
-        <v>Shibin Washing machine - Icici Amazon Pay</v>
+        <v>Lent to Albert</v>
       </c>
       <c r="F33">
-        <v>33105</v>
+        <v>78700</v>
       </c>
       <c r="G33" t="str">
-        <v>Federal-Ang</v>
+        <v>SBI</v>
       </c>
       <c r="H33" t="str">
-        <v>Bank Transfer</v>
+        <v>GPay</v>
       </c>
       <c r="I33" t="str">
-        <v/>
+        <v>Linked: DEBT-07 (Albert)</v>
       </c>
       <c r="J33" t="str">
         <v/>
@@ -1515,7 +1515,7 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>TXN-1031</v>
+        <v>TXN-1032</v>
       </c>
       <c r="B34" t="str">
         <v>2026-07-22</v>
@@ -1524,22 +1524,22 @@
         <v>Expense</v>
       </c>
       <c r="D34" t="str">
-        <v>Debt Given</v>
+        <v>Groceries</v>
       </c>
       <c r="E34" t="str">
-        <v>Lent to Albert</v>
+        <v>Guest visit mary jincy</v>
       </c>
       <c r="F34">
-        <v>78700</v>
+        <v>3000</v>
       </c>
       <c r="G34" t="str">
-        <v>SBI</v>
+        <v>Federal-Ang</v>
       </c>
       <c r="H34" t="str">
         <v>GPay</v>
       </c>
       <c r="I34" t="str">
-        <v>Linked: DEBT-07 (Albert)</v>
+        <v/>
       </c>
       <c r="J34" t="str">
         <v/>
@@ -1550,19 +1550,19 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>TXN-1032</v>
+        <v>TXN-1033</v>
       </c>
       <c r="B35" t="str">
-        <v>2026-07-22</v>
+        <v>2026-07-30</v>
       </c>
       <c r="C35" t="str">
         <v>Expense</v>
       </c>
       <c r="D35" t="str">
-        <v>Groceries</v>
+        <v>Family</v>
       </c>
       <c r="E35" t="str">
-        <v>Guest visit mary jincy</v>
+        <v>Amma</v>
       </c>
       <c r="F35">
         <v>3000</v>
@@ -1585,147 +1585,112 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>TXN-1033</v>
+        <v>TXN-1034</v>
       </c>
       <c r="B36" t="str">
-        <v>2026-07-30</v>
+        <v>2026-07-08</v>
       </c>
       <c r="C36" t="str">
         <v>Expense</v>
       </c>
       <c r="D36" t="str">
-        <v>Family</v>
+        <v>Family Support</v>
       </c>
       <c r="E36" t="str">
-        <v>Amma</v>
+        <v>Payment to amma</v>
       </c>
       <c r="F36">
-        <v>3000</v>
+        <v>1000</v>
       </c>
       <c r="G36" t="str">
         <v>Federal-Ang</v>
       </c>
       <c r="H36" t="str">
-        <v>GPay</v>
+        <v>Direct Credit</v>
       </c>
       <c r="I36" t="str">
-        <v/>
+        <v>Import: ACC_STATEMENT_XXXXX5530_23JUN2026_23JUL2026_1784733785805439.pdf (SECURED).pdf</v>
       </c>
       <c r="J36" t="str">
-        <v/>
+        <v>54001</v>
       </c>
       <c r="K36" t="str">
-        <v/>
+        <v>S20829825</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>TXN-1034</v>
+        <v>TXN-1035</v>
       </c>
       <c r="B37" t="str">
-        <v>2026-07-08</v>
+        <v>2026-07-16</v>
       </c>
       <c r="C37" t="str">
-        <v>Expense</v>
+        <v>Income</v>
       </c>
       <c r="D37" t="str">
-        <v>Family Support</v>
+        <v>Debt Settlement</v>
       </c>
       <c r="E37" t="str">
-        <v>Payment to amma</v>
+        <v>Receipt of loan amount</v>
       </c>
       <c r="F37">
-        <v>1000</v>
+        <v>925</v>
       </c>
       <c r="G37" t="str">
         <v>Federal-Ang</v>
       </c>
       <c r="H37" t="str">
-        <v>Direct Credit</v>
+        <v>GPay</v>
       </c>
       <c r="I37" t="str">
-        <v>Import: ACC_STATEMENT_XXXXX5530_23JUN2026_23JUL2026_1784733785805439.pdf (SECURED).pdf</v>
+        <v>Payment: DEBT-04 (Jomisha)</v>
       </c>
       <c r="J37" t="str">
-        <v>54001</v>
+        <v/>
       </c>
       <c r="K37" t="str">
-        <v>S20829825</v>
+        <v>S10292193</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>TXN-1035</v>
+        <v>TXN-1036</v>
       </c>
       <c r="B38" t="str">
-        <v>2026-07-16</v>
+        <v>2026-06-26</v>
       </c>
       <c r="C38" t="str">
         <v>Income</v>
       </c>
       <c r="D38" t="str">
-        <v>Debt Settlement</v>
+        <v>Gifts &amp; Allowance</v>
       </c>
       <c r="E38" t="str">
-        <v>Receipt of loan amount</v>
+        <v>Old payment</v>
       </c>
       <c r="F38">
-        <v>925</v>
+        <v>60000</v>
       </c>
       <c r="G38" t="str">
         <v>Federal-Ang</v>
       </c>
       <c r="H38" t="str">
-        <v>GPay</v>
+        <v>Direct Credit</v>
       </c>
       <c r="I38" t="str">
-        <v>Payment: DEBT-04 (Jomisha)</v>
+        <v>Import: ACC_STATEMENT_XXXXX5530_23JUN2026_23JUL2026_1784733785805439.pdf (SECURED).pdf</v>
       </c>
       <c r="J38" t="str">
-        <v/>
+        <v>43002</v>
       </c>
       <c r="K38" t="str">
-        <v>S10292193</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="str">
-        <v>TXN-1036</v>
-      </c>
-      <c r="B39" t="str">
-        <v>2026-06-26</v>
-      </c>
-      <c r="C39" t="str">
-        <v>Income</v>
-      </c>
-      <c r="D39" t="str">
-        <v>Gifts &amp; Allowance</v>
-      </c>
-      <c r="E39" t="str">
-        <v>Old payment</v>
-      </c>
-      <c r="F39">
-        <v>60000</v>
-      </c>
-      <c r="G39" t="str">
-        <v>Federal-Ang</v>
-      </c>
-      <c r="H39" t="str">
-        <v>Direct Credit</v>
-      </c>
-      <c r="I39" t="str">
-        <v>Import: ACC_STATEMENT_XXXXX5530_23JUN2026_23JUL2026_1784733785805439.pdf (SECURED).pdf</v>
-      </c>
-      <c r="J39" t="str">
-        <v>43002</v>
-      </c>
-      <c r="K39" t="str">
         <v>S7318245</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K39"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K38"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1861,10 +1826,10 @@
         <v>109308</v>
       </c>
       <c r="G5">
-        <v>39595.9</v>
+        <v>38735</v>
       </c>
       <c r="H5">
-        <v>88656.1</v>
+        <v>89517</v>
       </c>
       <c r="I5" t="str">
         <v>2026-07-20</v>
@@ -1873,7 +1838,7 @@
         <v>30367.1</v>
       </c>
       <c r="K5">
-        <v>58289</v>
+        <v>59149.9</v>
       </c>
       <c r="L5" t="str">
         <v>Discrepancy</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-15T21:54:08.405Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -726,7 +726,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F46"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -848,30 +848,30 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>12001</v>
+        <v>11201</v>
       </c>
       <c r="B8" t="str">
-        <v>APY Pension</v>
+        <v>Cash</v>
       </c>
       <c r="C8" t="str">
         <v>Asset</v>
       </c>
       <c r="D8" t="str">
-        <v>Investments</v>
+        <v>Cash &amp; Bank</v>
       </c>
       <c r="E8" t="str">
-        <v>Pension</v>
+        <v>Cash</v>
       </c>
       <c r="F8" t="str">
-        <v>apy</v>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>12002</v>
+        <v>12001</v>
       </c>
       <c r="B9" t="str">
-        <v>Zerodha Coin</v>
+        <v>APY Pension</v>
       </c>
       <c r="C9" t="str">
         <v>Asset</v>
@@ -880,18 +880,18 @@
         <v>Investments</v>
       </c>
       <c r="E9" t="str">
-        <v>Mutual Funds / Stocks</v>
+        <v>Pension</v>
       </c>
       <c r="F9" t="str">
-        <v>zerodha,coin</v>
+        <v>apy</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>12099</v>
+        <v>12002</v>
       </c>
       <c r="B10" t="str">
-        <v>Other Investments</v>
+        <v>Zerodha Coin</v>
       </c>
       <c r="C10" t="str">
         <v>Asset</v>
@@ -900,158 +900,158 @@
         <v>Investments</v>
       </c>
       <c r="E10" t="str">
-        <v>General</v>
+        <v>Mutual Funds / Stocks</v>
       </c>
       <c r="F10" t="str">
-        <v>nps,ppf,fd,deposit</v>
+        <v>zerodha,coin</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>13001</v>
+        <v>12099</v>
       </c>
       <c r="B11" t="str">
-        <v>Loans Given (Receivables)</v>
+        <v>Other Investments</v>
       </c>
       <c r="C11" t="str">
         <v>Asset</v>
       </c>
       <c r="D11" t="str">
-        <v>Receivables</v>
+        <v>Investments</v>
       </c>
       <c r="E11" t="str">
-        <v>Personal Loans Given</v>
+        <v>General</v>
       </c>
       <c r="F11" t="str">
-        <v>lent,jomisha,binison,albert</v>
+        <v>nps,ppf,fd,deposit</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>21001</v>
+        <v>13001</v>
       </c>
       <c r="B12" t="str">
-        <v>SBI Home Loan</v>
+        <v>Loans Given (Receivables)</v>
       </c>
       <c r="C12" t="str">
-        <v>Liability</v>
+        <v>Asset</v>
       </c>
       <c r="D12" t="str">
-        <v>Bank Loans</v>
+        <v>Receivables</v>
       </c>
       <c r="E12" t="str">
-        <v>Housing Loan</v>
+        <v>Personal Loans Given</v>
       </c>
       <c r="F12" t="str">
-        <v>home loan,housing loan</v>
+        <v>lent,jomisha,binison,albert</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>22001</v>
+        <v>21001</v>
       </c>
       <c r="B13" t="str">
-        <v>Personal Borrowings</v>
+        <v>SBI Home Loan</v>
       </c>
       <c r="C13" t="str">
         <v>Liability</v>
       </c>
       <c r="D13" t="str">
-        <v>Debts Payable</v>
+        <v>Bank Loans</v>
       </c>
       <c r="E13" t="str">
-        <v>From People</v>
+        <v>Housing Loan</v>
       </c>
       <c r="F13" t="str">
-        <v>borrowed</v>
+        <v>home loan,housing loan</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>23001</v>
+        <v>22001</v>
       </c>
       <c r="B14" t="str">
-        <v>Credit Card Payable</v>
+        <v>Personal Borrowings</v>
       </c>
       <c r="C14" t="str">
         <v>Liability</v>
       </c>
       <c r="D14" t="str">
-        <v>Credit Cards</v>
+        <v>Debts Payable</v>
       </c>
       <c r="E14" t="str">
-        <v>ICICI Amazon Pay</v>
+        <v>From People</v>
       </c>
       <c r="F14" t="str">
-        <v>icici amazon</v>
+        <v>borrowed</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>30001</v>
+        <v>23001</v>
       </c>
       <c r="B15" t="str">
-        <v>Opening Balances / Net Worth</v>
+        <v>Credit Card Payable</v>
       </c>
       <c r="C15" t="str">
-        <v>Equity</v>
+        <v>Liability</v>
       </c>
       <c r="D15" t="str">
-        <v>Capital</v>
+        <v>Credit Cards</v>
       </c>
       <c r="E15" t="str">
-        <v>Opening Balance</v>
+        <v>ICICI Amazon Pay</v>
       </c>
       <c r="F15" t="str">
-        <v/>
+        <v>icici amazon</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>41001</v>
+        <v>30001</v>
       </c>
       <c r="B16" t="str">
-        <v>Salary</v>
+        <v>Opening Balances / Net Worth</v>
       </c>
       <c r="C16" t="str">
-        <v>Income</v>
+        <v>Equity</v>
       </c>
       <c r="D16" t="str">
-        <v>Employment</v>
+        <v>Capital</v>
       </c>
       <c r="E16" t="str">
-        <v>Monthly Salary</v>
+        <v>Opening Balance</v>
       </c>
       <c r="F16" t="str">
-        <v>salary,sal cr,infopark</v>
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>41002</v>
+        <v>41001</v>
       </c>
       <c r="B17" t="str">
-        <v>Business Income</v>
+        <v>Salary</v>
       </c>
       <c r="C17" t="str">
         <v>Income</v>
       </c>
       <c r="D17" t="str">
-        <v>Business</v>
+        <v>Employment</v>
       </c>
       <c r="E17" t="str">
-        <v>General</v>
+        <v>Monthly Salary</v>
       </c>
       <c r="F17" t="str">
-        <v>business</v>
+        <v>salary,sal cr,infopark</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>41003</v>
+        <v>41002</v>
       </c>
       <c r="B18" t="str">
-        <v>Freelance Income</v>
+        <v>Business Income</v>
       </c>
       <c r="C18" t="str">
         <v>Income</v>
@@ -1060,38 +1060,38 @@
         <v>Business</v>
       </c>
       <c r="E18" t="str">
-        <v>Freelance</v>
+        <v>General</v>
       </c>
       <c r="F18" t="str">
-        <v>freelance</v>
+        <v>business</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>42001</v>
+        <v>41003</v>
       </c>
       <c r="B19" t="str">
-        <v>Interest Income</v>
+        <v>Freelance Income</v>
       </c>
       <c r="C19" t="str">
         <v>Income</v>
       </c>
       <c r="D19" t="str">
-        <v>Investment Income</v>
+        <v>Business</v>
       </c>
       <c r="E19" t="str">
-        <v>Bank / FD Interest</v>
+        <v>Freelance</v>
       </c>
       <c r="F19" t="str">
-        <v>interest,int.pd,sbint,sb int</v>
+        <v>freelance</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>42002</v>
+        <v>42001</v>
       </c>
       <c r="B20" t="str">
-        <v>Dividend Income</v>
+        <v>Interest Income</v>
       </c>
       <c r="C20" t="str">
         <v>Income</v>
@@ -1100,38 +1100,38 @@
         <v>Investment Income</v>
       </c>
       <c r="E20" t="str">
-        <v>Dividends</v>
+        <v>Bank / FD Interest</v>
       </c>
       <c r="F20" t="str">
-        <v>dividend,div,achcr</v>
+        <v>interest,int.pd,sbint,sb int</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>43001</v>
+        <v>42002</v>
       </c>
       <c r="B21" t="str">
-        <v>Rental Income</v>
+        <v>Dividend Income</v>
       </c>
       <c r="C21" t="str">
         <v>Income</v>
       </c>
       <c r="D21" t="str">
-        <v>Other Income</v>
+        <v>Investment Income</v>
       </c>
       <c r="E21" t="str">
-        <v>Rent Received</v>
+        <v>Dividends</v>
       </c>
       <c r="F21" t="str">
-        <v>rent received</v>
+        <v>dividend,div,achcr</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>43002</v>
+        <v>43001</v>
       </c>
       <c r="B22" t="str">
-        <v>Gifts &amp; Allowance</v>
+        <v>Rental Income</v>
       </c>
       <c r="C22" t="str">
         <v>Income</v>
@@ -1140,18 +1140,18 @@
         <v>Other Income</v>
       </c>
       <c r="E22" t="str">
-        <v>Gifts</v>
+        <v>Rent Received</v>
       </c>
       <c r="F22" t="str">
-        <v>gift received</v>
+        <v>rent received</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>43003</v>
+        <v>43002</v>
       </c>
       <c r="B23" t="str">
-        <v>Debt Settlement Received</v>
+        <v>Gifts &amp; Allowance</v>
       </c>
       <c r="C23" t="str">
         <v>Income</v>
@@ -1160,18 +1160,18 @@
         <v>Other Income</v>
       </c>
       <c r="E23" t="str">
-        <v>Loan Repaid to You</v>
+        <v>Gifts</v>
       </c>
       <c r="F23" t="str">
-        <v>repayment</v>
+        <v>gift received</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>49999</v>
+        <v>43003</v>
       </c>
       <c r="B24" t="str">
-        <v>Other Income</v>
+        <v>Debt Settlement Received</v>
       </c>
       <c r="C24" t="str">
         <v>Income</v>
@@ -1180,38 +1180,38 @@
         <v>Other Income</v>
       </c>
       <c r="E24" t="str">
-        <v>Miscellaneous</v>
+        <v>Loan Repaid to You</v>
       </c>
       <c r="F24" t="str">
-        <v/>
+        <v>repayment</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>51001</v>
+        <v>49999</v>
       </c>
       <c r="B25" t="str">
-        <v>Rent / Housing</v>
+        <v>Other Income</v>
       </c>
       <c r="C25" t="str">
-        <v>Expense</v>
+        <v>Income</v>
       </c>
       <c r="D25" t="str">
-        <v>Household</v>
+        <v>Other Income</v>
       </c>
       <c r="E25" t="str">
-        <v>Rent &amp; Maintenance</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="F25" t="str">
-        <v>rent,maintenance</v>
+        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>51002</v>
+        <v>51001</v>
       </c>
       <c r="B26" t="str">
-        <v>Utilities - Electricity &amp; Water</v>
+        <v>Rent / Housing</v>
       </c>
       <c r="C26" t="str">
         <v>Expense</v>
@@ -1220,18 +1220,18 @@
         <v>Household</v>
       </c>
       <c r="E26" t="str">
-        <v>Electricity / Water</v>
+        <v>Rent &amp; Maintenance</v>
       </c>
       <c r="F26" t="str">
-        <v>kseb,electricity,water bill</v>
+        <v>rent,maintenance</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>51003</v>
+        <v>51002</v>
       </c>
       <c r="B27" t="str">
-        <v>Utilities - Internet &amp; Mobile</v>
+        <v>Utilities - Electricity &amp; Water</v>
       </c>
       <c r="C27" t="str">
         <v>Expense</v>
@@ -1240,18 +1240,18 @@
         <v>Household</v>
       </c>
       <c r="E27" t="str">
-        <v>Recharge / Broadband</v>
+        <v>Electricity / Water</v>
       </c>
       <c r="F27" t="str">
-        <v>recharge,airtel,jio,bsnl,broadband,wifi</v>
+        <v>kseb,electricity,water bill</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>51004</v>
+        <v>51003</v>
       </c>
       <c r="B28" t="str">
-        <v>Gas / LPG</v>
+        <v>Utilities - Internet &amp; Mobile</v>
       </c>
       <c r="C28" t="str">
         <v>Expense</v>
@@ -1260,18 +1260,18 @@
         <v>Household</v>
       </c>
       <c r="E28" t="str">
-        <v>Cooking Gas</v>
+        <v>Recharge / Broadband</v>
       </c>
       <c r="F28" t="str">
-        <v>lpg,indane,gas</v>
+        <v>recharge,airtel,jio,bsnl,broadband,wifi</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>51005</v>
+        <v>51004</v>
       </c>
       <c r="B29" t="str">
-        <v>Household Appliances</v>
+        <v>Gas / LPG</v>
       </c>
       <c r="C29" t="str">
         <v>Expense</v>
@@ -1280,38 +1280,38 @@
         <v>Household</v>
       </c>
       <c r="E29" t="str">
-        <v>Appliances &amp; Repairs</v>
+        <v>Cooking Gas</v>
       </c>
       <c r="F29" t="str">
-        <v>washing machine,appliance,repair</v>
+        <v>lpg,indane,gas</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>52001</v>
+        <v>51005</v>
       </c>
       <c r="B30" t="str">
-        <v>Groceries</v>
+        <v>Household Appliances</v>
       </c>
       <c r="C30" t="str">
         <v>Expense</v>
       </c>
       <c r="D30" t="str">
-        <v>Food</v>
+        <v>Household</v>
       </c>
       <c r="E30" t="str">
-        <v>Provisions</v>
+        <v>Appliances &amp; Repairs</v>
       </c>
       <c r="F30" t="str">
-        <v>grocery,supermarket,mart,bigbasket,blinkit,zepto,dmart</v>
+        <v>washing machine,appliance,repair</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>52002</v>
+        <v>52001</v>
       </c>
       <c r="B31" t="str">
-        <v>Dining Out</v>
+        <v>Groceries</v>
       </c>
       <c r="C31" t="str">
         <v>Expense</v>
@@ -1320,38 +1320,38 @@
         <v>Food</v>
       </c>
       <c r="E31" t="str">
-        <v>Restaurants &amp; Delivery</v>
+        <v>Provisions</v>
       </c>
       <c r="F31" t="str">
-        <v>swiggy,zomato,restaurant,hotel,cafe</v>
+        <v>grocery,supermarket,mart,bigbasket,blinkit,zepto,dmart</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>53001</v>
+        <v>52002</v>
       </c>
       <c r="B32" t="str">
-        <v>Transport &amp; Fuel</v>
+        <v>Dining Out</v>
       </c>
       <c r="C32" t="str">
         <v>Expense</v>
       </c>
       <c r="D32" t="str">
-        <v>Transport</v>
+        <v>Food</v>
       </c>
       <c r="E32" t="str">
-        <v>Fuel / Taxi / Toll</v>
+        <v>Restaurants &amp; Delivery</v>
       </c>
       <c r="F32" t="str">
-        <v>uber,ola,rapido,petrol,fuel,hpcl,bpcl,fastag</v>
+        <v>swiggy,zomato,restaurant,hotel,cafe</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>53002</v>
+        <v>53001</v>
       </c>
       <c r="B33" t="str">
-        <v>Travel</v>
+        <v>Transport &amp; Fuel</v>
       </c>
       <c r="C33" t="str">
         <v>Expense</v>
@@ -1360,38 +1360,38 @@
         <v>Transport</v>
       </c>
       <c r="E33" t="str">
-        <v>Trips &amp; Tickets</v>
+        <v>Fuel / Taxi / Toll</v>
       </c>
       <c r="F33" t="str">
-        <v>irctc,makemytrip,redbus,indigo</v>
+        <v>uber,ola,rapido,petrol,fuel,hpcl,bpcl,fastag</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>54001</v>
+        <v>53002</v>
       </c>
       <c r="B34" t="str">
-        <v>Family Support</v>
+        <v>Travel</v>
       </c>
       <c r="C34" t="str">
         <v>Expense</v>
       </c>
       <c r="D34" t="str">
-        <v>Family &amp; Personal</v>
+        <v>Transport</v>
       </c>
       <c r="E34" t="str">
-        <v>Family / Amma</v>
+        <v>Trips &amp; Tickets</v>
       </c>
       <c r="F34" t="str">
-        <v>amma,family</v>
+        <v>irctc,makemytrip,redbus,indigo</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>54002</v>
+        <v>54001</v>
       </c>
       <c r="B35" t="str">
-        <v>Health &amp; Medical</v>
+        <v>Family Support</v>
       </c>
       <c r="C35" t="str">
         <v>Expense</v>
@@ -1400,18 +1400,18 @@
         <v>Family &amp; Personal</v>
       </c>
       <c r="E35" t="str">
-        <v>Pharmacy / Hospital</v>
+        <v>Family / Amma</v>
       </c>
       <c r="F35" t="str">
-        <v>pharmacy,medical,hospital,clinic</v>
+        <v>amma,family</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>54003</v>
+        <v>54002</v>
       </c>
       <c r="B36" t="str">
-        <v>Education</v>
+        <v>Health &amp; Medical</v>
       </c>
       <c r="C36" t="str">
         <v>Expense</v>
@@ -1420,18 +1420,18 @@
         <v>Family &amp; Personal</v>
       </c>
       <c r="E36" t="str">
-        <v>Fees &amp; Courses</v>
+        <v>Pharmacy / Hospital</v>
       </c>
       <c r="F36" t="str">
-        <v>school,college,course,tuition</v>
+        <v>pharmacy,medical,hospital,clinic</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>54004</v>
+        <v>54003</v>
       </c>
       <c r="B37" t="str">
-        <v>Shopping</v>
+        <v>Education</v>
       </c>
       <c r="C37" t="str">
         <v>Expense</v>
@@ -1440,18 +1440,18 @@
         <v>Family &amp; Personal</v>
       </c>
       <c r="E37" t="str">
-        <v>Online &amp; Retail</v>
+        <v>Fees &amp; Courses</v>
       </c>
       <c r="F37" t="str">
-        <v>amazon,flipkart,myntra,ajio</v>
+        <v>school,college,course,tuition</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>54005</v>
+        <v>54004</v>
       </c>
       <c r="B38" t="str">
-        <v>Gifts &amp; Functions</v>
+        <v>Shopping</v>
       </c>
       <c r="C38" t="str">
         <v>Expense</v>
@@ -1460,38 +1460,38 @@
         <v>Family &amp; Personal</v>
       </c>
       <c r="E38" t="str">
-        <v>Guests &amp; Gifts</v>
+        <v>Online &amp; Retail</v>
       </c>
       <c r="F38" t="str">
-        <v>guest,marriage,function</v>
+        <v>amazon,flipkart,myntra,ajio</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>55001</v>
+        <v>54005</v>
       </c>
       <c r="B39" t="str">
-        <v>Loan EMI / Repayment</v>
+        <v>Gifts &amp; Functions</v>
       </c>
       <c r="C39" t="str">
         <v>Expense</v>
       </c>
       <c r="D39" t="str">
-        <v>Financial</v>
+        <v>Family &amp; Personal</v>
       </c>
       <c r="E39" t="str">
-        <v>EMIs</v>
+        <v>Guests &amp; Gifts</v>
       </c>
       <c r="F39" t="str">
-        <v>emi,loan repay</v>
+        <v>guest,marriage,function</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>55002</v>
+        <v>55001</v>
       </c>
       <c r="B40" t="str">
-        <v>Credit Card Payment</v>
+        <v>Loan EMI / Repayment</v>
       </c>
       <c r="C40" t="str">
         <v>Expense</v>
@@ -1500,18 +1500,18 @@
         <v>Financial</v>
       </c>
       <c r="E40" t="str">
-        <v>Card Bills</v>
+        <v>EMIs</v>
       </c>
       <c r="F40" t="str">
-        <v>cc payment,card payment</v>
+        <v>emi,loan repay</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>55003</v>
+        <v>55002</v>
       </c>
       <c r="B41" t="str">
-        <v>Investment Contribution</v>
+        <v>Credit Card Payment</v>
       </c>
       <c r="C41" t="str">
         <v>Expense</v>
@@ -1520,18 +1520,18 @@
         <v>Financial</v>
       </c>
       <c r="E41" t="str">
-        <v>SIP / Deposits</v>
+        <v>Card Bills</v>
       </c>
       <c r="F41" t="str">
-        <v>sip</v>
+        <v>cc payment,card payment</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>55004</v>
+        <v>55003</v>
       </c>
       <c r="B42" t="str">
-        <v>Debt Given (Lent Out)</v>
+        <v>Investment Contribution</v>
       </c>
       <c r="C42" t="str">
         <v>Expense</v>
@@ -1540,18 +1540,18 @@
         <v>Financial</v>
       </c>
       <c r="E42" t="str">
-        <v>Money Lent</v>
+        <v>SIP / Deposits</v>
       </c>
       <c r="F42" t="str">
-        <v>lent to</v>
+        <v>sip</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>55005</v>
+        <v>55004</v>
       </c>
       <c r="B43" t="str">
-        <v>Taxes &amp; GST</v>
+        <v>Debt Given (Lent Out)</v>
       </c>
       <c r="C43" t="str">
         <v>Expense</v>
@@ -1560,18 +1560,18 @@
         <v>Financial</v>
       </c>
       <c r="E43" t="str">
-        <v>GST / Filing</v>
+        <v>Money Lent</v>
       </c>
       <c r="F43" t="str">
-        <v>gst,filing fee,tax</v>
+        <v>lent to</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>55006</v>
+        <v>55005</v>
       </c>
       <c r="B44" t="str">
-        <v>Insurance</v>
+        <v>Taxes &amp; GST</v>
       </c>
       <c r="C44" t="str">
         <v>Expense</v>
@@ -1580,35 +1580,55 @@
         <v>Financial</v>
       </c>
       <c r="E44" t="str">
-        <v>Premiums</v>
+        <v>GST / Filing</v>
       </c>
       <c r="F44" t="str">
-        <v>insurance,lic,premium</v>
+        <v>gst,filing fee,tax</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
+        <v>55006</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Insurance</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Financial</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Premiums</v>
+      </c>
+      <c r="F45" t="str">
+        <v>insurance,lic,premium</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
         <v>59999</v>
       </c>
-      <c r="B45" t="str">
+      <c r="B46" t="str">
         <v>Other Expenses</v>
       </c>
-      <c r="C45" t="str">
-        <v>Expense</v>
-      </c>
-      <c r="D45" t="str">
+      <c r="C46" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D46" t="str">
         <v>Other</v>
       </c>
-      <c r="E45" t="str">
+      <c r="E46" t="str">
         <v>Miscellaneous</v>
       </c>
-      <c r="F45" t="str">
+      <c r="F46" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F45"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F46"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-15T21:55:01.005Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -472,7 +472,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M4"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -540,9 +540,50 @@
         <v>Main Account</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>ACC-01</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="C4" t="str">
+        <v>000001</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="M4" t="str">
+        <v>11201</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-15T21:59:18.271Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -472,7 +472,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M5"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -581,9 +581,50 @@
         <v>11201</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>ACC-02</v>
+      </c>
+      <c r="B5" t="str">
+        <v>FDRL5530</v>
+      </c>
+      <c r="C5" t="str">
+        <v>10020100375530</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Savings</v>
+      </c>
+      <c r="E5">
+        <v>18944.08</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>18944.08</v>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="M5" t="str">
+        <v>11003</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-15T22:04:59.913Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K6"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -463,9 +463,114 @@
         <v>Bank Reference</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>TXN-1001</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Investment</v>
+      </c>
+      <c r="E4" t="str">
+        <v>APY</v>
+      </c>
+      <c r="F4">
+        <v>409</v>
+      </c>
+      <c r="G4" t="str">
+        <v>FDRL5530</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Linked: INV-01</v>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v>500161796770</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>TXN-1002</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Debt Given</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Baby</v>
+      </c>
+      <c r="F5">
+        <v>25000</v>
+      </c>
+      <c r="G5" t="str">
+        <v>FDRL5530</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Linked: DEBT-01 (Baby)</v>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v>S73279105</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>TXN-1003</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2026-07-05</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Investment</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Zeroda Coin</v>
+      </c>
+      <c r="F6">
+        <v>1996</v>
+      </c>
+      <c r="G6" t="str">
+        <v>FDRL5530</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Linked: INV-02</v>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v>S39703384</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K6"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -601,10 +706,10 @@
         <v>0</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>27405</v>
       </c>
       <c r="H5">
-        <v>18944.08</v>
+        <v>-8460.92</v>
       </c>
       <c r="I5" t="str">
         <v/>
@@ -631,7 +736,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:R4"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -718,16 +823,72 @@
         <v>Main Account</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>DEBT-01</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Debt Receivable</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Baby</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Posted 2026-07-01</v>
+      </c>
+      <c r="E4">
+        <v>25000</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>25000</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>25000</v>
+      </c>
+      <c r="L4" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v>Open</v>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N5"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -799,9 +960,97 @@
         <v>Opening Balance</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>INV-01</v>
+      </c>
+      <c r="B4" t="str">
+        <v>APY</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Other</v>
+      </c>
+      <c r="D4" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="E4">
+        <v>409</v>
+      </c>
+      <c r="F4">
+        <v>409</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4" t="str">
+        <v>FDRL5530</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Open</v>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>INV-02</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Zeroda Coin</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Other</v>
+      </c>
+      <c r="D5" t="str">
+        <v>2026-07-05</v>
+      </c>
+      <c r="E5">
+        <v>1996</v>
+      </c>
+      <c r="F5">
+        <v>1996</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5" t="str">
+        <v>FDRL5530</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Open</v>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-15T22:06:14.893Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -834,7 +834,7 @@
         <v>Baby</v>
       </c>
       <c r="D4" t="str">
-        <v>Posted 2026-07-01</v>
+        <v>Debt given for expense</v>
       </c>
       <c r="E4">
         <v>25000</v>
@@ -861,7 +861,7 @@
         <v>2026-07-01</v>
       </c>
       <c r="M4" t="str">
-        <v/>
+        <v>2026-08-01</v>
       </c>
       <c r="N4" t="str">
         <v>Open</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-15T22:07:37.213Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K7"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -568,9 +568,44 @@
         <v>S39703384</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>TXN-1004</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2026-07-05</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Investment</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Addiitonal invenstment through coin</v>
+      </c>
+      <c r="F7">
+        <v>1331</v>
+      </c>
+      <c r="G7" t="str">
+        <v>FDRL5530</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Linked: INV-02 (top-up)</v>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v>S39762571</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -706,10 +741,10 @@
         <v>0</v>
       </c>
       <c r="G5">
-        <v>27405</v>
+        <v>28736</v>
       </c>
       <c r="H5">
-        <v>-8460.92</v>
+        <v>-9791.92</v>
       </c>
       <c r="I5" t="str">
         <v/>
@@ -1018,10 +1053,10 @@
         <v>2026-07-05</v>
       </c>
       <c r="E5">
-        <v>1996</v>
+        <v>3327</v>
       </c>
       <c r="F5">
-        <v>1996</v>
+        <v>3327</v>
       </c>
       <c r="G5">
         <v>0</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-15T22:10:06.122Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -612,7 +612,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M4"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -721,50 +721,9 @@
         <v>11201</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>ACC-02</v>
-      </c>
-      <c r="B5" t="str">
-        <v>FDRL5530</v>
-      </c>
-      <c r="C5" t="str">
-        <v>10020100375530</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Savings</v>
-      </c>
-      <c r="E5">
-        <v>18944.08</v>
-      </c>
-      <c r="F5">
-        <v>0</v>
-      </c>
-      <c r="G5">
-        <v>28736</v>
-      </c>
-      <c r="H5">
-        <v>-9791.92</v>
-      </c>
-      <c r="I5" t="str">
-        <v/>
-      </c>
-      <c r="J5" t="str">
-        <v/>
-      </c>
-      <c r="K5" t="str">
-        <v/>
-      </c>
-      <c r="L5" t="str">
-        <v>Pending</v>
-      </c>
-      <c r="M5" t="str">
-        <v>11003</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2348,7 +2307,7 @@
         <v>Theme</v>
       </c>
       <c r="B6" t="str">
-        <v>dark</v>
+        <v>light</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-15T22:13:54.785Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -612,7 +612,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M5"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -721,9 +721,50 @@
         <v>11201</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>ACC-02</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Federa</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v>Savings</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="M5" t="str">
+        <v>11003</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-16T11:03:43.863Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -726,25 +726,25 @@
         <v>ACC-02</v>
       </c>
       <c r="B5" t="str">
-        <v>Federa</v>
+        <v>FDRL5530</v>
       </c>
       <c r="C5" t="str">
-        <v/>
+        <v>10020100375530</v>
       </c>
       <c r="D5" t="str">
         <v>Savings</v>
       </c>
       <c r="E5">
-        <v>0</v>
+        <v>18756</v>
       </c>
       <c r="F5">
         <v>0</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>28736</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>-9980</v>
       </c>
       <c r="I5" t="str">
         <v/>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-17T13:04:53.345Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -923,7 +923,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N6"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -1083,9 +1083,53 @@
         <v/>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>INV-03</v>
+      </c>
+      <c r="B6" t="str">
+        <v>KITES</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Stocks</v>
+      </c>
+      <c r="D6" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="E6">
+        <v>264004</v>
+      </c>
+      <c r="F6">
+        <v>264004</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v>Open</v>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N6"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-17T23:17:04.853Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K17"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -603,9 +603,359 @@
         <v>S39762571</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>TXN-1005</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2026-07-05</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Utilities - Internet &amp; Mobile</v>
+      </c>
+      <c r="E8" t="str">
+        <v>JIO Wifi</v>
+      </c>
+      <c r="F8">
+        <v>860.9</v>
+      </c>
+      <c r="G8" t="str">
+        <v>FDRL5530</v>
+      </c>
+      <c r="H8" t="str">
+        <v>GPay</v>
+      </c>
+      <c r="I8" t="str">
+        <v>Import: ACC_STATEMENT_XXXXX5530_01JUL2026_16AUG2026_1786811285545316.pdf</v>
+      </c>
+      <c r="J8" t="str">
+        <v>51003</v>
+      </c>
+      <c r="K8" t="str">
+        <v>S43126360</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>TXN-1006</v>
+      </c>
+      <c r="B9" t="str">
+        <v>2026-07-09</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Utilities - Internet &amp; Mobile</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Airtel Mobile</v>
+      </c>
+      <c r="F9">
+        <v>199</v>
+      </c>
+      <c r="G9" t="str">
+        <v>FDRL5530</v>
+      </c>
+      <c r="H9" t="str">
+        <v>GPay</v>
+      </c>
+      <c r="I9" t="str">
+        <v>Import: ACC_STATEMENT_XXXXX5530_01JUL2026_16AUG2026_1786811285545316.pdf</v>
+      </c>
+      <c r="J9" t="str">
+        <v>51003</v>
+      </c>
+      <c r="K9" t="str">
+        <v>S12627360</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>TXN-1007</v>
+      </c>
+      <c r="B10" t="str">
+        <v>2026-07-09</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Utilities - Internet &amp; Mobile</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Airtel SMS Oversease</v>
+      </c>
+      <c r="F10">
+        <v>118</v>
+      </c>
+      <c r="G10" t="str">
+        <v>FDRL5530</v>
+      </c>
+      <c r="H10" t="str">
+        <v>GPay</v>
+      </c>
+      <c r="I10" t="str">
+        <v>Import: ACC_STATEMENT_XXXXX5530_01JUL2026_16AUG2026_1786811285545316.pdf</v>
+      </c>
+      <c r="J10" t="str">
+        <v>51003</v>
+      </c>
+      <c r="K10" t="str">
+        <v>S12662114</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>TXN-1008</v>
+      </c>
+      <c r="B11" t="str">
+        <v>2026-07-09</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Gifts &amp; Functions</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Anusha passam</v>
+      </c>
+      <c r="F11">
+        <v>2500</v>
+      </c>
+      <c r="G11" t="str">
+        <v>FDRL5530</v>
+      </c>
+      <c r="H11" t="str">
+        <v>GPay</v>
+      </c>
+      <c r="I11" t="str">
+        <v>Import: ACC_STATEMENT_XXXXX5530_01JUL2026_16AUG2026_1786811285545316.pdf</v>
+      </c>
+      <c r="J11" t="str">
+        <v>54005</v>
+      </c>
+      <c r="K11" t="str">
+        <v>S21578154</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>TXN-1009</v>
+      </c>
+      <c r="B12" t="str">
+        <v>2026-07-20</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Gifts &amp; Functions</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Merin Passam</v>
+      </c>
+      <c r="F12">
+        <v>300</v>
+      </c>
+      <c r="G12" t="str">
+        <v>FDRL5530</v>
+      </c>
+      <c r="H12" t="str">
+        <v>GPay</v>
+      </c>
+      <c r="I12" t="str">
+        <v>Import: ACC_STATEMENT_XXXXX5530_01JUL2026_16AUG2026_1786811285545316.pdf</v>
+      </c>
+      <c r="J12" t="str">
+        <v>54005</v>
+      </c>
+      <c r="K12" t="str">
+        <v>S89121143</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>TXN-1010</v>
+      </c>
+      <c r="B13" t="str">
+        <v>2026-07-22</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Health &amp; Medical</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Amma expense</v>
+      </c>
+      <c r="F13">
+        <v>3000</v>
+      </c>
+      <c r="G13" t="str">
+        <v>FDRL5530</v>
+      </c>
+      <c r="H13" t="str">
+        <v>GPay</v>
+      </c>
+      <c r="I13" t="str">
+        <v>Import: ACC_STATEMENT_XXXXX5530_01JUL2026_16AUG2026_1786811285545316.pdf</v>
+      </c>
+      <c r="J13" t="str">
+        <v>54002</v>
+      </c>
+      <c r="K13" t="str">
+        <v>S26788660</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>TXN-1011</v>
+      </c>
+      <c r="B14" t="str">
+        <v>2026-07-25</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Gifts &amp; Functions</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Shyma C Joji Medical</v>
+      </c>
+      <c r="F14">
+        <v>10000</v>
+      </c>
+      <c r="G14" t="str">
+        <v>FDRL5530</v>
+      </c>
+      <c r="H14" t="str">
+        <v>GPay</v>
+      </c>
+      <c r="I14" t="str">
+        <v>Import: ACC_STATEMENT_XXXXX5530_01JUL2026_16AUG2026_1786811285545316.pdf</v>
+      </c>
+      <c r="J14" t="str">
+        <v>54005</v>
+      </c>
+      <c r="K14" t="str">
+        <v>S68627622</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>TXN-1012</v>
+      </c>
+      <c r="B15" t="str">
+        <v>2026-07-30</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Family Support</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Famly Expense</v>
+      </c>
+      <c r="F15">
+        <v>3000</v>
+      </c>
+      <c r="G15" t="str">
+        <v>FDRL5530</v>
+      </c>
+      <c r="H15" t="str">
+        <v>GPay</v>
+      </c>
+      <c r="I15" t="str">
+        <v>Import: ACC_STATEMENT_XXXXX5530_01JUL2026_16AUG2026_1786811285545316.pdf</v>
+      </c>
+      <c r="J15" t="str">
+        <v>54001</v>
+      </c>
+      <c r="K15" t="str">
+        <v>S53907286</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>TXN-1013</v>
+      </c>
+      <c r="B16" t="str">
+        <v>2026-08-05</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Investment</v>
+      </c>
+      <c r="E16" t="str">
+        <v>ACHDR/ZERODHA BROKING</v>
+      </c>
+      <c r="F16">
+        <v>1996</v>
+      </c>
+      <c r="G16" t="str">
+        <v>FDRL5530</v>
+      </c>
+      <c r="H16" t="str">
+        <v>Bank Transfer</v>
+      </c>
+      <c r="I16" t="str">
+        <v>Linked: INV-02 (top-up)</v>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16" t="str">
+        <v>S42450843</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>TXN-1014</v>
+      </c>
+      <c r="B17" t="str">
+        <v>2026-08-05</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Investment</v>
+      </c>
+      <c r="E17" t="str">
+        <v>ACHDR/ZERODHA BROKING</v>
+      </c>
+      <c r="F17">
+        <v>1331</v>
+      </c>
+      <c r="G17" t="str">
+        <v>FDRL5530</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Bank Import</v>
+      </c>
+      <c r="I17" t="str">
+        <v>Linked: INV-02 (top-up)</v>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+      <c r="K17" t="str">
+        <v>S42712734</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K17"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -741,10 +1091,10 @@
         <v>0</v>
       </c>
       <c r="G5">
-        <v>28736</v>
+        <v>52040.9</v>
       </c>
       <c r="H5">
-        <v>-9980</v>
+        <v>-33284.9</v>
       </c>
       <c r="I5" t="str">
         <v/>
@@ -1053,10 +1403,10 @@
         <v>2026-07-05</v>
       </c>
       <c r="E5">
-        <v>3327</v>
+        <v>6654</v>
       </c>
       <c r="F5">
-        <v>3327</v>
+        <v>6654</v>
       </c>
       <c r="G5">
         <v>0</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-17T23:17:53.269Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K16"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -675,7 +675,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>TXN-1007</v>
+        <v>TXN-1008</v>
       </c>
       <c r="B10" t="str">
         <v>2026-07-09</v>
@@ -684,13 +684,13 @@
         <v>Expense</v>
       </c>
       <c r="D10" t="str">
-        <v>Utilities - Internet &amp; Mobile</v>
+        <v>Gifts &amp; Functions</v>
       </c>
       <c r="E10" t="str">
-        <v>Airtel SMS Oversease</v>
+        <v>Anusha passam</v>
       </c>
       <c r="F10">
-        <v>118</v>
+        <v>2500</v>
       </c>
       <c r="G10" t="str">
         <v>FDRL5530</v>
@@ -702,18 +702,18 @@
         <v>Import: ACC_STATEMENT_XXXXX5530_01JUL2026_16AUG2026_1786811285545316.pdf</v>
       </c>
       <c r="J10" t="str">
-        <v>51003</v>
+        <v>54005</v>
       </c>
       <c r="K10" t="str">
-        <v>S12662114</v>
+        <v>S21578154</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>TXN-1008</v>
+        <v>TXN-1009</v>
       </c>
       <c r="B11" t="str">
-        <v>2026-07-09</v>
+        <v>2026-07-20</v>
       </c>
       <c r="C11" t="str">
         <v>Expense</v>
@@ -722,10 +722,10 @@
         <v>Gifts &amp; Functions</v>
       </c>
       <c r="E11" t="str">
-        <v>Anusha passam</v>
+        <v>Merin Passam</v>
       </c>
       <c r="F11">
-        <v>2500</v>
+        <v>300</v>
       </c>
       <c r="G11" t="str">
         <v>FDRL5530</v>
@@ -740,27 +740,27 @@
         <v>54005</v>
       </c>
       <c r="K11" t="str">
-        <v>S21578154</v>
+        <v>S89121143</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>TXN-1009</v>
+        <v>TXN-1010</v>
       </c>
       <c r="B12" t="str">
-        <v>2026-07-20</v>
+        <v>2026-07-22</v>
       </c>
       <c r="C12" t="str">
         <v>Expense</v>
       </c>
       <c r="D12" t="str">
-        <v>Gifts &amp; Functions</v>
+        <v>Health &amp; Medical</v>
       </c>
       <c r="E12" t="str">
-        <v>Merin Passam</v>
+        <v>Amma expense</v>
       </c>
       <c r="F12">
-        <v>300</v>
+        <v>3000</v>
       </c>
       <c r="G12" t="str">
         <v>FDRL5530</v>
@@ -772,30 +772,30 @@
         <v>Import: ACC_STATEMENT_XXXXX5530_01JUL2026_16AUG2026_1786811285545316.pdf</v>
       </c>
       <c r="J12" t="str">
-        <v>54005</v>
+        <v>54002</v>
       </c>
       <c r="K12" t="str">
-        <v>S89121143</v>
+        <v>S26788660</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>TXN-1010</v>
+        <v>TXN-1011</v>
       </c>
       <c r="B13" t="str">
-        <v>2026-07-22</v>
+        <v>2026-07-25</v>
       </c>
       <c r="C13" t="str">
         <v>Expense</v>
       </c>
       <c r="D13" t="str">
-        <v>Health &amp; Medical</v>
+        <v>Gifts &amp; Functions</v>
       </c>
       <c r="E13" t="str">
-        <v>Amma expense</v>
+        <v>Shyma C Joji Medical</v>
       </c>
       <c r="F13">
-        <v>3000</v>
+        <v>10000</v>
       </c>
       <c r="G13" t="str">
         <v>FDRL5530</v>
@@ -807,30 +807,30 @@
         <v>Import: ACC_STATEMENT_XXXXX5530_01JUL2026_16AUG2026_1786811285545316.pdf</v>
       </c>
       <c r="J13" t="str">
-        <v>54002</v>
+        <v>54005</v>
       </c>
       <c r="K13" t="str">
-        <v>S26788660</v>
+        <v>S68627622</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>TXN-1011</v>
+        <v>TXN-1012</v>
       </c>
       <c r="B14" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-30</v>
       </c>
       <c r="C14" t="str">
         <v>Expense</v>
       </c>
       <c r="D14" t="str">
-        <v>Gifts &amp; Functions</v>
+        <v>Family Support</v>
       </c>
       <c r="E14" t="str">
-        <v>Shyma C Joji Medical</v>
+        <v>Famly Expense</v>
       </c>
       <c r="F14">
-        <v>10000</v>
+        <v>3000</v>
       </c>
       <c r="G14" t="str">
         <v>FDRL5530</v>
@@ -842,50 +842,50 @@
         <v>Import: ACC_STATEMENT_XXXXX5530_01JUL2026_16AUG2026_1786811285545316.pdf</v>
       </c>
       <c r="J14" t="str">
-        <v>54005</v>
+        <v>54001</v>
       </c>
       <c r="K14" t="str">
-        <v>S68627622</v>
+        <v>S53907286</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>TXN-1012</v>
+        <v>TXN-1013</v>
       </c>
       <c r="B15" t="str">
-        <v>2026-07-30</v>
+        <v>2026-08-05</v>
       </c>
       <c r="C15" t="str">
         <v>Expense</v>
       </c>
       <c r="D15" t="str">
-        <v>Family Support</v>
+        <v>Investment</v>
       </c>
       <c r="E15" t="str">
-        <v>Famly Expense</v>
+        <v>ACHDR/ZERODHA BROKING</v>
       </c>
       <c r="F15">
-        <v>3000</v>
+        <v>1996</v>
       </c>
       <c r="G15" t="str">
         <v>FDRL5530</v>
       </c>
       <c r="H15" t="str">
-        <v>GPay</v>
+        <v>Bank Transfer</v>
       </c>
       <c r="I15" t="str">
-        <v>Import: ACC_STATEMENT_XXXXX5530_01JUL2026_16AUG2026_1786811285545316.pdf</v>
+        <v>Linked: INV-02 (top-up)</v>
       </c>
       <c r="J15" t="str">
-        <v>54001</v>
+        <v/>
       </c>
       <c r="K15" t="str">
-        <v>S53907286</v>
+        <v>S42450843</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>TXN-1013</v>
+        <v>TXN-1014</v>
       </c>
       <c r="B16" t="str">
         <v>2026-08-05</v>
@@ -900,13 +900,13 @@
         <v>ACHDR/ZERODHA BROKING</v>
       </c>
       <c r="F16">
-        <v>1996</v>
+        <v>1331</v>
       </c>
       <c r="G16" t="str">
         <v>FDRL5530</v>
       </c>
       <c r="H16" t="str">
-        <v>Bank Transfer</v>
+        <v>Bank Import</v>
       </c>
       <c r="I16" t="str">
         <v>Linked: INV-02 (top-up)</v>
@@ -915,47 +915,12 @@
         <v/>
       </c>
       <c r="K16" t="str">
-        <v>S42450843</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>TXN-1014</v>
-      </c>
-      <c r="B17" t="str">
-        <v>2026-08-05</v>
-      </c>
-      <c r="C17" t="str">
-        <v>Expense</v>
-      </c>
-      <c r="D17" t="str">
-        <v>Investment</v>
-      </c>
-      <c r="E17" t="str">
-        <v>ACHDR/ZERODHA BROKING</v>
-      </c>
-      <c r="F17">
-        <v>1331</v>
-      </c>
-      <c r="G17" t="str">
-        <v>FDRL5530</v>
-      </c>
-      <c r="H17" t="str">
-        <v>Bank Import</v>
-      </c>
-      <c r="I17" t="str">
-        <v>Linked: INV-02 (top-up)</v>
-      </c>
-      <c r="J17" t="str">
-        <v/>
-      </c>
-      <c r="K17" t="str">
         <v>S42712734</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K16"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1091,10 +1056,10 @@
         <v>0</v>
       </c>
       <c r="G5">
-        <v>52040.9</v>
+        <v>51922.9</v>
       </c>
       <c r="H5">
-        <v>-33284.9</v>
+        <v>-33166.9</v>
       </c>
       <c r="I5" t="str">
         <v/>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-17T23:20:06.020Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K23"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -918,9 +918,254 @@
         <v>S42712734</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>TXN-1015</v>
+      </c>
+      <c r="B17" t="str">
+        <v>2026-07-09</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Income</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Dividends / Profit</v>
+      </c>
+      <c r="E17" t="str">
+        <v>ACHCR/TMPVL DIV</v>
+      </c>
+      <c r="F17">
+        <v>78</v>
+      </c>
+      <c r="G17" t="str">
+        <v>FDRL5530</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="I17" t="str">
+        <v>Dividend: INV-03 (KITES)</v>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+      <c r="K17" t="str">
+        <v>S14649706</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>TXN-1016</v>
+      </c>
+      <c r="B18" t="str">
+        <v>2026-07-10</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Income</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Dividends / Profit</v>
+      </c>
+      <c r="E18" t="str">
+        <v>ACHCR/TATAPOWERDIV1007</v>
+      </c>
+      <c r="F18">
+        <v>150</v>
+      </c>
+      <c r="G18" t="str">
+        <v>FDRL5530</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="I18" t="str">
+        <v>Dividend: INV-03 (KITES)</v>
+      </c>
+      <c r="J18" t="str">
+        <v/>
+      </c>
+      <c r="K18" t="str">
+        <v>S22783397</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>TXN-1017</v>
+      </c>
+      <c r="B19" t="str">
+        <v>2026-07-15</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Income</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Dividends / Profit</v>
+      </c>
+      <c r="E19" t="str">
+        <v>ACHCR/ExideIndustFnl20</v>
+      </c>
+      <c r="F19">
+        <v>50</v>
+      </c>
+      <c r="G19" t="str">
+        <v>FDRL5530</v>
+      </c>
+      <c r="H19" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="I19" t="str">
+        <v>Dividend: INV-03 (KITES)</v>
+      </c>
+      <c r="J19" t="str">
+        <v/>
+      </c>
+      <c r="K19" t="str">
+        <v>S4335896</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>TXN-1018</v>
+      </c>
+      <c r="B20" t="str">
+        <v>2026-07-28</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Income</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Dividends / Profit</v>
+      </c>
+      <c r="E20" t="str">
+        <v>ACHCR/ITC LIMITED</v>
+      </c>
+      <c r="F20">
+        <v>32</v>
+      </c>
+      <c r="G20" t="str">
+        <v>FDRL5530</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="I20" t="str">
+        <v>Dividend: INV-03 (KITES)</v>
+      </c>
+      <c r="J20" t="str">
+        <v/>
+      </c>
+      <c r="K20" t="str">
+        <v>S8407528</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>TXN-1019</v>
+      </c>
+      <c r="B21" t="str">
+        <v>2026-07-28</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Income</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Dividend Income</v>
+      </c>
+      <c r="E21" t="str">
+        <v>ACHCR/Hindalco Fin Div</v>
+      </c>
+      <c r="F21">
+        <v>5</v>
+      </c>
+      <c r="G21" t="str">
+        <v>FDRL5530</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Bank Import</v>
+      </c>
+      <c r="I21" t="str">
+        <v>Import: ACC_STATEMENT_XXXXX5530_01JUL2026_16AUG2026_1786811285545316.pdf</v>
+      </c>
+      <c r="J21" t="str">
+        <v>42002</v>
+      </c>
+      <c r="K21" t="str">
+        <v>S16605168</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>TXN-1020</v>
+      </c>
+      <c r="B22" t="str">
+        <v>2026-08-06</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Income</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Dividends / Profit</v>
+      </c>
+      <c r="E22" t="str">
+        <v>ACHCR/POWERGRID</v>
+      </c>
+      <c r="F22">
+        <v>35</v>
+      </c>
+      <c r="G22" t="str">
+        <v>FDRL5530</v>
+      </c>
+      <c r="H22" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="I22" t="str">
+        <v>Dividend: INV-03 (KITES)</v>
+      </c>
+      <c r="J22" t="str">
+        <v/>
+      </c>
+      <c r="K22" t="str">
+        <v>S65674387</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>TXN-1021</v>
+      </c>
+      <c r="B23" t="str">
+        <v>2026-08-07</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Income</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Freelance Income</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Freelance income from tittu</v>
+      </c>
+      <c r="F23">
+        <v>5000</v>
+      </c>
+      <c r="G23" t="str">
+        <v>FDRL5530</v>
+      </c>
+      <c r="H23" t="str">
+        <v>GPay</v>
+      </c>
+      <c r="I23" t="str">
+        <v>Import: ACC_STATEMENT_XXXXX5530_01JUL2026_16AUG2026_1786811285545316.pdf</v>
+      </c>
+      <c r="J23" t="str">
+        <v>41003</v>
+      </c>
+      <c r="K23" t="str">
+        <v>S82403501</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K23"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1053,13 +1298,13 @@
         <v>18756</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>5350</v>
       </c>
       <c r="G5">
         <v>51922.9</v>
       </c>
       <c r="H5">
-        <v>-33166.9</v>
+        <v>-27816.9</v>
       </c>
       <c r="I5" t="str">
         <v/>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-17T23:23:42.813Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -1696,7 +1696,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F47"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -2578,27 +2578,47 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
+        <v>55007</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Bank Charges</v>
+      </c>
+      <c r="E46" t="str">
+        <v/>
+      </c>
+      <c r="F46" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
         <v>59999</v>
       </c>
-      <c r="B46" t="str">
+      <c r="B47" t="str">
         <v>Other Expenses</v>
       </c>
-      <c r="C46" t="str">
-        <v>Expense</v>
-      </c>
-      <c r="D46" t="str">
+      <c r="C47" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D47" t="str">
         <v>Other</v>
       </c>
-      <c r="E46" t="str">
+      <c r="E47" t="str">
         <v>Miscellaneous</v>
       </c>
-      <c r="F46" t="str">
+      <c r="F47" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F46"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F47"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-17T23:28:02.129Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K24"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1163,9 +1163,44 @@
         <v>S82403501</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>TXN-1022</v>
+      </c>
+      <c r="B24" t="str">
+        <v>2026-07-29</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="E24" t="str">
+        <v>CHRG/MOB ALERT/JUN26</v>
+      </c>
+      <c r="F24">
+        <v>2.84</v>
+      </c>
+      <c r="G24" t="str">
+        <v>FDRL5530</v>
+      </c>
+      <c r="H24" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="I24" t="str">
+        <v>Import: ACC_STATEMENT_XXXXX5530_01JUL2026_16AUG2026_1786811285545316.pdf</v>
+      </c>
+      <c r="J24" t="str">
+        <v>55007</v>
+      </c>
+      <c r="K24" t="str">
+        <v>S30523821</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K24"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1301,10 +1336,10 @@
         <v>5350</v>
       </c>
       <c r="G5">
-        <v>51922.9</v>
+        <v>51925.74</v>
       </c>
       <c r="H5">
-        <v>-27816.9</v>
+        <v>-27819.74</v>
       </c>
       <c r="I5" t="str">
         <v/>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-18T00:43:16.267Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:L24"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -415,7 +415,8 @@
     <col min="8" max="8" width="15.83203125" customWidth="1"/>
     <col min="9" max="9" width="24.83203125" customWidth="1"/>
     <col min="10" max="10" width="12.83203125" customWidth="1"/>
-    <col min="11" max="11" width="14.83203125" customWidth="1"/>
+    <col min="11" max="11" width="13.83203125" customWidth="1"/>
+    <col min="12" max="12" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -460,6 +461,9 @@
         <v>COA Account</v>
       </c>
       <c r="K3" t="str">
+        <v>Offset Account</v>
+      </c>
+      <c r="L3" t="str">
         <v>Bank Reference</v>
       </c>
     </row>
@@ -495,6 +499,9 @@
         <v/>
       </c>
       <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
         <v>500161796770</v>
       </c>
     </row>
@@ -530,6 +537,9 @@
         <v/>
       </c>
       <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
         <v>S73279105</v>
       </c>
     </row>
@@ -565,6 +575,9 @@
         <v/>
       </c>
       <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
         <v>S39703384</v>
       </c>
     </row>
@@ -600,6 +613,9 @@
         <v/>
       </c>
       <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
         <v>S39762571</v>
       </c>
     </row>
@@ -635,6 +651,9 @@
         <v>51003</v>
       </c>
       <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
         <v>S43126360</v>
       </c>
     </row>
@@ -670,6 +689,9 @@
         <v>51003</v>
       </c>
       <c r="K9" t="str">
+        <v/>
+      </c>
+      <c r="L9" t="str">
         <v>S12627360</v>
       </c>
     </row>
@@ -705,6 +727,9 @@
         <v>54005</v>
       </c>
       <c r="K10" t="str">
+        <v/>
+      </c>
+      <c r="L10" t="str">
         <v>S21578154</v>
       </c>
     </row>
@@ -740,6 +765,9 @@
         <v>54005</v>
       </c>
       <c r="K11" t="str">
+        <v/>
+      </c>
+      <c r="L11" t="str">
         <v>S89121143</v>
       </c>
     </row>
@@ -775,6 +803,9 @@
         <v>54002</v>
       </c>
       <c r="K12" t="str">
+        <v/>
+      </c>
+      <c r="L12" t="str">
         <v>S26788660</v>
       </c>
     </row>
@@ -810,6 +841,9 @@
         <v>54005</v>
       </c>
       <c r="K13" t="str">
+        <v/>
+      </c>
+      <c r="L13" t="str">
         <v>S68627622</v>
       </c>
     </row>
@@ -845,6 +879,9 @@
         <v>54001</v>
       </c>
       <c r="K14" t="str">
+        <v/>
+      </c>
+      <c r="L14" t="str">
         <v>S53907286</v>
       </c>
     </row>
@@ -880,6 +917,9 @@
         <v/>
       </c>
       <c r="K15" t="str">
+        <v/>
+      </c>
+      <c r="L15" t="str">
         <v>S42450843</v>
       </c>
     </row>
@@ -915,6 +955,9 @@
         <v/>
       </c>
       <c r="K16" t="str">
+        <v/>
+      </c>
+      <c r="L16" t="str">
         <v>S42712734</v>
       </c>
     </row>
@@ -950,6 +993,9 @@
         <v/>
       </c>
       <c r="K17" t="str">
+        <v/>
+      </c>
+      <c r="L17" t="str">
         <v>S14649706</v>
       </c>
     </row>
@@ -985,6 +1031,9 @@
         <v/>
       </c>
       <c r="K18" t="str">
+        <v/>
+      </c>
+      <c r="L18" t="str">
         <v>S22783397</v>
       </c>
     </row>
@@ -1020,6 +1069,9 @@
         <v/>
       </c>
       <c r="K19" t="str">
+        <v/>
+      </c>
+      <c r="L19" t="str">
         <v>S4335896</v>
       </c>
     </row>
@@ -1055,6 +1107,9 @@
         <v/>
       </c>
       <c r="K20" t="str">
+        <v/>
+      </c>
+      <c r="L20" t="str">
         <v>S8407528</v>
       </c>
     </row>
@@ -1090,6 +1145,9 @@
         <v>42002</v>
       </c>
       <c r="K21" t="str">
+        <v/>
+      </c>
+      <c r="L21" t="str">
         <v>S16605168</v>
       </c>
     </row>
@@ -1125,6 +1183,9 @@
         <v/>
       </c>
       <c r="K22" t="str">
+        <v/>
+      </c>
+      <c r="L22" t="str">
         <v>S65674387</v>
       </c>
     </row>
@@ -1160,6 +1221,9 @@
         <v>41003</v>
       </c>
       <c r="K23" t="str">
+        <v/>
+      </c>
+      <c r="L23" t="str">
         <v>S82403501</v>
       </c>
     </row>
@@ -1195,12 +1259,15 @@
         <v>55007</v>
       </c>
       <c r="K24" t="str">
+        <v/>
+      </c>
+      <c r="L24" t="str">
         <v>S30523821</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L24"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1731,7 +1798,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F48"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -1953,130 +2020,130 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>21001</v>
+        <v>13002</v>
       </c>
       <c r="B13" t="str">
-        <v>SBI Home Loan</v>
+        <v>Payment on Behlaf</v>
       </c>
       <c r="C13" t="str">
-        <v>Liability</v>
+        <v>Asset</v>
       </c>
       <c r="D13" t="str">
-        <v>Bank Loans</v>
+        <v>Receivables</v>
       </c>
       <c r="E13" t="str">
-        <v>Housing Loan</v>
+        <v>Card payment</v>
       </c>
       <c r="F13" t="str">
-        <v>home loan,housing loan</v>
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>22001</v>
+        <v>21001</v>
       </c>
       <c r="B14" t="str">
-        <v>Personal Borrowings</v>
+        <v>SBI Home Loan</v>
       </c>
       <c r="C14" t="str">
         <v>Liability</v>
       </c>
       <c r="D14" t="str">
-        <v>Debts Payable</v>
+        <v>Bank Loans</v>
       </c>
       <c r="E14" t="str">
-        <v>From People</v>
+        <v>Housing Loan</v>
       </c>
       <c r="F14" t="str">
-        <v>borrowed</v>
+        <v>home loan,housing loan</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>23001</v>
+        <v>22001</v>
       </c>
       <c r="B15" t="str">
-        <v>Credit Card Payable</v>
+        <v>Personal Borrowings</v>
       </c>
       <c r="C15" t="str">
         <v>Liability</v>
       </c>
       <c r="D15" t="str">
-        <v>Credit Cards</v>
+        <v>Debts Payable</v>
       </c>
       <c r="E15" t="str">
-        <v>ICICI Amazon Pay</v>
+        <v>From People</v>
       </c>
       <c r="F15" t="str">
-        <v>icici amazon</v>
+        <v>borrowed</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>30001</v>
+        <v>23001</v>
       </c>
       <c r="B16" t="str">
-        <v>Opening Balances / Net Worth</v>
+        <v>Credit Card Payable</v>
       </c>
       <c r="C16" t="str">
-        <v>Equity</v>
+        <v>Liability</v>
       </c>
       <c r="D16" t="str">
-        <v>Capital</v>
+        <v>Credit Cards</v>
       </c>
       <c r="E16" t="str">
-        <v>Opening Balance</v>
+        <v>ICICI Amazon Pay</v>
       </c>
       <c r="F16" t="str">
-        <v/>
+        <v>icici amazon</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>41001</v>
+        <v>30001</v>
       </c>
       <c r="B17" t="str">
-        <v>Salary</v>
+        <v>Opening Balances / Net Worth</v>
       </c>
       <c r="C17" t="str">
-        <v>Income</v>
+        <v>Equity</v>
       </c>
       <c r="D17" t="str">
-        <v>Employment</v>
+        <v>Capital</v>
       </c>
       <c r="E17" t="str">
-        <v>Monthly Salary</v>
+        <v>Opening Balance</v>
       </c>
       <c r="F17" t="str">
-        <v>salary,sal cr,infopark</v>
+        <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>41002</v>
+        <v>41001</v>
       </c>
       <c r="B18" t="str">
-        <v>Business Income</v>
+        <v>Salary</v>
       </c>
       <c r="C18" t="str">
         <v>Income</v>
       </c>
       <c r="D18" t="str">
-        <v>Business</v>
+        <v>Employment</v>
       </c>
       <c r="E18" t="str">
-        <v>General</v>
+        <v>Monthly Salary</v>
       </c>
       <c r="F18" t="str">
-        <v>business</v>
+        <v>salary,sal cr,infopark</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>41003</v>
+        <v>41002</v>
       </c>
       <c r="B19" t="str">
-        <v>Freelance Income</v>
+        <v>Business Income</v>
       </c>
       <c r="C19" t="str">
         <v>Income</v>
@@ -2085,38 +2152,38 @@
         <v>Business</v>
       </c>
       <c r="E19" t="str">
-        <v>Freelance</v>
+        <v>General</v>
       </c>
       <c r="F19" t="str">
-        <v>freelance</v>
+        <v>business</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>42001</v>
+        <v>41003</v>
       </c>
       <c r="B20" t="str">
-        <v>Interest Income</v>
+        <v>Freelance Income</v>
       </c>
       <c r="C20" t="str">
         <v>Income</v>
       </c>
       <c r="D20" t="str">
-        <v>Investment Income</v>
+        <v>Business</v>
       </c>
       <c r="E20" t="str">
-        <v>Bank / FD Interest</v>
+        <v>Freelance</v>
       </c>
       <c r="F20" t="str">
-        <v>interest,int.pd,sbint,sb int</v>
+        <v>freelance</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>42002</v>
+        <v>42001</v>
       </c>
       <c r="B21" t="str">
-        <v>Dividend Income</v>
+        <v>Interest Income</v>
       </c>
       <c r="C21" t="str">
         <v>Income</v>
@@ -2125,38 +2192,38 @@
         <v>Investment Income</v>
       </c>
       <c r="E21" t="str">
-        <v>Dividends</v>
+        <v>Bank / FD Interest</v>
       </c>
       <c r="F21" t="str">
-        <v>dividend,div,achcr</v>
+        <v>interest,int.pd,sbint,sb int</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>43001</v>
+        <v>42002</v>
       </c>
       <c r="B22" t="str">
-        <v>Rental Income</v>
+        <v>Dividend Income</v>
       </c>
       <c r="C22" t="str">
         <v>Income</v>
       </c>
       <c r="D22" t="str">
-        <v>Other Income</v>
+        <v>Investment Income</v>
       </c>
       <c r="E22" t="str">
-        <v>Rent Received</v>
+        <v>Dividends</v>
       </c>
       <c r="F22" t="str">
-        <v>rent received</v>
+        <v>dividend,div,achcr</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>43002</v>
+        <v>43001</v>
       </c>
       <c r="B23" t="str">
-        <v>Gifts &amp; Allowance</v>
+        <v>Rental Income</v>
       </c>
       <c r="C23" t="str">
         <v>Income</v>
@@ -2165,18 +2232,18 @@
         <v>Other Income</v>
       </c>
       <c r="E23" t="str">
-        <v>Gifts</v>
+        <v>Rent Received</v>
       </c>
       <c r="F23" t="str">
-        <v>gift received</v>
+        <v>rent received</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>43003</v>
+        <v>43002</v>
       </c>
       <c r="B24" t="str">
-        <v>Debt Settlement Received</v>
+        <v>Gifts &amp; Allowance</v>
       </c>
       <c r="C24" t="str">
         <v>Income</v>
@@ -2185,18 +2252,18 @@
         <v>Other Income</v>
       </c>
       <c r="E24" t="str">
-        <v>Loan Repaid to You</v>
+        <v>Gifts</v>
       </c>
       <c r="F24" t="str">
-        <v>repayment</v>
+        <v>gift received</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>49999</v>
+        <v>43003</v>
       </c>
       <c r="B25" t="str">
-        <v>Other Income</v>
+        <v>Debt Settlement Received</v>
       </c>
       <c r="C25" t="str">
         <v>Income</v>
@@ -2205,38 +2272,38 @@
         <v>Other Income</v>
       </c>
       <c r="E25" t="str">
-        <v>Miscellaneous</v>
+        <v>Loan Repaid to You</v>
       </c>
       <c r="F25" t="str">
-        <v/>
+        <v>repayment</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>51001</v>
+        <v>49999</v>
       </c>
       <c r="B26" t="str">
-        <v>Rent / Housing</v>
+        <v>Other Income</v>
       </c>
       <c r="C26" t="str">
-        <v>Expense</v>
+        <v>Income</v>
       </c>
       <c r="D26" t="str">
-        <v>Household</v>
+        <v>Other Income</v>
       </c>
       <c r="E26" t="str">
-        <v>Rent &amp; Maintenance</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="F26" t="str">
-        <v>rent,maintenance</v>
+        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>51002</v>
+        <v>51001</v>
       </c>
       <c r="B27" t="str">
-        <v>Utilities - Electricity &amp; Water</v>
+        <v>Rent / Housing</v>
       </c>
       <c r="C27" t="str">
         <v>Expense</v>
@@ -2245,18 +2312,18 @@
         <v>Household</v>
       </c>
       <c r="E27" t="str">
-        <v>Electricity / Water</v>
+        <v>Rent &amp; Maintenance</v>
       </c>
       <c r="F27" t="str">
-        <v>kseb,electricity,water bill</v>
+        <v>rent,maintenance</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>51003</v>
+        <v>51002</v>
       </c>
       <c r="B28" t="str">
-        <v>Utilities - Internet &amp; Mobile</v>
+        <v>Utilities - Electricity &amp; Water</v>
       </c>
       <c r="C28" t="str">
         <v>Expense</v>
@@ -2265,18 +2332,18 @@
         <v>Household</v>
       </c>
       <c r="E28" t="str">
-        <v>Recharge / Broadband</v>
+        <v>Electricity / Water</v>
       </c>
       <c r="F28" t="str">
-        <v>recharge,airtel,jio,bsnl,broadband,wifi</v>
+        <v>kseb,electricity,water bill</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>51004</v>
+        <v>51003</v>
       </c>
       <c r="B29" t="str">
-        <v>Gas / LPG</v>
+        <v>Utilities - Internet &amp; Mobile</v>
       </c>
       <c r="C29" t="str">
         <v>Expense</v>
@@ -2285,18 +2352,18 @@
         <v>Household</v>
       </c>
       <c r="E29" t="str">
-        <v>Cooking Gas</v>
+        <v>Recharge / Broadband</v>
       </c>
       <c r="F29" t="str">
-        <v>lpg,indane,gas</v>
+        <v>recharge,airtel,jio,bsnl,broadband,wifi</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>51005</v>
+        <v>51004</v>
       </c>
       <c r="B30" t="str">
-        <v>Household Appliances</v>
+        <v>Gas / LPG</v>
       </c>
       <c r="C30" t="str">
         <v>Expense</v>
@@ -2305,38 +2372,38 @@
         <v>Household</v>
       </c>
       <c r="E30" t="str">
-        <v>Appliances &amp; Repairs</v>
+        <v>Cooking Gas</v>
       </c>
       <c r="F30" t="str">
-        <v>washing machine,appliance,repair</v>
+        <v>lpg,indane,gas</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>52001</v>
+        <v>51005</v>
       </c>
       <c r="B31" t="str">
-        <v>Groceries</v>
+        <v>Household Appliances</v>
       </c>
       <c r="C31" t="str">
         <v>Expense</v>
       </c>
       <c r="D31" t="str">
-        <v>Food</v>
+        <v>Household</v>
       </c>
       <c r="E31" t="str">
-        <v>Provisions</v>
+        <v>Appliances &amp; Repairs</v>
       </c>
       <c r="F31" t="str">
-        <v>grocery,supermarket,mart,bigbasket,blinkit,zepto,dmart</v>
+        <v>washing machine,appliance,repair</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>52002</v>
+        <v>52001</v>
       </c>
       <c r="B32" t="str">
-        <v>Dining Out</v>
+        <v>Groceries</v>
       </c>
       <c r="C32" t="str">
         <v>Expense</v>
@@ -2345,38 +2412,38 @@
         <v>Food</v>
       </c>
       <c r="E32" t="str">
-        <v>Restaurants &amp; Delivery</v>
+        <v>Provisions</v>
       </c>
       <c r="F32" t="str">
-        <v>swiggy,zomato,restaurant,hotel,cafe</v>
+        <v>grocery,supermarket,mart,bigbasket,blinkit,zepto,dmart</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>53001</v>
+        <v>52002</v>
       </c>
       <c r="B33" t="str">
-        <v>Transport &amp; Fuel</v>
+        <v>Dining Out</v>
       </c>
       <c r="C33" t="str">
         <v>Expense</v>
       </c>
       <c r="D33" t="str">
-        <v>Transport</v>
+        <v>Food</v>
       </c>
       <c r="E33" t="str">
-        <v>Fuel / Taxi / Toll</v>
+        <v>Restaurants &amp; Delivery</v>
       </c>
       <c r="F33" t="str">
-        <v>uber,ola,rapido,petrol,fuel,hpcl,bpcl,fastag</v>
+        <v>swiggy,zomato,restaurant,hotel,cafe</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>53002</v>
+        <v>53001</v>
       </c>
       <c r="B34" t="str">
-        <v>Travel</v>
+        <v>Transport &amp; Fuel</v>
       </c>
       <c r="C34" t="str">
         <v>Expense</v>
@@ -2385,38 +2452,38 @@
         <v>Transport</v>
       </c>
       <c r="E34" t="str">
-        <v>Trips &amp; Tickets</v>
+        <v>Fuel / Taxi / Toll</v>
       </c>
       <c r="F34" t="str">
-        <v>irctc,makemytrip,redbus,indigo</v>
+        <v>uber,ola,rapido,petrol,fuel,hpcl,bpcl,fastag</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>54001</v>
+        <v>53002</v>
       </c>
       <c r="B35" t="str">
-        <v>Family Support</v>
+        <v>Travel</v>
       </c>
       <c r="C35" t="str">
         <v>Expense</v>
       </c>
       <c r="D35" t="str">
-        <v>Family &amp; Personal</v>
+        <v>Transport</v>
       </c>
       <c r="E35" t="str">
-        <v>Family / Amma</v>
+        <v>Trips &amp; Tickets</v>
       </c>
       <c r="F35" t="str">
-        <v>amma,family</v>
+        <v>irctc,makemytrip,redbus,indigo</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>54002</v>
+        <v>54001</v>
       </c>
       <c r="B36" t="str">
-        <v>Health &amp; Medical</v>
+        <v>Family Support</v>
       </c>
       <c r="C36" t="str">
         <v>Expense</v>
@@ -2425,18 +2492,18 @@
         <v>Family &amp; Personal</v>
       </c>
       <c r="E36" t="str">
-        <v>Pharmacy / Hospital</v>
+        <v>Family / Amma</v>
       </c>
       <c r="F36" t="str">
-        <v>pharmacy,medical,hospital,clinic</v>
+        <v>amma,family</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>54003</v>
+        <v>54002</v>
       </c>
       <c r="B37" t="str">
-        <v>Education</v>
+        <v>Health &amp; Medical</v>
       </c>
       <c r="C37" t="str">
         <v>Expense</v>
@@ -2445,18 +2512,18 @@
         <v>Family &amp; Personal</v>
       </c>
       <c r="E37" t="str">
-        <v>Fees &amp; Courses</v>
+        <v>Pharmacy / Hospital</v>
       </c>
       <c r="F37" t="str">
-        <v>school,college,course,tuition</v>
+        <v>pharmacy,medical,hospital,clinic</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>54004</v>
+        <v>54003</v>
       </c>
       <c r="B38" t="str">
-        <v>Shopping</v>
+        <v>Education</v>
       </c>
       <c r="C38" t="str">
         <v>Expense</v>
@@ -2465,18 +2532,18 @@
         <v>Family &amp; Personal</v>
       </c>
       <c r="E38" t="str">
-        <v>Online &amp; Retail</v>
+        <v>Fees &amp; Courses</v>
       </c>
       <c r="F38" t="str">
-        <v>amazon,flipkart,myntra,ajio</v>
+        <v>school,college,course,tuition</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>54005</v>
+        <v>54004</v>
       </c>
       <c r="B39" t="str">
-        <v>Gifts &amp; Functions</v>
+        <v>Shopping</v>
       </c>
       <c r="C39" t="str">
         <v>Expense</v>
@@ -2485,38 +2552,38 @@
         <v>Family &amp; Personal</v>
       </c>
       <c r="E39" t="str">
-        <v>Guests &amp; Gifts</v>
+        <v>Online &amp; Retail</v>
       </c>
       <c r="F39" t="str">
-        <v>guest,marriage,function</v>
+        <v>amazon,flipkart,myntra,ajio</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>55001</v>
+        <v>54005</v>
       </c>
       <c r="B40" t="str">
-        <v>Loan EMI / Repayment</v>
+        <v>Gifts &amp; Functions</v>
       </c>
       <c r="C40" t="str">
         <v>Expense</v>
       </c>
       <c r="D40" t="str">
-        <v>Financial</v>
+        <v>Family &amp; Personal</v>
       </c>
       <c r="E40" t="str">
-        <v>EMIs</v>
+        <v>Guests &amp; Gifts</v>
       </c>
       <c r="F40" t="str">
-        <v>emi,loan repay</v>
+        <v>guest,marriage,function</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>55002</v>
+        <v>55001</v>
       </c>
       <c r="B41" t="str">
-        <v>Credit Card Payment</v>
+        <v>Loan EMI / Repayment</v>
       </c>
       <c r="C41" t="str">
         <v>Expense</v>
@@ -2525,18 +2592,18 @@
         <v>Financial</v>
       </c>
       <c r="E41" t="str">
-        <v>Card Bills</v>
+        <v>EMIs</v>
       </c>
       <c r="F41" t="str">
-        <v>cc payment,card payment</v>
+        <v>emi,loan repay</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>55003</v>
+        <v>55002</v>
       </c>
       <c r="B42" t="str">
-        <v>Investment Contribution</v>
+        <v>Credit Card Payment</v>
       </c>
       <c r="C42" t="str">
         <v>Expense</v>
@@ -2545,18 +2612,18 @@
         <v>Financial</v>
       </c>
       <c r="E42" t="str">
-        <v>SIP / Deposits</v>
+        <v>Card Bills</v>
       </c>
       <c r="F42" t="str">
-        <v>sip</v>
+        <v>cc payment,card payment</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>55004</v>
+        <v>55003</v>
       </c>
       <c r="B43" t="str">
-        <v>Debt Given (Lent Out)</v>
+        <v>Investment Contribution</v>
       </c>
       <c r="C43" t="str">
         <v>Expense</v>
@@ -2565,18 +2632,18 @@
         <v>Financial</v>
       </c>
       <c r="E43" t="str">
-        <v>Money Lent</v>
+        <v>SIP / Deposits</v>
       </c>
       <c r="F43" t="str">
-        <v>lent to</v>
+        <v>sip</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>55005</v>
+        <v>55004</v>
       </c>
       <c r="B44" t="str">
-        <v>Taxes &amp; GST</v>
+        <v>Debt Given (Lent Out)</v>
       </c>
       <c r="C44" t="str">
         <v>Expense</v>
@@ -2585,18 +2652,18 @@
         <v>Financial</v>
       </c>
       <c r="E44" t="str">
-        <v>GST / Filing</v>
+        <v>Money Lent</v>
       </c>
       <c r="F44" t="str">
-        <v>gst,filing fee,tax</v>
+        <v>lent to</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>55006</v>
+        <v>55005</v>
       </c>
       <c r="B45" t="str">
-        <v>Insurance</v>
+        <v>Taxes &amp; GST</v>
       </c>
       <c r="C45" t="str">
         <v>Expense</v>
@@ -2605,55 +2672,75 @@
         <v>Financial</v>
       </c>
       <c r="E45" t="str">
-        <v>Premiums</v>
+        <v>GST / Filing</v>
       </c>
       <c r="F45" t="str">
-        <v>insurance,lic,premium</v>
+        <v>gst,filing fee,tax</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>55007</v>
+        <v>55006</v>
       </c>
       <c r="B46" t="str">
-        <v>Charges</v>
+        <v>Insurance</v>
       </c>
       <c r="C46" t="str">
         <v>Expense</v>
       </c>
       <c r="D46" t="str">
-        <v>Bank Charges</v>
+        <v>Financial</v>
       </c>
       <c r="E46" t="str">
-        <v/>
+        <v>Premiums</v>
       </c>
       <c r="F46" t="str">
-        <v/>
+        <v>insurance,lic,premium</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
+        <v>55007</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Charges</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Bank Charges</v>
+      </c>
+      <c r="E47" t="str">
+        <v/>
+      </c>
+      <c r="F47" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
         <v>59999</v>
       </c>
-      <c r="B47" t="str">
+      <c r="B48" t="str">
         <v>Other Expenses</v>
       </c>
-      <c r="C47" t="str">
-        <v>Expense</v>
-      </c>
-      <c r="D47" t="str">
+      <c r="C48" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D48" t="str">
         <v>Other</v>
       </c>
-      <c r="E47" t="str">
+      <c r="E48" t="str">
         <v>Miscellaneous</v>
       </c>
-      <c r="F47" t="str">
+      <c r="F48" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F47"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F48"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-19T21:24:12.910Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L36"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1683,9 +1683,47 @@
         <v/>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>TXN-1033</v>
+      </c>
+      <c r="B36" t="str">
+        <v>2026-07-23</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Journal</v>
+      </c>
+      <c r="D36" t="str">
+        <v>HDFC-Aluva Bank</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Savings</v>
+      </c>
+      <c r="F36">
+        <v>5000</v>
+      </c>
+      <c r="G36" t="str">
+        <v/>
+      </c>
+      <c r="H36" t="str">
+        <v>Bank Transfer</v>
+      </c>
+      <c r="I36" t="str">
+        <v/>
+      </c>
+      <c r="J36" t="str">
+        <v>11002</v>
+      </c>
+      <c r="K36" t="str">
+        <v>11001</v>
+      </c>
+      <c r="L36" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L36"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-19T21:33:09.743Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L37"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1721,9 +1721,47 @@
         <v/>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>TXN-1034</v>
+      </c>
+      <c r="B37" t="str">
+        <v>2026-07-16</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Transfer</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Transfer</v>
+      </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
+      <c r="F37">
+        <v>1000</v>
+      </c>
+      <c r="G37" t="str">
+        <v>HDFC- Aluva → HDFC- Info</v>
+      </c>
+      <c r="H37" t="str">
+        <v>Bank Transfer</v>
+      </c>
+      <c r="I37" t="str">
+        <v/>
+      </c>
+      <c r="J37" t="str">
+        <v/>
+      </c>
+      <c r="K37" t="str">
+        <v/>
+      </c>
+      <c r="L37" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L37"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1815,13 +1853,13 @@
         <v>6463</v>
       </c>
       <c r="F4">
-        <v>219562</v>
+        <v>220562</v>
       </c>
       <c r="G4">
         <v>160503.77</v>
       </c>
       <c r="H4">
-        <v>65521.23</v>
+        <v>66521.23</v>
       </c>
       <c r="I4" t="str">
         <v>2026-07-20</v>
@@ -1830,7 +1868,7 @@
         <v>140134.46</v>
       </c>
       <c r="K4">
-        <v>-74613.23</v>
+        <v>-73613.23</v>
       </c>
       <c r="L4" t="str">
         <v>Discrepancy</v>
@@ -1900,10 +1938,10 @@
         <v>20028</v>
       </c>
       <c r="G6">
-        <v>5891</v>
+        <v>6891</v>
       </c>
       <c r="H6">
-        <v>25215.46</v>
+        <v>24215.46</v>
       </c>
       <c r="I6" t="str">
         <v/>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-19T21:49:28.645Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -1768,7 +1768,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M6"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -1838,37 +1838,37 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ACC-02</v>
+        <v>ACC-03</v>
       </c>
       <c r="B4" t="str">
-        <v>HDFC- Info</v>
+        <v>Federal-Ang</v>
       </c>
       <c r="C4" t="str">
-        <v>50100465194051</v>
+        <v>10020100375530</v>
       </c>
       <c r="D4" t="str">
         <v>Savings</v>
       </c>
       <c r="E4">
-        <v>6463</v>
+        <v>18944</v>
       </c>
       <c r="F4">
-        <v>220562</v>
+        <v>48383</v>
       </c>
       <c r="G4">
-        <v>160503.77</v>
+        <v>35595.9</v>
       </c>
       <c r="H4">
-        <v>66521.23</v>
+        <v>31731.1</v>
       </c>
       <c r="I4" t="str">
         <v>2026-07-20</v>
       </c>
       <c r="J4">
-        <v>140134.46</v>
+        <v>30367.1</v>
       </c>
       <c r="K4">
-        <v>-73613.23</v>
+        <v>1364</v>
       </c>
       <c r="L4" t="str">
         <v>Discrepancy</v>
@@ -1879,40 +1879,40 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ACC-03</v>
+        <v>ACC-01</v>
       </c>
       <c r="B5" t="str">
-        <v>Federal-Ang</v>
+        <v>HDFC- Aluva</v>
       </c>
       <c r="C5" t="str">
-        <v>10020100375530</v>
+        <v>50100523900334</v>
       </c>
       <c r="D5" t="str">
         <v>Savings</v>
       </c>
       <c r="E5">
-        <v>18944</v>
+        <v>11078.46</v>
       </c>
       <c r="F5">
-        <v>48383</v>
+        <v>20028</v>
       </c>
       <c r="G5">
-        <v>35595.9</v>
+        <v>6891</v>
       </c>
       <c r="H5">
-        <v>31731.1</v>
+        <v>24215.46</v>
       </c>
       <c r="I5" t="str">
-        <v>2026-07-20</v>
-      </c>
-      <c r="J5">
-        <v>30367.1</v>
-      </c>
-      <c r="K5">
-        <v>1364</v>
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
       </c>
       <c r="L5" t="str">
-        <v>Discrepancy</v>
+        <v>Pending</v>
       </c>
       <c r="M5" t="str">
         <v/>
@@ -1920,28 +1920,28 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ACC-01</v>
+        <v>ACC-04</v>
       </c>
       <c r="B6" t="str">
-        <v>HDFC- Aluva</v>
+        <v>SBI</v>
       </c>
       <c r="C6" t="str">
-        <v>50100523900334</v>
+        <v>43602594069</v>
       </c>
       <c r="D6" t="str">
         <v>Savings</v>
       </c>
       <c r="E6">
-        <v>11078.46</v>
+        <v>84324.2</v>
       </c>
       <c r="F6">
-        <v>20028</v>
+        <v>50000</v>
       </c>
       <c r="G6">
-        <v>6891</v>
+        <v>78700</v>
       </c>
       <c r="H6">
-        <v>24215.46</v>
+        <v>55624.2</v>
       </c>
       <c r="I6" t="str">
         <v/>
@@ -1959,50 +1959,9 @@
         <v/>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>ACC-04</v>
-      </c>
-      <c r="B7" t="str">
-        <v>SBI</v>
-      </c>
-      <c r="C7" t="str">
-        <v>43602594069</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Savings</v>
-      </c>
-      <c r="E7">
-        <v>84324.2</v>
-      </c>
-      <c r="F7">
-        <v>50000</v>
-      </c>
-      <c r="G7">
-        <v>78700</v>
-      </c>
-      <c r="H7">
-        <v>55624.2</v>
-      </c>
-      <c r="I7" t="str">
-        <v/>
-      </c>
-      <c r="J7" t="str">
-        <v/>
-      </c>
-      <c r="K7" t="str">
-        <v/>
-      </c>
-      <c r="L7" t="str">
-        <v>Pending</v>
-      </c>
-      <c r="M7" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M6"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-19T21:50:11.734Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -1768,7 +1768,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M7"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -1959,9 +1959,50 @@
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>ACC-02</v>
+      </c>
+      <c r="B7" t="str">
+        <v>HDFC- Info</v>
+      </c>
+      <c r="C7" t="str">
+        <v>50100465194051</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Savings</v>
+      </c>
+      <c r="E7">
+        <v>6463</v>
+      </c>
+      <c r="F7">
+        <v>220562</v>
+      </c>
+      <c r="G7">
+        <v>165503.77</v>
+      </c>
+      <c r="H7">
+        <v>61521.23</v>
+      </c>
+      <c r="I7" t="str">
+        <v>2026-07-20</v>
+      </c>
+      <c r="J7">
+        <v>140134.46</v>
+      </c>
+      <c r="K7">
+        <v>-78613.23</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Discrepancy</v>
+      </c>
+      <c r="M7" t="str">
+        <v>11001</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M7"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-19T22:04:23.301Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -1768,7 +1768,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M6"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -1959,50 +1959,9 @@
         <v/>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>ACC-02</v>
-      </c>
-      <c r="B7" t="str">
-        <v>HDFC- Info</v>
-      </c>
-      <c r="C7" t="str">
-        <v>50100465194051</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Savings</v>
-      </c>
-      <c r="E7">
-        <v>6463</v>
-      </c>
-      <c r="F7">
-        <v>220562</v>
-      </c>
-      <c r="G7">
-        <v>165503.77</v>
-      </c>
-      <c r="H7">
-        <v>61521.23</v>
-      </c>
-      <c r="I7" t="str">
-        <v>2026-07-20</v>
-      </c>
-      <c r="J7">
-        <v>140134.46</v>
-      </c>
-      <c r="K7">
-        <v>-78613.23</v>
-      </c>
-      <c r="L7" t="str">
-        <v>Discrepancy</v>
-      </c>
-      <c r="M7" t="str">
-        <v>11001</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M6"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-19T22:04:33.976Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -1768,7 +1768,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M7"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -1959,9 +1959,50 @@
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>ACC-02</v>
+      </c>
+      <c r="B7" t="str">
+        <v>HDFC- Info</v>
+      </c>
+      <c r="C7" t="str">
+        <v>50100465194051</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Savings</v>
+      </c>
+      <c r="E7">
+        <v>6463</v>
+      </c>
+      <c r="F7">
+        <v>220562</v>
+      </c>
+      <c r="G7">
+        <v>165503.77</v>
+      </c>
+      <c r="H7">
+        <v>61521.23</v>
+      </c>
+      <c r="I7" t="str">
+        <v>2026-07-20</v>
+      </c>
+      <c r="J7">
+        <v>140134.46</v>
+      </c>
+      <c r="K7">
+        <v>-78613.23</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Discrepancy</v>
+      </c>
+      <c r="M7" t="str">
+        <v>11001</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M7"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-19T22:05:29.119Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -1920,84 +1920,84 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ACC-04</v>
+        <v>ACC-02</v>
       </c>
       <c r="B6" t="str">
-        <v>SBI</v>
+        <v>HDFC- Info</v>
       </c>
       <c r="C6" t="str">
-        <v>43602594069</v>
+        <v>50100465194051</v>
       </c>
       <c r="D6" t="str">
         <v>Savings</v>
       </c>
       <c r="E6">
-        <v>84324.2</v>
+        <v>6463</v>
       </c>
       <c r="F6">
-        <v>50000</v>
+        <v>220562</v>
       </c>
       <c r="G6">
-        <v>78700</v>
+        <v>165503.77</v>
       </c>
       <c r="H6">
-        <v>55624.2</v>
+        <v>61521.23</v>
       </c>
       <c r="I6" t="str">
-        <v/>
-      </c>
-      <c r="J6" t="str">
-        <v/>
-      </c>
-      <c r="K6" t="str">
-        <v/>
+        <v>2026-07-20</v>
+      </c>
+      <c r="J6">
+        <v>140134.46</v>
+      </c>
+      <c r="K6">
+        <v>-78613.23</v>
       </c>
       <c r="L6" t="str">
-        <v>Pending</v>
+        <v>Discrepancy</v>
       </c>
       <c r="M6" t="str">
-        <v/>
+        <v>11001</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ACC-02</v>
+        <v>ACC-04</v>
       </c>
       <c r="B7" t="str">
-        <v>HDFC- Info</v>
+        <v>SBI</v>
       </c>
       <c r="C7" t="str">
-        <v>50100465194051</v>
+        <v>43602594069</v>
       </c>
       <c r="D7" t="str">
         <v>Savings</v>
       </c>
       <c r="E7">
-        <v>6463</v>
+        <v>84324.2</v>
       </c>
       <c r="F7">
-        <v>220562</v>
+        <v>55000</v>
       </c>
       <c r="G7">
-        <v>165503.77</v>
+        <v>78700</v>
       </c>
       <c r="H7">
-        <v>61521.23</v>
+        <v>60624.2</v>
       </c>
       <c r="I7" t="str">
-        <v>2026-07-20</v>
-      </c>
-      <c r="J7">
-        <v>140134.46</v>
-      </c>
-      <c r="K7">
-        <v>-78613.23</v>
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v/>
       </c>
       <c r="L7" t="str">
-        <v>Discrepancy</v>
+        <v>Pending</v>
       </c>
       <c r="M7" t="str">
-        <v>11001</v>
+        <v>11002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-19T22:08:12.944Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -1838,40 +1838,40 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ACC-03</v>
+        <v>ACC-01</v>
       </c>
       <c r="B4" t="str">
-        <v>Federal-Ang</v>
+        <v>HDFC- Aluva</v>
       </c>
       <c r="C4" t="str">
-        <v>10020100375530</v>
+        <v>50100523900334</v>
       </c>
       <c r="D4" t="str">
         <v>Savings</v>
       </c>
       <c r="E4">
-        <v>18944</v>
+        <v>11078.46</v>
       </c>
       <c r="F4">
-        <v>48383</v>
+        <v>20028</v>
       </c>
       <c r="G4">
-        <v>35595.9</v>
+        <v>6891</v>
       </c>
       <c r="H4">
-        <v>31731.1</v>
+        <v>24215.46</v>
       </c>
       <c r="I4" t="str">
-        <v>2026-07-20</v>
-      </c>
-      <c r="J4">
-        <v>30367.1</v>
-      </c>
-      <c r="K4">
-        <v>1364</v>
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
       </c>
       <c r="L4" t="str">
-        <v>Discrepancy</v>
+        <v>Pending</v>
       </c>
       <c r="M4" t="str">
         <v/>
@@ -1879,125 +1879,125 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ACC-01</v>
+        <v>ACC-02</v>
       </c>
       <c r="B5" t="str">
-        <v>HDFC- Aluva</v>
+        <v>HDFC- Info</v>
       </c>
       <c r="C5" t="str">
-        <v>50100523900334</v>
+        <v>50100465194051</v>
       </c>
       <c r="D5" t="str">
         <v>Savings</v>
       </c>
       <c r="E5">
-        <v>11078.46</v>
+        <v>6463</v>
       </c>
       <c r="F5">
-        <v>20028</v>
+        <v>220562</v>
       </c>
       <c r="G5">
-        <v>6891</v>
+        <v>165503.77</v>
       </c>
       <c r="H5">
-        <v>24215.46</v>
+        <v>61521.23</v>
       </c>
       <c r="I5" t="str">
-        <v/>
-      </c>
-      <c r="J5" t="str">
-        <v/>
-      </c>
-      <c r="K5" t="str">
-        <v/>
+        <v>2026-07-20</v>
+      </c>
+      <c r="J5">
+        <v>140134.46</v>
+      </c>
+      <c r="K5">
+        <v>-78613.23</v>
       </c>
       <c r="L5" t="str">
-        <v>Pending</v>
+        <v>Discrepancy</v>
       </c>
       <c r="M5" t="str">
-        <v/>
+        <v>11001</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ACC-02</v>
+        <v>ACC-04</v>
       </c>
       <c r="B6" t="str">
-        <v>HDFC- Info</v>
+        <v>SBI</v>
       </c>
       <c r="C6" t="str">
-        <v>50100465194051</v>
+        <v>43602594069</v>
       </c>
       <c r="D6" t="str">
         <v>Savings</v>
       </c>
       <c r="E6">
-        <v>6463</v>
+        <v>84324.2</v>
       </c>
       <c r="F6">
-        <v>220562</v>
+        <v>55000</v>
       </c>
       <c r="G6">
-        <v>165503.77</v>
+        <v>78700</v>
       </c>
       <c r="H6">
-        <v>61521.23</v>
+        <v>60624.2</v>
       </c>
       <c r="I6" t="str">
-        <v>2026-07-20</v>
-      </c>
-      <c r="J6">
-        <v>140134.46</v>
-      </c>
-      <c r="K6">
-        <v>-78613.23</v>
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v/>
       </c>
       <c r="L6" t="str">
-        <v>Discrepancy</v>
+        <v>Pending</v>
       </c>
       <c r="M6" t="str">
-        <v>11001</v>
+        <v>11002</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ACC-04</v>
+        <v>ACC-03</v>
       </c>
       <c r="B7" t="str">
-        <v>SBI</v>
+        <v>Federal-Ang</v>
       </c>
       <c r="C7" t="str">
-        <v>43602594069</v>
+        <v>10020100375530</v>
       </c>
       <c r="D7" t="str">
         <v>Savings</v>
       </c>
       <c r="E7">
-        <v>84324.2</v>
+        <v>18944</v>
       </c>
       <c r="F7">
-        <v>55000</v>
+        <v>48383</v>
       </c>
       <c r="G7">
-        <v>78700</v>
+        <v>35595.9</v>
       </c>
       <c r="H7">
-        <v>60624.2</v>
+        <v>31731.1</v>
       </c>
       <c r="I7" t="str">
-        <v/>
-      </c>
-      <c r="J7" t="str">
-        <v/>
-      </c>
-      <c r="K7" t="str">
-        <v/>
+        <v>2026-07-20</v>
+      </c>
+      <c r="J7">
+        <v>30367.1</v>
+      </c>
+      <c r="K7">
+        <v>1364</v>
       </c>
       <c r="L7" t="str">
-        <v>Pending</v>
+        <v>Discrepancy</v>
       </c>
       <c r="M7" t="str">
-        <v>11002</v>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-19T23:02:17.534Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -1862,37 +1862,37 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ACC-02</v>
+        <v>ACC-03</v>
       </c>
       <c r="B4" t="str">
-        <v>HDFC- Info</v>
+        <v>Federal-Ang</v>
       </c>
       <c r="C4" t="str">
-        <v>50100465194051</v>
+        <v>10020100375530</v>
       </c>
       <c r="D4" t="str">
         <v>Savings</v>
       </c>
       <c r="E4">
-        <v>6463</v>
+        <v>18944</v>
       </c>
       <c r="F4">
-        <v>219562</v>
+        <v>48383</v>
       </c>
       <c r="G4">
-        <v>160503.77</v>
+        <v>35595.9</v>
       </c>
       <c r="H4">
-        <v>65521.23</v>
+        <v>31731.1</v>
       </c>
       <c r="I4" t="str">
         <v>2026-07-20</v>
       </c>
       <c r="J4">
-        <v>140134.46</v>
+        <v>30367.1</v>
       </c>
       <c r="K4">
-        <v>-74613.23</v>
+        <v>1364</v>
       </c>
       <c r="L4" t="str">
         <v>Discrepancy</v>
@@ -1903,40 +1903,40 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ACC-03</v>
+        <v>ACC-01</v>
       </c>
       <c r="B5" t="str">
-        <v>Federal-Ang</v>
+        <v>HDFC- Aluva</v>
       </c>
       <c r="C5" t="str">
-        <v>10020100375530</v>
+        <v>50100523900334</v>
       </c>
       <c r="D5" t="str">
         <v>Savings</v>
       </c>
       <c r="E5">
-        <v>18944</v>
+        <v>11078.46</v>
       </c>
       <c r="F5">
-        <v>48383</v>
+        <v>20028</v>
       </c>
       <c r="G5">
-        <v>35595.9</v>
+        <v>5891</v>
       </c>
       <c r="H5">
-        <v>31731.1</v>
+        <v>25215.46</v>
       </c>
       <c r="I5" t="str">
-        <v>2026-07-20</v>
-      </c>
-      <c r="J5">
-        <v>30367.1</v>
-      </c>
-      <c r="K5">
-        <v>1364</v>
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
       </c>
       <c r="L5" t="str">
-        <v>Discrepancy</v>
+        <v>Pending</v>
       </c>
       <c r="M5" t="str">
         <v/>
@@ -1944,28 +1944,28 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ACC-01</v>
+        <v>ACC-04</v>
       </c>
       <c r="B6" t="str">
-        <v>HDFC- Aluva</v>
+        <v>SBI</v>
       </c>
       <c r="C6" t="str">
-        <v>50100523900334</v>
+        <v>43602594069</v>
       </c>
       <c r="D6" t="str">
         <v>Savings</v>
       </c>
       <c r="E6">
-        <v>11078.46</v>
+        <v>84324.2</v>
       </c>
       <c r="F6">
-        <v>20028</v>
+        <v>50000</v>
       </c>
       <c r="G6">
-        <v>5891</v>
+        <v>78700</v>
       </c>
       <c r="H6">
-        <v>25215.46</v>
+        <v>55624.2</v>
       </c>
       <c r="I6" t="str">
         <v/>
@@ -1985,43 +1985,43 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ACC-04</v>
+        <v>ACC-02</v>
       </c>
       <c r="B7" t="str">
-        <v>SBI</v>
+        <v>HDFC- Info</v>
       </c>
       <c r="C7" t="str">
-        <v>43602594069</v>
+        <v>50100465194051</v>
       </c>
       <c r="D7" t="str">
         <v>Savings</v>
       </c>
       <c r="E7">
-        <v>84324.2</v>
+        <v>6463</v>
       </c>
       <c r="F7">
-        <v>50000</v>
+        <v>219562</v>
       </c>
       <c r="G7">
-        <v>78700</v>
+        <v>160503.77</v>
       </c>
       <c r="H7">
-        <v>55624.2</v>
+        <v>65521.23</v>
       </c>
       <c r="I7" t="str">
-        <v/>
-      </c>
-      <c r="J7" t="str">
-        <v/>
-      </c>
-      <c r="K7" t="str">
-        <v/>
+        <v>2026-07-20</v>
+      </c>
+      <c r="J7">
+        <v>140134.46</v>
+      </c>
+      <c r="K7">
+        <v>-74613.23</v>
       </c>
       <c r="L7" t="str">
-        <v>Pending</v>
+        <v>Discrepancy</v>
       </c>
       <c r="M7" t="str">
-        <v/>
+        <v>11001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-19T23:13:22.330Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -1862,40 +1862,40 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ACC-03</v>
+        <v>ACC-01</v>
       </c>
       <c r="B4" t="str">
-        <v>Federal-Ang</v>
+        <v>HDFC- Aluva</v>
       </c>
       <c r="C4" t="str">
-        <v>10020100375530</v>
+        <v>50100523900334</v>
       </c>
       <c r="D4" t="str">
         <v>Savings</v>
       </c>
       <c r="E4">
-        <v>18944</v>
+        <v>11078.46</v>
       </c>
       <c r="F4">
-        <v>48383</v>
+        <v>20028</v>
       </c>
       <c r="G4">
-        <v>35595.9</v>
+        <v>5891</v>
       </c>
       <c r="H4">
-        <v>31731.1</v>
+        <v>25215.46</v>
       </c>
       <c r="I4" t="str">
-        <v>2026-07-20</v>
-      </c>
-      <c r="J4">
-        <v>30367.1</v>
-      </c>
-      <c r="K4">
-        <v>1364</v>
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
       </c>
       <c r="L4" t="str">
-        <v>Discrepancy</v>
+        <v>Pending</v>
       </c>
       <c r="M4" t="str">
         <v/>
@@ -1903,28 +1903,28 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ACC-01</v>
+        <v>ACC-04</v>
       </c>
       <c r="B5" t="str">
-        <v>HDFC- Aluva</v>
+        <v>SBI</v>
       </c>
       <c r="C5" t="str">
-        <v>50100523900334</v>
+        <v>43602594069</v>
       </c>
       <c r="D5" t="str">
         <v>Savings</v>
       </c>
       <c r="E5">
-        <v>11078.46</v>
+        <v>84324.2</v>
       </c>
       <c r="F5">
-        <v>20028</v>
+        <v>50000</v>
       </c>
       <c r="G5">
-        <v>5891</v>
+        <v>78700</v>
       </c>
       <c r="H5">
-        <v>25215.46</v>
+        <v>55624.2</v>
       </c>
       <c r="I5" t="str">
         <v/>
@@ -1944,84 +1944,84 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ACC-04</v>
+        <v>ACC-02</v>
       </c>
       <c r="B6" t="str">
-        <v>SBI</v>
+        <v>HDFC- Info</v>
       </c>
       <c r="C6" t="str">
-        <v>43602594069</v>
+        <v>50100465194051</v>
       </c>
       <c r="D6" t="str">
         <v>Savings</v>
       </c>
       <c r="E6">
-        <v>84324.2</v>
+        <v>6463</v>
       </c>
       <c r="F6">
-        <v>50000</v>
+        <v>219562</v>
       </c>
       <c r="G6">
-        <v>78700</v>
+        <v>160503.77</v>
       </c>
       <c r="H6">
-        <v>55624.2</v>
+        <v>65521.23</v>
       </c>
       <c r="I6" t="str">
-        <v/>
-      </c>
-      <c r="J6" t="str">
-        <v/>
-      </c>
-      <c r="K6" t="str">
-        <v/>
+        <v>2026-07-20</v>
+      </c>
+      <c r="J6">
+        <v>140134.46</v>
+      </c>
+      <c r="K6">
+        <v>-74613.23</v>
       </c>
       <c r="L6" t="str">
-        <v>Pending</v>
+        <v>Discrepancy</v>
       </c>
       <c r="M6" t="str">
-        <v/>
+        <v>11001</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ACC-02</v>
+        <v>ACC-03</v>
       </c>
       <c r="B7" t="str">
-        <v>HDFC- Info</v>
+        <v>Federal-Ang</v>
       </c>
       <c r="C7" t="str">
-        <v>50100465194051</v>
+        <v>10020100375530</v>
       </c>
       <c r="D7" t="str">
         <v>Savings</v>
       </c>
       <c r="E7">
-        <v>6463</v>
+        <v>18944</v>
       </c>
       <c r="F7">
-        <v>219562</v>
+        <v>48383</v>
       </c>
       <c r="G7">
-        <v>160503.77</v>
+        <v>35595.9</v>
       </c>
       <c r="H7">
-        <v>65521.23</v>
+        <v>31731.1</v>
       </c>
       <c r="I7" t="str">
         <v>2026-07-20</v>
       </c>
       <c r="J7">
-        <v>140134.46</v>
+        <v>30367.1</v>
       </c>
       <c r="K7">
-        <v>-74613.23</v>
+        <v>1364</v>
       </c>
       <c r="L7" t="str">
         <v>Discrepancy</v>
       </c>
       <c r="M7" t="str">
-        <v>11001</v>
+        <v>11002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-19T23:14:13.944Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M35"/>
+  <dimension ref="A1:M36"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1783,9 +1783,50 @@
         <v/>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>TXN-1033</v>
+      </c>
+      <c r="B36" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D36" t="str">
+        <v>HDFC-Info Bank</v>
+      </c>
+      <c r="E36" t="str">
+        <v>test vouhcer postings</v>
+      </c>
+      <c r="F36">
+        <v>300</v>
+      </c>
+      <c r="G36" t="str">
+        <v/>
+      </c>
+      <c r="H36" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="I36" t="str">
+        <v/>
+      </c>
+      <c r="J36" t="str">
+        <v/>
+      </c>
+      <c r="K36" t="str">
+        <v/>
+      </c>
+      <c r="L36" t="str">
+        <v>[{"kind":"Bank","acct":"11001","sub":"bank:HDFC- Info","dr":0,"cr":300},{"kind":"Ledger","acct":"52001","sub":"","dr":300,"cr":0}]</v>
+      </c>
+      <c r="M36" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M36"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1962,10 +2003,10 @@
         <v>219562</v>
       </c>
       <c r="G6">
-        <v>160503.77</v>
+        <v>160803.77</v>
       </c>
       <c r="H6">
-        <v>65521.23</v>
+        <v>65221.23</v>
       </c>
       <c r="I6" t="str">
         <v>2026-07-20</v>
@@ -1974,7 +2015,7 @@
         <v>140134.46</v>
       </c>
       <c r="K6">
-        <v>-74613.23</v>
+        <v>-74913.23</v>
       </c>
       <c r="L6" t="str">
         <v>Discrepancy</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-19T23:14:46.794Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:M37"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1824,9 +1824,50 @@
         <v/>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>TXN-1034</v>
+      </c>
+      <c r="B37" t="str">
+        <v>2026-08-19</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D37" t="str">
+        <v>HDFC-Info Bank</v>
+      </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
+      <c r="F37">
+        <v>400</v>
+      </c>
+      <c r="G37" t="str">
+        <v/>
+      </c>
+      <c r="H37" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="I37" t="str">
+        <v/>
+      </c>
+      <c r="J37" t="str">
+        <v/>
+      </c>
+      <c r="K37" t="str">
+        <v/>
+      </c>
+      <c r="L37" t="str">
+        <v>[{"kind":"Bank","acct":"11001","sub":"bank:HDFC- Info","dr":0,"cr":400},{"kind":"Ledger","acct":"55001","sub":"","dr":400,"cr":0}]</v>
+      </c>
+      <c r="M37" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M37"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2003,10 +2044,10 @@
         <v>219562</v>
       </c>
       <c r="G6">
-        <v>160803.77</v>
+        <v>161203.77</v>
       </c>
       <c r="H6">
-        <v>65221.23</v>
+        <v>64821.23</v>
       </c>
       <c r="I6" t="str">
         <v>2026-07-20</v>
@@ -2015,7 +2056,7 @@
         <v>140134.46</v>
       </c>
       <c r="K6">
-        <v>-74913.23</v>
+        <v>-75313.23</v>
       </c>
       <c r="L6" t="str">
         <v>Discrepancy</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-19T23:33:25.035Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M37"/>
+  <dimension ref="A1:M38"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1865,9 +1865,50 @@
         <v/>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>TXN-1035</v>
+      </c>
+      <c r="B38" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Federal-Ang Bank</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Testing</v>
+      </c>
+      <c r="F38">
+        <v>120</v>
+      </c>
+      <c r="G38" t="str">
+        <v/>
+      </c>
+      <c r="H38" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="I38" t="str">
+        <v/>
+      </c>
+      <c r="J38" t="str">
+        <v/>
+      </c>
+      <c r="K38" t="str">
+        <v/>
+      </c>
+      <c r="L38" t="str">
+        <v>[{"kind":"Bank","acct":"11003","sub":"bank:HDFC- Aluva","dr":0,"cr":120},{"kind":"Ledger","acct":"52001","sub":"","dr":120,"cr":0}]</v>
+      </c>
+      <c r="M38" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M38"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1962,10 +2003,10 @@
         <v>20028</v>
       </c>
       <c r="G4">
-        <v>5891</v>
+        <v>6011</v>
       </c>
       <c r="H4">
-        <v>25215.46</v>
+        <v>25095.46</v>
       </c>
       <c r="I4" t="str">
         <v/>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-19T23:34:07.140Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -1876,7 +1876,7 @@
         <v>Voucher</v>
       </c>
       <c r="D38" t="str">
-        <v>Federal-Ang Bank</v>
+        <v>HDFC-Info Bank</v>
       </c>
       <c r="E38" t="str">
         <v>Testing</v>
@@ -1900,7 +1900,7 @@
         <v/>
       </c>
       <c r="L38" t="str">
-        <v>[{"kind":"Bank","acct":"11003","sub":"bank:HDFC- Aluva","dr":0,"cr":120},{"kind":"Ledger","acct":"52001","sub":"","dr":120,"cr":0}]</v>
+        <v>[{"kind":"Bank","acct":"11001","sub":"bank:HDFC- Info","dr":0,"cr":120},{"kind":"Ledger","acct":"52001","sub":"","dr":120,"cr":0}]</v>
       </c>
       <c r="M38" t="str">
         <v/>
@@ -2003,10 +2003,10 @@
         <v>20028</v>
       </c>
       <c r="G4">
-        <v>6011</v>
+        <v>5891</v>
       </c>
       <c r="H4">
-        <v>25095.46</v>
+        <v>25215.46</v>
       </c>
       <c r="I4" t="str">
         <v/>
@@ -2085,10 +2085,10 @@
         <v>219562</v>
       </c>
       <c r="G6">
-        <v>161203.77</v>
+        <v>161323.77</v>
       </c>
       <c r="H6">
-        <v>64821.23</v>
+        <v>64701.23</v>
       </c>
       <c r="I6" t="str">
         <v>2026-07-20</v>
@@ -2097,7 +2097,7 @@
         <v>140134.46</v>
       </c>
       <c r="K6">
-        <v>-75313.23</v>
+        <v>-75433.23</v>
       </c>
       <c r="L6" t="str">
         <v>Discrepancy</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-19T23:35:21.057Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M38"/>
+  <dimension ref="A1:M39"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1906,9 +1906,50 @@
         <v/>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>TXN-1036</v>
+      </c>
+      <c r="B39" t="str">
+        <v>2026-08-19</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D39" t="str">
+        <v>APY Pension</v>
+      </c>
+      <c r="E39" t="str">
+        <v/>
+      </c>
+      <c r="F39">
+        <v>409</v>
+      </c>
+      <c r="G39" t="str">
+        <v/>
+      </c>
+      <c r="H39" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="I39" t="str">
+        <v/>
+      </c>
+      <c r="J39" t="str">
+        <v/>
+      </c>
+      <c r="K39" t="str">
+        <v/>
+      </c>
+      <c r="L39" t="str">
+        <v>[{"kind":"Investment","acct":"12001","sub":"inv:INV-04","dr":409,"cr":0},{"kind":"Bank","acct":"11002","sub":"bank:Federal-Ang","dr":0,"cr":409}]</v>
+      </c>
+      <c r="M39" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M39"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2126,10 +2167,10 @@
         <v>48383</v>
       </c>
       <c r="G7">
-        <v>35595.9</v>
+        <v>36004.9</v>
       </c>
       <c r="H7">
-        <v>31731.1</v>
+        <v>31322.1</v>
       </c>
       <c r="I7" t="str">
         <v>2026-07-20</v>
@@ -2138,7 +2179,7 @@
         <v>30367.1</v>
       </c>
       <c r="K7">
-        <v>1364</v>
+        <v>955</v>
       </c>
       <c r="L7" t="str">
         <v>Discrepancy</v>
@@ -2618,10 +2659,10 @@
         <v>2026-07-01</v>
       </c>
       <c r="E4">
-        <v>409</v>
+        <v>818</v>
       </c>
       <c r="F4">
-        <v>409</v>
+        <v>818</v>
       </c>
       <c r="G4">
         <v>0</v>
@@ -2642,7 +2683,7 @@
         <v/>
       </c>
       <c r="M4" t="str">
-        <v/>
+        <v>12001</v>
       </c>
       <c r="N4" t="str">
         <v/>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-19T23:41:26.811Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M39"/>
+  <dimension ref="A1:M40"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1947,9 +1947,50 @@
         <v/>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>TXN-1037</v>
+      </c>
+      <c r="B40" t="str">
+        <v>2026-08-06</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D40" t="str">
+        <v>APY Pension</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Test</v>
+      </c>
+      <c r="F40">
+        <v>409</v>
+      </c>
+      <c r="G40" t="str">
+        <v/>
+      </c>
+      <c r="H40" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="I40" t="str">
+        <v/>
+      </c>
+      <c r="J40" t="str">
+        <v/>
+      </c>
+      <c r="K40" t="str">
+        <v/>
+      </c>
+      <c r="L40" t="str">
+        <v>[{"kind":"Investment","acct":"12001","sub":"inv:INV-04","dr":409,"cr":0},{"kind":"Bank","acct":"11002","sub":"bank:Federal-Ang","dr":0,"cr":409}]</v>
+      </c>
+      <c r="M40" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M39"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M40"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2167,10 +2208,10 @@
         <v>48383</v>
       </c>
       <c r="G7">
-        <v>36004.9</v>
+        <v>36413.9</v>
       </c>
       <c r="H7">
-        <v>31322.1</v>
+        <v>30913.1</v>
       </c>
       <c r="I7" t="str">
         <v>2026-07-20</v>
@@ -2179,7 +2220,7 @@
         <v>30367.1</v>
       </c>
       <c r="K7">
-        <v>955</v>
+        <v>546</v>
       </c>
       <c r="L7" t="str">
         <v>Discrepancy</v>
@@ -2659,10 +2700,10 @@
         <v>2026-07-01</v>
       </c>
       <c r="E4">
-        <v>818</v>
+        <v>1227</v>
       </c>
       <c r="F4">
-        <v>818</v>
+        <v>1227</v>
       </c>
       <c r="G4">
         <v>0</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-19T23:47:32.724Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M40"/>
+  <dimension ref="A1:M41"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1988,9 +1988,50 @@
         <v/>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>TXN-1038</v>
+      </c>
+      <c r="B41" t="str">
+        <v>2026-08-19</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D41" t="str">
+        <v>(new)</v>
+      </c>
+      <c r="E41" t="str">
+        <v/>
+      </c>
+      <c r="F41">
+        <v>450</v>
+      </c>
+      <c r="G41" t="str">
+        <v/>
+      </c>
+      <c r="H41" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="I41" t="str">
+        <v/>
+      </c>
+      <c r="J41" t="str">
+        <v/>
+      </c>
+      <c r="K41" t="str">
+        <v/>
+      </c>
+      <c r="L41" t="str">
+        <v>[{"kind":"Loan","acct":"(new)","sub":"ld:DEBT-08","dr":0,"cr":400},{"kind":"Bank","acct":"11002","sub":"bank:Federal-Ang","dr":450,"cr":0},{"kind":"Ledger","acct":"55002","sub":"","dr":0,"cr":50}]</v>
+      </c>
+      <c r="M41" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M40"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M41"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2205,13 +2246,13 @@
         <v>18944</v>
       </c>
       <c r="F7">
-        <v>48383</v>
+        <v>48833</v>
       </c>
       <c r="G7">
         <v>36413.9</v>
       </c>
       <c r="H7">
-        <v>30913.1</v>
+        <v>31363.1</v>
       </c>
       <c r="I7" t="str">
         <v>2026-07-20</v>
@@ -2220,7 +2261,7 @@
         <v>30367.1</v>
       </c>
       <c r="K7">
-        <v>546</v>
+        <v>996</v>
       </c>
       <c r="L7" t="str">
         <v>Discrepancy</v>
@@ -2238,7 +2279,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R8"/>
+  <dimension ref="A1:R9"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -2605,9 +2646,65 @@
         <v/>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>DEBT-08</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Debt Payable</v>
+      </c>
+      <c r="C9" t="str">
+        <v>From voucher</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Posted 2026-08-19</v>
+      </c>
+      <c r="E9">
+        <v>400</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>400</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>400</v>
+      </c>
+      <c r="L9" t="str">
+        <v>2026-08-19</v>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
+        <v>Open</v>
+      </c>
+      <c r="O9" t="str">
+        <v/>
+      </c>
+      <c r="P9" t="str">
+        <v/>
+      </c>
+      <c r="Q9" t="str">
+        <v>TXN-1038</v>
+      </c>
+      <c r="R9" t="str">
+        <v>(new)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R9"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-19T23:49:19.485Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M41"/>
+  <dimension ref="A1:M42"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2029,9 +2029,50 @@
         <v/>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>TXN-1039</v>
+      </c>
+      <c r="B42" t="str">
+        <v>2026-08-19</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Debt Repayment</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Repaid From voucher</v>
+      </c>
+      <c r="F42">
+        <v>400</v>
+      </c>
+      <c r="G42" t="str">
+        <v>HDFC- Info</v>
+      </c>
+      <c r="H42" t="str">
+        <v/>
+      </c>
+      <c r="I42" t="str">
+        <v>Auto-Posted: DEBT-08 (From voucher)</v>
+      </c>
+      <c r="J42" t="str">
+        <v/>
+      </c>
+      <c r="K42" t="str">
+        <v/>
+      </c>
+      <c r="L42" t="str">
+        <v/>
+      </c>
+      <c r="M42" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M42"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2208,10 +2249,10 @@
         <v>219562</v>
       </c>
       <c r="G6">
-        <v>161323.77</v>
+        <v>161723.77</v>
       </c>
       <c r="H6">
-        <v>64701.23</v>
+        <v>64301.23</v>
       </c>
       <c r="I6" t="str">
         <v>2026-07-20</v>
@@ -2220,7 +2261,7 @@
         <v>140134.46</v>
       </c>
       <c r="K6">
-        <v>-75433.23</v>
+        <v>-75833.23</v>
       </c>
       <c r="L6" t="str">
         <v>Discrepancy</v>
@@ -2675,10 +2716,10 @@
         <v>400</v>
       </c>
       <c r="J9">
+        <v>400</v>
+      </c>
+      <c r="K9">
         <v>0</v>
-      </c>
-      <c r="K9">
-        <v>400</v>
       </c>
       <c r="L9" t="str">
         <v>2026-08-19</v>
@@ -2687,16 +2728,16 @@
         <v/>
       </c>
       <c r="N9" t="str">
-        <v>Open</v>
+        <v>Closed</v>
       </c>
       <c r="O9" t="str">
-        <v/>
+        <v>2026-08-19</v>
       </c>
       <c r="P9" t="str">
-        <v/>
+        <v>HDFC- Info</v>
       </c>
       <c r="Q9" t="str">
-        <v>TXN-1038</v>
+        <v>TXN-1039</v>
       </c>
       <c r="R9" t="str">
         <v>(new)</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-19T23:51:02.665Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -2412,16 +2412,16 @@
         <v>LOAN-01</v>
       </c>
       <c r="B4" t="str">
-        <v>Bank Loan Payable</v>
+        <v>Debt Payable</v>
       </c>
       <c r="C4" t="str">
-        <v>SBI Home Loan</v>
+        <v>Shibin</v>
       </c>
       <c r="D4" t="str">
-        <v>Housing Loan</v>
+        <v>test loadn</v>
       </c>
       <c r="E4">
-        <v>5758624</v>
+        <v>1200</v>
       </c>
       <c r="F4">
         <v>0</v>
@@ -2433,13 +2433,13 @@
         <v>0</v>
       </c>
       <c r="I4">
-        <v>5758624</v>
+        <v>1200</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>5758624</v>
+        <v>1200</v>
       </c>
       <c r="L4" t="str">
         <v>2026-08-14</v>
@@ -2460,7 +2460,7 @@
         <v/>
       </c>
       <c r="R4" t="str">
-        <v/>
+        <v>22001</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-20T14:46:21.526Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M42"/>
+  <dimension ref="A1:M43"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2070,9 +2070,50 @@
         <v/>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>TXN-1040</v>
+      </c>
+      <c r="B43" t="str">
+        <v>2026-07-16</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D43" t="str">
+        <v>SBI Bank</v>
+      </c>
+      <c r="E43" t="str">
+        <v>Rent paid</v>
+      </c>
+      <c r="F43">
+        <v>2300</v>
+      </c>
+      <c r="G43" t="str">
+        <v/>
+      </c>
+      <c r="H43" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="I43" t="str">
+        <v/>
+      </c>
+      <c r="J43" t="str">
+        <v/>
+      </c>
+      <c r="K43" t="str">
+        <v/>
+      </c>
+      <c r="L43" t="str">
+        <v>[{"kind":"Bank","acct":"11004","sub":"bank:SBI","dr":0,"cr":2300},{"kind":"Ledger","acct":"51001","sub":"","dr":2000,"cr":0},{"kind":"Ledger","acct":"51002","sub":"","dr":300,"cr":0}]</v>
+      </c>
+      <c r="M43" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M42"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M43"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2208,10 +2249,10 @@
         <v>50000</v>
       </c>
       <c r="G5">
-        <v>78700</v>
+        <v>81000</v>
       </c>
       <c r="H5">
-        <v>55624.2</v>
+        <v>53324.2</v>
       </c>
       <c r="I5" t="str">
         <v/>
@@ -2226,7 +2267,7 @@
         <v>Pending</v>
       </c>
       <c r="M5" t="str">
-        <v/>
+        <v>11004</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-20T14:48:44.788Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M43"/>
+  <dimension ref="A1:M44"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2111,9 +2111,50 @@
         <v/>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>TXN-1041</v>
+      </c>
+      <c r="B44" t="str">
+        <v>2026-08-20</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Personal Borrowings</v>
+      </c>
+      <c r="E44" t="str">
+        <v/>
+      </c>
+      <c r="F44">
+        <v>300</v>
+      </c>
+      <c r="G44" t="str">
+        <v/>
+      </c>
+      <c r="H44" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="I44" t="str">
+        <v/>
+      </c>
+      <c r="J44" t="str">
+        <v/>
+      </c>
+      <c r="K44" t="str">
+        <v/>
+      </c>
+      <c r="L44" t="str">
+        <v>[{"kind":"Loan","acct":"22001","sub":"ld:LOAN-01","dr":0,"cr":300},{"kind":"Bank","acct":"11004","sub":"bank:SBI","dr":300,"cr":0}]</v>
+      </c>
+      <c r="M44" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M43"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M44"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2246,13 +2287,13 @@
         <v>84324.2</v>
       </c>
       <c r="F5">
-        <v>50000</v>
+        <v>50300</v>
       </c>
       <c r="G5">
         <v>81000</v>
       </c>
       <c r="H5">
-        <v>53324.2</v>
+        <v>53624.2</v>
       </c>
       <c r="I5" t="str">
         <v/>
@@ -2462,7 +2503,7 @@
         <v>test loadn</v>
       </c>
       <c r="E4">
-        <v>1200</v>
+        <v>1500</v>
       </c>
       <c r="F4">
         <v>0</v>
@@ -2474,13 +2515,13 @@
         <v>0</v>
       </c>
       <c r="I4">
-        <v>1200</v>
+        <v>1500</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>1200</v>
+        <v>1500</v>
       </c>
       <c r="L4" t="str">
         <v>2026-08-14</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-20T14:49:23.720Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -2506,22 +2506,22 @@
         <v>1500</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>184.17</v>
       </c>
       <c r="I4">
-        <v>1500</v>
+        <v>1841.7</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>1500</v>
+        <v>1841.7</v>
       </c>
       <c r="L4" t="str">
         <v>2026-08-14</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-20T18:23:35.104Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -1792,7 +1792,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:O8"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -2056,9 +2056,56 @@
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>CARD-01</v>
+      </c>
+      <c r="B8" t="str">
+        <v>ICICI BANK</v>
+      </c>
+      <c r="C8" t="str">
+        <v>100020100</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Credit Card</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="M8" t="str">
+        <v>23001</v>
+      </c>
+      <c r="N8" t="str">
+        <v>Credit Card</v>
+      </c>
+      <c r="O8">
+        <v>350000</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O8"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-20T18:26:47.436Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M35"/>
+  <dimension ref="A1:M36"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1783,9 +1783,50 @@
         <v/>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>TXN-1033</v>
+      </c>
+      <c r="B36" t="str">
+        <v>2026-08-20</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Credit Card Payable</v>
+      </c>
+      <c r="E36" t="str">
+        <v/>
+      </c>
+      <c r="F36">
+        <v>3500</v>
+      </c>
+      <c r="G36" t="str">
+        <v/>
+      </c>
+      <c r="H36" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="I36" t="str">
+        <v/>
+      </c>
+      <c r="J36" t="str">
+        <v/>
+      </c>
+      <c r="K36" t="str">
+        <v/>
+      </c>
+      <c r="L36" t="str">
+        <v>[{"kind":"Bank","acct":"23001","sub":"bank:ICICI BANK","dr":0,"cr":3500},{"kind":"Ledger","acct":"51003","sub":"","dr":3500,"cr":0}]</v>
+      </c>
+      <c r="M36" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M36"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2076,10 +2117,10 @@
         <v>0</v>
       </c>
       <c r="G8">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="I8" t="str">
         <v/>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-20T20:29:03.899Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:M37"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1824,9 +1824,50 @@
         <v/>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>TXN-1034</v>
+      </c>
+      <c r="B37" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Debt Given</v>
+      </c>
+      <c r="E37" t="str">
+        <v>BIJU ACHAN - Bike insurance</v>
+      </c>
+      <c r="F37">
+        <v>924</v>
+      </c>
+      <c r="G37" t="str">
+        <v>ICICI BANK</v>
+      </c>
+      <c r="H37" t="str">
+        <v>Bank Import</v>
+      </c>
+      <c r="I37" t="str">
+        <v>Linked: DEBT-08 (BIJU ACHAN - Bike insurance)</v>
+      </c>
+      <c r="J37" t="str">
+        <v/>
+      </c>
+      <c r="K37" t="str">
+        <v/>
+      </c>
+      <c r="L37" t="str">
+        <v/>
+      </c>
+      <c r="M37" t="str">
+        <v>13669854335</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M37"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2117,10 +2158,10 @@
         <v>0</v>
       </c>
       <c r="G8">
-        <v>3500</v>
+        <v>4424</v>
       </c>
       <c r="H8">
-        <v>3500</v>
+        <v>4424</v>
       </c>
       <c r="I8" t="str">
         <v/>
@@ -2153,7 +2194,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S8"/>
+  <dimension ref="A1:S9"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -2540,9 +2581,68 @@
         <v/>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>DEBT-08</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Debt Receivable</v>
+      </c>
+      <c r="C9" t="str">
+        <v>BIJU ACHAN - Bike insurance</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Posted 2026-06-25</v>
+      </c>
+      <c r="E9">
+        <v>924</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>924</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>924</v>
+      </c>
+      <c r="L9" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
+        <v>Open</v>
+      </c>
+      <c r="O9" t="str">
+        <v/>
+      </c>
+      <c r="P9" t="str">
+        <v/>
+      </c>
+      <c r="Q9" t="str">
+        <v/>
+      </c>
+      <c r="R9" t="str">
+        <v/>
+      </c>
+      <c r="S9" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S9"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-20T20:30:23.536Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -2303,22 +2303,22 @@
         <v>5758624</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>7.3</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>330</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>40505.71</v>
       </c>
       <c r="I4">
-        <v>5758624</v>
+        <v>13366884.3</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>5758624</v>
+        <v>13366884.3</v>
       </c>
       <c r="L4" t="str">
         <v>2026-08-14</v>
@@ -2339,7 +2339,7 @@
         <v/>
       </c>
       <c r="R4" t="str">
-        <v/>
+        <v>21001</v>
       </c>
       <c r="S4" t="str">
         <v/>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-21T10:55:40.286Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M37"/>
+  <dimension ref="A1:M38"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1865,9 +1865,50 @@
         <v>13669854335</v>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>TXN-1035</v>
+      </c>
+      <c r="B38" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D38" t="str">
+        <v>(new)</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Mobile - NeeNa</v>
+      </c>
+      <c r="F38">
+        <v>20004</v>
+      </c>
+      <c r="G38" t="str">
+        <v/>
+      </c>
+      <c r="H38" t="str">
+        <v>Card</v>
+      </c>
+      <c r="I38" t="str">
+        <v/>
+      </c>
+      <c r="J38" t="str">
+        <v/>
+      </c>
+      <c r="K38" t="str">
+        <v/>
+      </c>
+      <c r="L38" t="str">
+        <v>[{"kind":"Loan","acct":"(new)","sub":"ld:DEBT-09","dr":20004,"cr":0},{"kind":"Bank","acct":"23001","sub":"bank:ICICI BANK","dr":0,"cr":20004}]</v>
+      </c>
+      <c r="M38" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M38"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2158,10 +2199,10 @@
         <v>0</v>
       </c>
       <c r="G8">
-        <v>4424</v>
+        <v>24428</v>
       </c>
       <c r="H8">
-        <v>4424</v>
+        <v>24428</v>
       </c>
       <c r="I8" t="str">
         <v/>
@@ -2194,7 +2235,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S9"/>
+  <dimension ref="A1:S10"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -2640,9 +2681,68 @@
         <v/>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>DEBT-09</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Debt Receivable</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Mobile - NeeNa</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Posted 2026-08-01</v>
+      </c>
+      <c r="E10">
+        <v>20004</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>20004</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>20004</v>
+      </c>
+      <c r="L10" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
+      <c r="N10" t="str">
+        <v>Open</v>
+      </c>
+      <c r="O10" t="str">
+        <v/>
+      </c>
+      <c r="P10" t="str">
+        <v/>
+      </c>
+      <c r="Q10" t="str">
+        <v>TXN-1035</v>
+      </c>
+      <c r="R10" t="str">
+        <v>(new)</v>
+      </c>
+      <c r="S10" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S10"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-21T10:56:11.846Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -2698,22 +2698,22 @@
         <v>20004</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G10">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H10">
-        <v>0</v>
+        <v>3422.06</v>
       </c>
       <c r="I10">
-        <v>20004</v>
+        <v>20532.36</v>
       </c>
       <c r="J10">
         <v>0</v>
       </c>
       <c r="K10">
-        <v>20004</v>
+        <v>20532.36</v>
       </c>
       <c r="L10" t="str">
         <v>2026-08-01</v>
@@ -2734,7 +2734,7 @@
         <v>TXN-1035</v>
       </c>
       <c r="R10" t="str">
-        <v>(new)</v>
+        <v>13001</v>
       </c>
       <c r="S10" t="str">
         <v/>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-21T11:12:45.632Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M38"/>
+  <dimension ref="A1:M39"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1906,16 +1906,57 @@
         <v/>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>TXN-1036</v>
+      </c>
+      <c r="B39" t="str">
+        <v>2026-08-21</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Household Appliances</v>
+      </c>
+      <c r="E39" t="str">
+        <v/>
+      </c>
+      <c r="F39">
+        <v>20004</v>
+      </c>
+      <c r="G39" t="str">
+        <v/>
+      </c>
+      <c r="H39" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="I39" t="str">
+        <v>EMI plan: EMI-01</v>
+      </c>
+      <c r="J39" t="str">
+        <v/>
+      </c>
+      <c r="K39" t="str">
+        <v/>
+      </c>
+      <c r="L39" t="str">
+        <v>[{"kind":"Ledger","acct":"51005","sub":"","dr":20004,"cr":0},{"kind":"Bank","acct":"23001","sub":"bank:ICICI BANK","dr":0,"cr":20004}]</v>
+      </c>
+      <c r="M39" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M39"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:P8"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -1932,6 +1973,7 @@
     <col min="13" max="13" width="12.83203125" customWidth="1"/>
     <col min="14" max="14" width="13.83203125" customWidth="1"/>
     <col min="15" max="15" width="13.83203125" customWidth="1"/>
+    <col min="16" max="16" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1990,6 +2032,9 @@
       <c r="O3" t="str">
         <v>Credit Limit</v>
       </c>
+      <c r="P3" t="str">
+        <v>Payment Due Day</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -2037,6 +2082,9 @@
       <c r="O4" t="str">
         <v/>
       </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -2084,6 +2132,9 @@
       <c r="O5" t="str">
         <v/>
       </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -2131,6 +2182,9 @@
       <c r="O6" t="str">
         <v/>
       </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -2178,6 +2232,9 @@
       <c r="O7" t="str">
         <v/>
       </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -2199,10 +2256,10 @@
         <v>0</v>
       </c>
       <c r="G8">
-        <v>24428</v>
+        <v>44432</v>
       </c>
       <c r="H8">
-        <v>24428</v>
+        <v>44432</v>
       </c>
       <c r="I8" t="str">
         <v/>
@@ -2225,17 +2282,20 @@
       <c r="O8">
         <v>350000</v>
       </c>
+      <c r="P8" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P8"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S10"/>
+  <dimension ref="A1:S11"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -2740,9 +2800,68 @@
         <v/>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>EMI-01</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Bank Loan Payable</v>
+      </c>
+      <c r="C11" t="str">
+        <v>EMI purchase</v>
+      </c>
+      <c r="D11" t="str">
+        <v>EMI · voucher TXN-1036</v>
+      </c>
+      <c r="E11">
+        <v>20004</v>
+      </c>
+      <c r="F11">
+        <v>9.4</v>
+      </c>
+      <c r="G11">
+        <v>12</v>
+      </c>
+      <c r="H11">
+        <v>1753.09</v>
+      </c>
+      <c r="I11">
+        <v>21037.08</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>21037.08</v>
+      </c>
+      <c r="L11" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="M11" t="str">
+        <v/>
+      </c>
+      <c r="N11" t="str">
+        <v>Open</v>
+      </c>
+      <c r="O11" t="str">
+        <v/>
+      </c>
+      <c r="P11" t="str">
+        <v/>
+      </c>
+      <c r="Q11" t="str">
+        <v>TXN-1036</v>
+      </c>
+      <c r="R11" t="str">
+        <v>21001</v>
+      </c>
+      <c r="S11" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S11"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-21T12:00:05.811Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M28"/>
+  <dimension ref="A1:M29"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1496,9 +1496,50 @@
         <v/>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>TXN-10026</v>
+      </c>
+      <c r="B29" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D29" t="str">
+        <v>(new)</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Neena Phone</v>
+      </c>
+      <c r="F29">
+        <v>20004</v>
+      </c>
+      <c r="G29" t="str">
+        <v/>
+      </c>
+      <c r="H29" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="I29" t="str">
+        <v/>
+      </c>
+      <c r="J29" t="str">
+        <v/>
+      </c>
+      <c r="K29" t="str">
+        <v/>
+      </c>
+      <c r="L29" t="str">
+        <v>[{"kind":"Loan","acct":"(new)","sub":"ld:DEBT-06","dr":20004,"cr":0},{"kind":"Bank","acct":"23002","sub":"bank:ICICI Amazon Card","dr":0,"cr":20004}]</v>
+      </c>
+      <c r="M29" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M29"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1605,10 +1646,10 @@
         <v>170180</v>
       </c>
       <c r="G4">
-        <v>58800</v>
+        <v>85800</v>
       </c>
       <c r="H4">
-        <v>171380</v>
+        <v>144380</v>
       </c>
       <c r="I4" t="str">
         <v/>
@@ -1755,10 +1796,10 @@
         <v>1240</v>
       </c>
       <c r="G7">
-        <v>860</v>
+        <v>79560</v>
       </c>
       <c r="H7">
-        <v>50380</v>
+        <v>-28320</v>
       </c>
       <c r="I7" t="str">
         <v/>
@@ -1805,10 +1846,10 @@
         <v>5000</v>
       </c>
       <c r="G8">
-        <v>0</v>
+        <v>12000</v>
       </c>
       <c r="H8">
-        <v>10000</v>
+        <v>-2000</v>
       </c>
       <c r="I8" t="str">
         <v/>
@@ -1855,10 +1896,10 @@
         <v>3373</v>
       </c>
       <c r="G9">
-        <v>34029</v>
+        <v>66033</v>
       </c>
       <c r="H9">
-        <v>30656</v>
+        <v>62660</v>
       </c>
       <c r="I9" t="str">
         <v/>
@@ -1944,7 +1985,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S11"/>
+  <dimension ref="A1:S12"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -2295,13 +2336,13 @@
         <v>240</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>21695.58</v>
       </c>
       <c r="I8">
-        <v>1950000</v>
+        <v>5206939.2</v>
       </c>
       <c r="J8">
-        <v>0</v>
+        <v>3256939.2</v>
       </c>
       <c r="K8">
         <v>1950000</v>
@@ -2354,13 +2395,13 @@
         <v>36</v>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>3843.95</v>
       </c>
       <c r="I9">
-        <v>78000</v>
+        <v>138382.2</v>
       </c>
       <c r="J9">
-        <v>0</v>
+        <v>60382.2</v>
       </c>
       <c r="K9">
         <v>78000</v>
@@ -2472,13 +2513,13 @@
         <v>12</v>
       </c>
       <c r="H11">
-        <v>0</v>
+        <v>2972.4</v>
       </c>
       <c r="I11">
-        <v>33105</v>
+        <v>35668.8</v>
       </c>
       <c r="J11">
-        <v>0</v>
+        <v>2563.8</v>
       </c>
       <c r="K11">
         <v>33105</v>
@@ -2508,9 +2549,68 @@
         <v/>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>DEBT-06</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Debt Receivable</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Neena Phone</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Posted 2026-08-01</v>
+      </c>
+      <c r="E12">
+        <v>20004</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>20004</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>20004</v>
+      </c>
+      <c r="L12" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="M12" t="str">
+        <v/>
+      </c>
+      <c r="N12" t="str">
+        <v>Open</v>
+      </c>
+      <c r="O12" t="str">
+        <v/>
+      </c>
+      <c r="P12" t="str">
+        <v/>
+      </c>
+      <c r="Q12" t="str">
+        <v>TXN-10026</v>
+      </c>
+      <c r="R12" t="str">
+        <v>(new)</v>
+      </c>
+      <c r="S12" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S12"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-21T12:14:45.294Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -1985,7 +1985,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S12"/>
+  <dimension ref="A1:U12"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -2006,6 +2006,8 @@
     <col min="17" max="17" width="18.83203125" customWidth="1"/>
     <col min="18" max="18" width="18.83203125" customWidth="1"/>
     <col min="19" max="19" width="14.83203125" customWidth="1"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1"/>
+    <col min="21" max="21" width="9.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2015,7 +2017,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Interest-aware tracking. Net Payable = EMI x Term. Payments reduce Balance Due. Credit cards track available = limit − balance.</v>
+        <v>Interest-aware tracking. Net Payable = EMI x Term. Payments reduce Balance Due. Monthly commitments recur on a Due Day.</v>
       </c>
     </row>
     <row r="3">
@@ -2076,6 +2078,12 @@
       <c r="S3" t="str">
         <v>Credit Limit</v>
       </c>
+      <c r="T3" t="str">
+        <v>Monthly</v>
+      </c>
+      <c r="U3" t="str">
+        <v>Due Day</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -2135,6 +2143,12 @@
       <c r="S4" t="str">
         <v/>
       </c>
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -2194,6 +2208,12 @@
       <c r="S5" t="str">
         <v/>
       </c>
+      <c r="T5" t="str">
+        <v/>
+      </c>
+      <c r="U5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -2253,6 +2273,12 @@
       <c r="S6" t="str">
         <v/>
       </c>
+      <c r="T6" t="str">
+        <v/>
+      </c>
+      <c r="U6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -2312,6 +2338,12 @@
       <c r="S7" t="str">
         <v/>
       </c>
+      <c r="T7" t="str">
+        <v/>
+      </c>
+      <c r="U7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -2371,6 +2403,12 @@
       <c r="S8" t="str">
         <v/>
       </c>
+      <c r="T8" t="str">
+        <v/>
+      </c>
+      <c r="U8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -2430,6 +2468,12 @@
       <c r="S9" t="str">
         <v/>
       </c>
+      <c r="T9" t="str">
+        <v/>
+      </c>
+      <c r="U9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -2489,6 +2533,12 @@
       <c r="S10" t="str">
         <v/>
       </c>
+      <c r="T10" t="str">
+        <v/>
+      </c>
+      <c r="U10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -2548,6 +2598,12 @@
       <c r="S11" t="str">
         <v/>
       </c>
+      <c r="T11" t="str">
+        <v/>
+      </c>
+      <c r="U11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -2566,22 +2622,22 @@
         <v>20004</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H12">
-        <v>0</v>
+        <v>5095.12</v>
       </c>
       <c r="I12">
-        <v>20004</v>
+        <v>20380.48</v>
       </c>
       <c r="J12">
         <v>0</v>
       </c>
       <c r="K12">
-        <v>20004</v>
+        <v>20380.48</v>
       </c>
       <c r="L12" t="str">
         <v>2026-08-01</v>
@@ -2602,15 +2658,21 @@
         <v>TXN-10026</v>
       </c>
       <c r="R12" t="str">
-        <v>(new)</v>
+        <v>13001</v>
       </c>
       <c r="S12" t="str">
         <v/>
+      </c>
+      <c r="T12" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="U12">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U12"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4879,7 +4941,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4929,9 +4991,17 @@
         <v>light</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>AllowDelete</v>
+      </c>
+      <c r="B7" t="str">
+        <v>No</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-21T12:15:06.411Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -2622,22 +2622,22 @@
         <v>20004</v>
       </c>
       <c r="F12">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G12">
         <v>4</v>
       </c>
       <c r="H12">
-        <v>5095.12</v>
+        <v>5126.65</v>
       </c>
       <c r="I12">
-        <v>20380.48</v>
+        <v>20506.6</v>
       </c>
       <c r="J12">
         <v>0</v>
       </c>
       <c r="K12">
-        <v>20380.48</v>
+        <v>20506.6</v>
       </c>
       <c r="L12" t="str">
         <v>2026-08-01</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-21T12:15:30.091Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -2625,19 +2625,19 @@
         <v>12</v>
       </c>
       <c r="G12">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H12">
-        <v>5126.65</v>
+        <v>3451.66</v>
       </c>
       <c r="I12">
-        <v>20506.6</v>
+        <v>20709.96</v>
       </c>
       <c r="J12">
         <v>0</v>
       </c>
       <c r="K12">
-        <v>20506.6</v>
+        <v>20709.96</v>
       </c>
       <c r="L12" t="str">
         <v>2026-08-01</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-21T16:54:32.363Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -1607,10 +1607,10 @@
         <v>170180</v>
       </c>
       <c r="G4">
-        <v>58800</v>
+        <v>85800</v>
       </c>
       <c r="H4">
-        <v>171380</v>
+        <v>144380</v>
       </c>
       <c r="I4" t="str">
         <v/>
@@ -1757,10 +1757,10 @@
         <v>1240</v>
       </c>
       <c r="G7">
-        <v>860</v>
+        <v>79560</v>
       </c>
       <c r="H7">
-        <v>50380</v>
+        <v>-28320</v>
       </c>
       <c r="I7" t="str">
         <v/>
@@ -1807,10 +1807,10 @@
         <v>5000</v>
       </c>
       <c r="G8">
-        <v>0</v>
+        <v>12000</v>
       </c>
       <c r="H8">
-        <v>10000</v>
+        <v>-2000</v>
       </c>
       <c r="I8" t="str">
         <v/>
@@ -1857,10 +1857,10 @@
         <v>3373</v>
       </c>
       <c r="G9">
-        <v>34029</v>
+        <v>46029</v>
       </c>
       <c r="H9">
-        <v>30656</v>
+        <v>42656</v>
       </c>
       <c r="I9" t="str">
         <v/>
@@ -1946,7 +1946,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:U12"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -2329,13 +2329,13 @@
         <v>240</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>21695.58</v>
       </c>
       <c r="I8">
-        <v>1950000</v>
+        <v>5206939.2</v>
       </c>
       <c r="J8">
-        <v>0</v>
+        <v>3256939.2</v>
       </c>
       <c r="K8">
         <v>1950000</v>
@@ -2394,13 +2394,13 @@
         <v>36</v>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>3843.95</v>
       </c>
       <c r="I9">
-        <v>78000</v>
+        <v>138382.2</v>
       </c>
       <c r="J9">
-        <v>0</v>
+        <v>60382.2</v>
       </c>
       <c r="K9">
         <v>78000</v>
@@ -2524,13 +2524,13 @@
         <v>12</v>
       </c>
       <c r="H11">
-        <v>0</v>
+        <v>2972.4</v>
       </c>
       <c r="I11">
-        <v>33105</v>
+        <v>35668.8</v>
       </c>
       <c r="J11">
-        <v>0</v>
+        <v>2563.8</v>
       </c>
       <c r="K11">
         <v>33105</v>
@@ -2566,9 +2566,74 @@
         <v/>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>DEBT-06</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Debt Receivable</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Neena</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Mobile Purchase</v>
+      </c>
+      <c r="E12">
+        <v>20004</v>
+      </c>
+      <c r="F12">
+        <v>9</v>
+      </c>
+      <c r="G12">
+        <v>6</v>
+      </c>
+      <c r="H12">
+        <v>3422.06</v>
+      </c>
+      <c r="I12">
+        <v>20532.36</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>20532.36</v>
+      </c>
+      <c r="L12" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="M12" t="str">
+        <v/>
+      </c>
+      <c r="N12" t="str">
+        <v>Open</v>
+      </c>
+      <c r="O12" t="str">
+        <v/>
+      </c>
+      <c r="P12" t="str">
+        <v/>
+      </c>
+      <c r="Q12" t="str">
+        <v/>
+      </c>
+      <c r="R12" t="str">
+        <v>13001</v>
+      </c>
+      <c r="S12" t="str">
+        <v/>
+      </c>
+      <c r="T12" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="U12">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:U11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U12"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-21T17:18:43.264Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -3260,7 +3260,7 @@
         <v>Monthly</v>
       </c>
       <c r="E4" t="str">
-        <v>2026-08-25</v>
+        <v>2026-09-25</v>
       </c>
       <c r="F4">
         <v>399</v>
@@ -3288,8 +3288,8 @@
       <c r="E5" t="str">
         <v>2026-08-23</v>
       </c>
-      <c r="F5">
-        <v>500</v>
+      <c r="F5" t="str">
+        <v/>
       </c>
       <c r="G5" t="str">
         <v>Active</v>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-21T19:56:01.944Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -414,7 +414,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O32"/>
+  <dimension ref="A1:O33"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1853,9 +1853,56 @@
         <v>EVT-02</v>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>TXN-10030</v>
+      </c>
+      <c r="B33" t="str">
+        <v>2026-08-21</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Commitment</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Interest Expense</v>
+      </c>
+      <c r="F33" t="str">
+        <v/>
+      </c>
+      <c r="G33">
+        <v>399</v>
+      </c>
+      <c r="H33" t="str">
+        <v/>
+      </c>
+      <c r="I33" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="J33" t="str">
+        <v>Commitment: CM-01</v>
+      </c>
+      <c r="K33" t="str">
+        <v/>
+      </c>
+      <c r="L33" t="str">
+        <v/>
+      </c>
+      <c r="M33" t="str">
+        <v>[{"kind":"Commitment","acct":"55008","sub":"cm:CM-01","cat":"","dr":399,"cr":0},{"kind":"Bank","acct":"23002","sub":"bank:ICICI Amazon Card","cat":"","dr":0,"cr":399}]</v>
+      </c>
+      <c r="N33" t="str">
+        <v/>
+      </c>
+      <c r="O33" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O33"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2212,10 +2259,10 @@
         <v>3373</v>
       </c>
       <c r="G9">
-        <v>46029</v>
+        <v>46428</v>
       </c>
       <c r="H9">
-        <v>42656</v>
+        <v>43055</v>
       </c>
       <c r="I9" t="str">
         <v/>
@@ -3558,7 +3605,7 @@
         <v>Monthly</v>
       </c>
       <c r="E4" t="str">
-        <v>2026-08-25</v>
+        <v>2026-09-25</v>
       </c>
       <c r="F4">
         <v>399</v>
@@ -5898,7 +5945,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L33"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -7064,16 +7111,54 @@
         <v>Yes</v>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>TXN-10030</v>
+      </c>
+      <c r="B33" t="str">
+        <v>2026-08-21</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Commitment</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Interest Expense</v>
+      </c>
+      <c r="F33">
+        <v>399</v>
+      </c>
+      <c r="G33" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="H33" t="str">
+        <v/>
+      </c>
+      <c r="I33" t="str">
+        <v>Commitment: CM-01</v>
+      </c>
+      <c r="J33" t="str">
+        <v/>
+      </c>
+      <c r="K33">
+        <v>2</v>
+      </c>
+      <c r="L33" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L33"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L63"/>
+  <dimension ref="A1:L65"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -9417,9 +9502,85 @@
         <v>ACC-01</v>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>TXN-10030-L1</v>
+      </c>
+      <c r="B64" t="str">
+        <v>TXN-10030</v>
+      </c>
+      <c r="C64">
+        <v>1</v>
+      </c>
+      <c r="D64">
+        <v>399</v>
+      </c>
+      <c r="E64" t="str">
+        <v>Dr</v>
+      </c>
+      <c r="F64" t="str">
+        <v>55008</v>
+      </c>
+      <c r="G64" t="str">
+        <v>Interest Expense</v>
+      </c>
+      <c r="H64" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="I64" t="str">
+        <v>Financial</v>
+      </c>
+      <c r="J64" t="str">
+        <v>Commitment</v>
+      </c>
+      <c r="K64" t="str">
+        <v/>
+      </c>
+      <c r="L64" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>TXN-10030-L2</v>
+      </c>
+      <c r="B65" t="str">
+        <v>TXN-10030</v>
+      </c>
+      <c r="C65">
+        <v>2</v>
+      </c>
+      <c r="D65">
+        <v>-399</v>
+      </c>
+      <c r="E65" t="str">
+        <v>Cr</v>
+      </c>
+      <c r="F65" t="str">
+        <v>23002</v>
+      </c>
+      <c r="G65" t="str">
+        <v>ICICI Amazon Card</v>
+      </c>
+      <c r="H65" t="str">
+        <v>Liability</v>
+      </c>
+      <c r="I65" t="str">
+        <v>Credit Cards</v>
+      </c>
+      <c r="J65" t="str">
+        <v>Bank</v>
+      </c>
+      <c r="K65" t="str">
+        <v>Card</v>
+      </c>
+      <c r="L65" t="str">
+        <v>CARD-01</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L63"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L65"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -10241,7 +10402,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -10438,9 +10599,38 @@
         <v>Bought gadget - split with Baby</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>TXN-10030-L2</v>
+      </c>
+      <c r="B9" t="str">
+        <v>CARD-01</v>
+      </c>
+      <c r="C9" t="str">
+        <v>TXN-10030</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9" t="str">
+        <v>2026-08-21</v>
+      </c>
+      <c r="F9">
+        <v>-399</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Cr</v>
+      </c>
+      <c r="H9" t="str">
+        <v>ICICI Amazon Card</v>
+      </c>
+      <c r="I9" t="str">
+        <v>Interest Expense</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I9"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-21T19:56:47.637Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -414,7 +414,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O33"/>
+  <dimension ref="A1:O34"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1900,9 +1900,56 @@
         <v/>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>TXN-10031</v>
+      </c>
+      <c r="B34" t="str">
+        <v>2026-08-21</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Commitment</v>
+      </c>
+      <c r="E34" t="str">
+        <v>CM</v>
+      </c>
+      <c r="F34" t="str">
+        <v/>
+      </c>
+      <c r="G34">
+        <v>700</v>
+      </c>
+      <c r="H34" t="str">
+        <v/>
+      </c>
+      <c r="I34" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="J34" t="str">
+        <v>Commitment: CM-02</v>
+      </c>
+      <c r="K34" t="str">
+        <v/>
+      </c>
+      <c r="L34" t="str">
+        <v/>
+      </c>
+      <c r="M34" t="str">
+        <v>[{"kind":"Commitment","acct":"CM","sub":"cm:CM-02","cat":"","dr":700,"cr":0},{"kind":"Bank","acct":"11001","sub":"bank:HDFC-Info","cat":"","dr":0,"cr":700}]</v>
+      </c>
+      <c r="N34" t="str">
+        <v/>
+      </c>
+      <c r="O34" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O34"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2009,10 +2056,10 @@
         <v>170180</v>
       </c>
       <c r="G4">
-        <v>365800</v>
+        <v>366500</v>
       </c>
       <c r="H4">
-        <v>-135620</v>
+        <v>-136320</v>
       </c>
       <c r="I4" t="str">
         <v/>
@@ -3637,7 +3684,7 @@
         <v>Weekly</v>
       </c>
       <c r="E5" t="str">
-        <v>2026-08-23</v>
+        <v>2026-08-30</v>
       </c>
       <c r="F5">
         <v>500</v>
@@ -5945,7 +5992,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L34"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -7149,16 +7196,54 @@
         <v>Yes</v>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>TXN-10031</v>
+      </c>
+      <c r="B34" t="str">
+        <v>2026-08-21</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Commitment</v>
+      </c>
+      <c r="E34" t="str">
+        <v>CM</v>
+      </c>
+      <c r="F34">
+        <v>700</v>
+      </c>
+      <c r="G34" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="H34" t="str">
+        <v/>
+      </c>
+      <c r="I34" t="str">
+        <v>Commitment: CM-02</v>
+      </c>
+      <c r="J34" t="str">
+        <v/>
+      </c>
+      <c r="K34">
+        <v>2</v>
+      </c>
+      <c r="L34" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L34"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L65"/>
+  <dimension ref="A1:L67"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -9578,16 +9663,92 @@
         <v>CARD-01</v>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>TXN-10031-L1</v>
+      </c>
+      <c r="B66" t="str">
+        <v>TXN-10031</v>
+      </c>
+      <c r="C66">
+        <v>1</v>
+      </c>
+      <c r="D66">
+        <v>700</v>
+      </c>
+      <c r="E66" t="str">
+        <v>Dr</v>
+      </c>
+      <c r="F66" t="str">
+        <v>CM</v>
+      </c>
+      <c r="G66" t="str">
+        <v>House cleaning</v>
+      </c>
+      <c r="H66" t="str">
+        <v/>
+      </c>
+      <c r="I66" t="str">
+        <v/>
+      </c>
+      <c r="J66" t="str">
+        <v>Commitment</v>
+      </c>
+      <c r="K66" t="str">
+        <v/>
+      </c>
+      <c r="L66" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>TXN-10031-L2</v>
+      </c>
+      <c r="B67" t="str">
+        <v>TXN-10031</v>
+      </c>
+      <c r="C67">
+        <v>2</v>
+      </c>
+      <c r="D67">
+        <v>-700</v>
+      </c>
+      <c r="E67" t="str">
+        <v>Cr</v>
+      </c>
+      <c r="F67" t="str">
+        <v>11001</v>
+      </c>
+      <c r="G67" t="str">
+        <v>HDFC-Info Bank</v>
+      </c>
+      <c r="H67" t="str">
+        <v>Asset</v>
+      </c>
+      <c r="I67" t="str">
+        <v>Cash &amp; Bank</v>
+      </c>
+      <c r="J67" t="str">
+        <v>Bank</v>
+      </c>
+      <c r="K67" t="str">
+        <v>Bank</v>
+      </c>
+      <c r="L67" t="str">
+        <v>ACC-01</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L65"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L67"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I30"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -10393,9 +10554,38 @@
         <v>Wedding gold advance · Event type: Gold</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>TXN-10031-L2</v>
+      </c>
+      <c r="B30" t="str">
+        <v>ACC-01</v>
+      </c>
+      <c r="C30" t="str">
+        <v>TXN-10031</v>
+      </c>
+      <c r="D30">
+        <v>2</v>
+      </c>
+      <c r="E30" t="str">
+        <v>2026-08-21</v>
+      </c>
+      <c r="F30">
+        <v>-700</v>
+      </c>
+      <c r="G30" t="str">
+        <v>Cr</v>
+      </c>
+      <c r="H30" t="str">
+        <v>HDFC-Info Bank</v>
+      </c>
+      <c r="I30" t="str">
+        <v>CM</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I30"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-21T19:58:12.322Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -414,7 +414,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O34"/>
+  <dimension ref="A1:O35"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1947,9 +1947,56 @@
         <v/>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>TXN-10032</v>
+      </c>
+      <c r="B35" t="str">
+        <v>2026-09-24</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Commitment</v>
+      </c>
+      <c r="E35" t="str">
+        <v>CM</v>
+      </c>
+      <c r="F35" t="str">
+        <v>Hose cleaning</v>
+      </c>
+      <c r="G35">
+        <v>800</v>
+      </c>
+      <c r="H35" t="str">
+        <v/>
+      </c>
+      <c r="I35" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="J35" t="str">
+        <v>Commitment: CM-02</v>
+      </c>
+      <c r="K35" t="str">
+        <v/>
+      </c>
+      <c r="L35" t="str">
+        <v/>
+      </c>
+      <c r="M35" t="str">
+        <v>[{"kind":"Commitment","acct":"CM","sub":"cm:CM-02","cat":"","dr":800,"cr":0},{"kind":"Bank","acct":"11003","sub":"bank:Federal-Ang","cat":"","dr":0,"cr":800}]</v>
+      </c>
+      <c r="N35" t="str">
+        <v/>
+      </c>
+      <c r="O35" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O35"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2156,10 +2203,10 @@
         <v>42000</v>
       </c>
       <c r="G6">
-        <v>41050</v>
+        <v>41850</v>
       </c>
       <c r="H6">
-        <v>28950</v>
+        <v>28150</v>
       </c>
       <c r="I6" t="str">
         <v/>
@@ -3684,7 +3731,7 @@
         <v>Weekly</v>
       </c>
       <c r="E5" t="str">
-        <v>2026-08-30</v>
+        <v>2026-09-06</v>
       </c>
       <c r="F5">
         <v>500</v>
@@ -5992,7 +6039,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L35"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -7234,16 +7281,54 @@
         <v>Yes</v>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>TXN-10032</v>
+      </c>
+      <c r="B35" t="str">
+        <v>2026-09-24</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Commitment</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Hose cleaning</v>
+      </c>
+      <c r="F35">
+        <v>800</v>
+      </c>
+      <c r="G35" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="H35" t="str">
+        <v/>
+      </c>
+      <c r="I35" t="str">
+        <v>Commitment: CM-02</v>
+      </c>
+      <c r="J35" t="str">
+        <v/>
+      </c>
+      <c r="K35">
+        <v>2</v>
+      </c>
+      <c r="L35" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L35"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L67"/>
+  <dimension ref="A1:L69"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -9739,16 +9824,92 @@
         <v>ACC-01</v>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>TXN-10032-L1</v>
+      </c>
+      <c r="B68" t="str">
+        <v>TXN-10032</v>
+      </c>
+      <c r="C68">
+        <v>1</v>
+      </c>
+      <c r="D68">
+        <v>800</v>
+      </c>
+      <c r="E68" t="str">
+        <v>Dr</v>
+      </c>
+      <c r="F68" t="str">
+        <v>CM</v>
+      </c>
+      <c r="G68" t="str">
+        <v>House cleaning</v>
+      </c>
+      <c r="H68" t="str">
+        <v/>
+      </c>
+      <c r="I68" t="str">
+        <v/>
+      </c>
+      <c r="J68" t="str">
+        <v>Commitment</v>
+      </c>
+      <c r="K68" t="str">
+        <v/>
+      </c>
+      <c r="L68" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>TXN-10032-L2</v>
+      </c>
+      <c r="B69" t="str">
+        <v>TXN-10032</v>
+      </c>
+      <c r="C69">
+        <v>2</v>
+      </c>
+      <c r="D69">
+        <v>-800</v>
+      </c>
+      <c r="E69" t="str">
+        <v>Cr</v>
+      </c>
+      <c r="F69" t="str">
+        <v>11003</v>
+      </c>
+      <c r="G69" t="str">
+        <v>Federal-Ang Bank</v>
+      </c>
+      <c r="H69" t="str">
+        <v>Asset</v>
+      </c>
+      <c r="I69" t="str">
+        <v>Cash &amp; Bank</v>
+      </c>
+      <c r="J69" t="str">
+        <v>Bank</v>
+      </c>
+      <c r="K69" t="str">
+        <v>Bank</v>
+      </c>
+      <c r="L69" t="str">
+        <v>ACC-03</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L67"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L69"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I31"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -10583,9 +10744,38 @@
         <v>CM</v>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>TXN-10032-L2</v>
+      </c>
+      <c r="B31" t="str">
+        <v>ACC-03</v>
+      </c>
+      <c r="C31" t="str">
+        <v>TXN-10032</v>
+      </c>
+      <c r="D31">
+        <v>2</v>
+      </c>
+      <c r="E31" t="str">
+        <v>2026-09-24</v>
+      </c>
+      <c r="F31">
+        <v>-800</v>
+      </c>
+      <c r="G31" t="str">
+        <v>Cr</v>
+      </c>
+      <c r="H31" t="str">
+        <v>Federal-Ang Bank</v>
+      </c>
+      <c r="I31" t="str">
+        <v>Hose cleaning</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I30"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I31"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-21T20:05:23.581Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -414,7 +414,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O35"/>
+  <dimension ref="A1:O36"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1994,9 +1994,56 @@
         <v/>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>TXN-10033</v>
+      </c>
+      <c r="B36" t="str">
+        <v>2026-08-21</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Event</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Property / Land</v>
+      </c>
+      <c r="F36" t="str">
+        <v>Paid to vendor</v>
+      </c>
+      <c r="G36">
+        <v>104000</v>
+      </c>
+      <c r="H36" t="str">
+        <v/>
+      </c>
+      <c r="I36" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="J36" t="str">
+        <v>Event type: Cement</v>
+      </c>
+      <c r="K36" t="str">
+        <v/>
+      </c>
+      <c r="L36" t="str">
+        <v/>
+      </c>
+      <c r="M36" t="str">
+        <v>[{"kind":"Event","acct":"14002","sub":"ev:EVT-01","cat":"Cement","dr":104000,"cr":0},{"kind":"Bank","acct":"11004","sub":"bank:SBI","cat":"","dr":0,"cr":104000}]</v>
+      </c>
+      <c r="N36" t="str">
+        <v/>
+      </c>
+      <c r="O36" t="str">
+        <v>EVT-01</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O36"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2253,10 +2300,10 @@
         <v>1240</v>
       </c>
       <c r="G7">
-        <v>79560</v>
+        <v>183560</v>
       </c>
       <c r="H7">
-        <v>-28320</v>
+        <v>-132320</v>
       </c>
       <c r="I7" t="str">
         <v/>
@@ -3993,10 +4040,10 @@
         <v/>
       </c>
       <c r="L4">
-        <v>165000</v>
+        <v>269000</v>
       </c>
       <c r="M4">
-        <v>0</v>
+        <v>104000</v>
       </c>
       <c r="N4">
         <v>165000</v>
@@ -6039,7 +6086,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L36"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -7319,16 +7366,54 @@
         <v>Yes</v>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>TXN-10033</v>
+      </c>
+      <c r="B36" t="str">
+        <v>2026-08-21</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Event</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Paid to vendor</v>
+      </c>
+      <c r="F36">
+        <v>104000</v>
+      </c>
+      <c r="G36" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="H36" t="str">
+        <v>EVT-01</v>
+      </c>
+      <c r="I36" t="str">
+        <v>Event type: Cement</v>
+      </c>
+      <c r="J36" t="str">
+        <v/>
+      </c>
+      <c r="K36">
+        <v>2</v>
+      </c>
+      <c r="L36" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L36"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L69"/>
+  <dimension ref="A1:L71"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -9900,16 +9985,92 @@
         <v>ACC-03</v>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>TXN-10033-L1</v>
+      </c>
+      <c r="B70" t="str">
+        <v>TXN-10033</v>
+      </c>
+      <c r="C70">
+        <v>1</v>
+      </c>
+      <c r="D70">
+        <v>104000</v>
+      </c>
+      <c r="E70" t="str">
+        <v>Dr</v>
+      </c>
+      <c r="F70" t="str">
+        <v>14002</v>
+      </c>
+      <c r="G70" t="str">
+        <v>Property / Land</v>
+      </c>
+      <c r="H70" t="str">
+        <v>Asset</v>
+      </c>
+      <c r="I70" t="str">
+        <v>Fixed Assets</v>
+      </c>
+      <c r="J70" t="str">
+        <v>Event</v>
+      </c>
+      <c r="K70" t="str">
+        <v>Fixed Asset</v>
+      </c>
+      <c r="L70" t="str">
+        <v>FA-01</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>TXN-10033-L2</v>
+      </c>
+      <c r="B71" t="str">
+        <v>TXN-10033</v>
+      </c>
+      <c r="C71">
+        <v>2</v>
+      </c>
+      <c r="D71">
+        <v>-104000</v>
+      </c>
+      <c r="E71" t="str">
+        <v>Cr</v>
+      </c>
+      <c r="F71" t="str">
+        <v>11004</v>
+      </c>
+      <c r="G71" t="str">
+        <v>SBI Bank</v>
+      </c>
+      <c r="H71" t="str">
+        <v>Asset</v>
+      </c>
+      <c r="I71" t="str">
+        <v>Cash &amp; Bank</v>
+      </c>
+      <c r="J71" t="str">
+        <v>Bank</v>
+      </c>
+      <c r="K71" t="str">
+        <v>Bank</v>
+      </c>
+      <c r="L71" t="str">
+        <v>ACC-04</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L69"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L71"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I32"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -10773,9 +10934,38 @@
         <v>Hose cleaning</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>TXN-10033-L2</v>
+      </c>
+      <c r="B32" t="str">
+        <v>ACC-04</v>
+      </c>
+      <c r="C32" t="str">
+        <v>TXN-10033</v>
+      </c>
+      <c r="D32">
+        <v>2</v>
+      </c>
+      <c r="E32" t="str">
+        <v>2026-08-21</v>
+      </c>
+      <c r="F32">
+        <v>-104000</v>
+      </c>
+      <c r="G32" t="str">
+        <v>Cr</v>
+      </c>
+      <c r="H32" t="str">
+        <v>SBI Bank</v>
+      </c>
+      <c r="I32" t="str">
+        <v>Paid to vendor</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I32"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -11255,7 +11445,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -11307,16 +11497,45 @@
         <v>Narration</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>TXN-10033-L1</v>
+      </c>
+      <c r="B4" t="str">
+        <v>FA-01</v>
+      </c>
+      <c r="C4" t="str">
+        <v>TXN-10033</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4" t="str">
+        <v>2026-08-21</v>
+      </c>
+      <c r="F4">
+        <v>104000</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Dr</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Property / Land</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Paid to vendor</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -11468,9 +11687,35 @@
         <v>Wedding gold advance · Event type: Gold</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>TXN-10033-E</v>
+      </c>
+      <c r="B8" t="str">
+        <v>EVT-01</v>
+      </c>
+      <c r="C8" t="str">
+        <v>TXN-10033</v>
+      </c>
+      <c r="D8" t="str">
+        <v>2026-08-21</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="F8">
+        <v>104000</v>
+      </c>
+      <c r="G8" t="str">
+        <v>debit</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Paid to vendor</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-21T20:17:59.106Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -414,7 +414,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O36"/>
+  <dimension ref="A1:O37"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2041,9 +2041,56 @@
         <v>EVT-01</v>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>TXN-10034</v>
+      </c>
+      <c r="B37" t="str">
+        <v>2026-08-21</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Event settle</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Event settlement</v>
+      </c>
+      <c r="F37" t="str">
+        <v>Capitalise event: My Home Construction</v>
+      </c>
+      <c r="G37">
+        <v>165000</v>
+      </c>
+      <c r="H37" t="str">
+        <v/>
+      </c>
+      <c r="I37" t="str">
+        <v/>
+      </c>
+      <c r="J37" t="str">
+        <v>Event settle: EVT-01</v>
+      </c>
+      <c r="K37" t="str">
+        <v/>
+      </c>
+      <c r="L37" t="str">
+        <v/>
+      </c>
+      <c r="M37" t="str">
+        <v>[{"kind":"Ledger","acct":"14002","sub":"","dr":165000,"cr":0},{"kind":"Ledger","acct":"29001","sub":"","dr":0,"cr":165000}]</v>
+      </c>
+      <c r="N37" t="str">
+        <v/>
+      </c>
+      <c r="O37" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O37"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3463,7 +3510,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N7"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -3667,16 +3714,60 @@
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>FA-04</v>
+      </c>
+      <c r="B7" t="str">
+        <v>My Home Construction</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Other</v>
+      </c>
+      <c r="D7" t="str">
+        <v>2026-08-21</v>
+      </c>
+      <c r="E7">
+        <v>165000</v>
+      </c>
+      <c r="F7">
+        <v>165000</v>
+      </c>
+      <c r="G7" t="str">
+        <v>14002</v>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v>Active</v>
+      </c>
+      <c r="N7" t="str">
+        <v>From event EVT-01</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:M9"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -3687,7 +3778,10 @@
     <col min="7" max="7" width="9.83203125" customWidth="1"/>
     <col min="8" max="8" width="14.83203125" customWidth="1"/>
     <col min="9" max="9" width="16.83203125" customWidth="1"/>
-    <col min="10" max="10" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
+    <col min="11" max="11" width="12.83203125" customWidth="1"/>
+    <col min="12" max="12" width="13.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3697,7 +3791,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Recurring financial tasks and reminders — recharges, cleaning, maintenance, subscriptions — with next-due tracking. Financial ones post a voucher on pay.</v>
+        <v>Recurring financial tasks and reminders — recharges, cleaning, maintenance, subscriptions — with next-due tracking. Financial ones post a voucher on pay. Records last paid date &amp; amount; can be closed as one-off.</v>
       </c>
     </row>
     <row r="3">
@@ -3729,6 +3823,15 @@
         <v>Main Account</v>
       </c>
       <c r="J3" t="str">
+        <v>Last Paid</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Last Amount</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Record Status</v>
+      </c>
+      <c r="M3" t="str">
         <v>Note</v>
       </c>
     </row>
@@ -3761,6 +3864,15 @@
         <v>55008</v>
       </c>
       <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v>Open</v>
+      </c>
+      <c r="M4" t="str">
         <v>98xxx</v>
       </c>
     </row>
@@ -3793,6 +3905,15 @@
         <v/>
       </c>
       <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v>Open</v>
+      </c>
+      <c r="M5" t="str">
         <v>Ramesh</v>
       </c>
     </row>
@@ -3827,6 +3948,15 @@
       <c r="J6" t="str">
         <v/>
       </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v>Open</v>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -3857,6 +3987,15 @@
         <v/>
       </c>
       <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v>Open</v>
+      </c>
+      <c r="M7" t="str">
         <v>Full exterior</v>
       </c>
     </row>
@@ -3891,6 +4030,15 @@
       <c r="J8" t="str">
         <v/>
       </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v>Open</v>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -3921,12 +4069,21 @@
         <v>55005</v>
       </c>
       <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9" t="str">
+        <v/>
+      </c>
+      <c r="L9" t="str">
+        <v>Open</v>
+      </c>
+      <c r="M9" t="str">
         <v>Land Tax</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M9"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4031,13 +4188,13 @@
         <v>Karukutty plot</v>
       </c>
       <c r="I4" t="str">
-        <v>Open</v>
+        <v>Completed</v>
       </c>
       <c r="J4" t="str">
-        <v/>
+        <v>2026-08-21</v>
       </c>
       <c r="K4" t="str">
-        <v/>
+        <v>Event settle: EVT-01</v>
       </c>
       <c r="L4">
         <v>269000</v>
@@ -4102,7 +4259,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G71"/>
+  <dimension ref="A1:G72"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -4815,22 +4972,22 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>30001</v>
+        <v>29001</v>
       </c>
       <c r="B33" t="str">
-        <v>Opening Balances / Net Worth</v>
+        <v>Event WIP Clearing</v>
       </c>
       <c r="C33" t="str">
-        <v>Equity</v>
+        <v>Liability</v>
       </c>
       <c r="D33" t="str">
-        <v>Capital</v>
+        <v>Clearing</v>
       </c>
       <c r="E33" t="str">
-        <v>Opening Balance</v>
+        <v/>
       </c>
       <c r="F33" t="str">
-        <v/>
+        <v>event,wip</v>
       </c>
       <c r="G33" t="str">
         <v/>
@@ -4838,22 +4995,22 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>41001</v>
+        <v>30001</v>
       </c>
       <c r="B34" t="str">
-        <v>Salary</v>
+        <v>Opening Balances / Net Worth</v>
       </c>
       <c r="C34" t="str">
-        <v>Income</v>
+        <v>Equity</v>
       </c>
       <c r="D34" t="str">
-        <v>Employment</v>
+        <v>Capital</v>
       </c>
       <c r="E34" t="str">
-        <v>Monthly Salary</v>
+        <v>Opening Balance</v>
       </c>
       <c r="F34" t="str">
-        <v>salary,sal cr,infopark</v>
+        <v/>
       </c>
       <c r="G34" t="str">
         <v/>
@@ -4861,22 +5018,22 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>41002</v>
+        <v>41001</v>
       </c>
       <c r="B35" t="str">
-        <v>Business Income</v>
+        <v>Salary</v>
       </c>
       <c r="C35" t="str">
         <v>Income</v>
       </c>
       <c r="D35" t="str">
-        <v>Business</v>
+        <v>Employment</v>
       </c>
       <c r="E35" t="str">
-        <v>General</v>
+        <v>Monthly Salary</v>
       </c>
       <c r="F35" t="str">
-        <v>business</v>
+        <v>salary,sal cr,infopark</v>
       </c>
       <c r="G35" t="str">
         <v/>
@@ -4884,10 +5041,10 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>41003</v>
+        <v>41002</v>
       </c>
       <c r="B36" t="str">
-        <v>Freelance Income</v>
+        <v>Business Income</v>
       </c>
       <c r="C36" t="str">
         <v>Income</v>
@@ -4896,10 +5053,10 @@
         <v>Business</v>
       </c>
       <c r="E36" t="str">
-        <v>Freelance</v>
+        <v>General</v>
       </c>
       <c r="F36" t="str">
-        <v>freelance</v>
+        <v>business</v>
       </c>
       <c r="G36" t="str">
         <v/>
@@ -4907,22 +5064,22 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>41004</v>
+        <v>41003</v>
       </c>
       <c r="B37" t="str">
-        <v>Bonus &amp; Incentives</v>
+        <v>Freelance Income</v>
       </c>
       <c r="C37" t="str">
         <v>Income</v>
       </c>
       <c r="D37" t="str">
-        <v>Employment</v>
+        <v>Business</v>
       </c>
       <c r="E37" t="str">
-        <v>bonus</v>
+        <v>Freelance</v>
       </c>
       <c r="F37" t="str">
-        <v/>
+        <v>freelance</v>
       </c>
       <c r="G37" t="str">
         <v/>
@@ -4930,22 +5087,22 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>42001</v>
+        <v>41004</v>
       </c>
       <c r="B38" t="str">
-        <v>Interest Income</v>
+        <v>Bonus &amp; Incentives</v>
       </c>
       <c r="C38" t="str">
         <v>Income</v>
       </c>
       <c r="D38" t="str">
-        <v>Investment Income</v>
+        <v>Employment</v>
       </c>
       <c r="E38" t="str">
-        <v>Bank / FD Interest</v>
+        <v>bonus</v>
       </c>
       <c r="F38" t="str">
-        <v>interest,int.pd,sbint,sb int</v>
+        <v/>
       </c>
       <c r="G38" t="str">
         <v/>
@@ -4953,10 +5110,10 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>42002</v>
+        <v>42001</v>
       </c>
       <c r="B39" t="str">
-        <v>Dividend Income</v>
+        <v>Interest Income</v>
       </c>
       <c r="C39" t="str">
         <v>Income</v>
@@ -4965,10 +5122,10 @@
         <v>Investment Income</v>
       </c>
       <c r="E39" t="str">
-        <v>Dividends</v>
+        <v>Bank / FD Interest</v>
       </c>
       <c r="F39" t="str">
-        <v>dividend,div,achcr</v>
+        <v>interest,int.pd,sbint,sb int</v>
       </c>
       <c r="G39" t="str">
         <v/>
@@ -4976,22 +5133,22 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>43001</v>
+        <v>42002</v>
       </c>
       <c r="B40" t="str">
-        <v>Rental Income</v>
+        <v>Dividend Income</v>
       </c>
       <c r="C40" t="str">
         <v>Income</v>
       </c>
       <c r="D40" t="str">
-        <v>Other Income</v>
+        <v>Investment Income</v>
       </c>
       <c r="E40" t="str">
-        <v>Rent Received</v>
+        <v>Dividends</v>
       </c>
       <c r="F40" t="str">
-        <v>rent received</v>
+        <v>dividend,div,achcr</v>
       </c>
       <c r="G40" t="str">
         <v/>
@@ -4999,10 +5156,10 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>43002</v>
+        <v>43001</v>
       </c>
       <c r="B41" t="str">
-        <v>Gifts &amp; Allowance</v>
+        <v>Rental Income</v>
       </c>
       <c r="C41" t="str">
         <v>Income</v>
@@ -5011,10 +5168,10 @@
         <v>Other Income</v>
       </c>
       <c r="E41" t="str">
-        <v>Gifts</v>
+        <v>Rent Received</v>
       </c>
       <c r="F41" t="str">
-        <v>gift received</v>
+        <v>rent received</v>
       </c>
       <c r="G41" t="str">
         <v/>
@@ -5022,10 +5179,10 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>43003</v>
+        <v>43002</v>
       </c>
       <c r="B42" t="str">
-        <v>Debt Settlement Received</v>
+        <v>Gifts &amp; Allowance</v>
       </c>
       <c r="C42" t="str">
         <v>Income</v>
@@ -5034,10 +5191,10 @@
         <v>Other Income</v>
       </c>
       <c r="E42" t="str">
-        <v>Loan Repaid to You</v>
+        <v>Gifts</v>
       </c>
       <c r="F42" t="str">
-        <v>repayment</v>
+        <v>gift received</v>
       </c>
       <c r="G42" t="str">
         <v/>
@@ -5045,10 +5202,10 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>44001</v>
+        <v>43003</v>
       </c>
       <c r="B43" t="str">
-        <v>Cashback &amp; Rewards</v>
+        <v>Debt Settlement Received</v>
       </c>
       <c r="C43" t="str">
         <v>Income</v>
@@ -5057,10 +5214,10 @@
         <v>Other Income</v>
       </c>
       <c r="E43" t="str">
-        <v>cashback,reward</v>
+        <v>Loan Repaid to You</v>
       </c>
       <c r="F43" t="str">
-        <v/>
+        <v>repayment</v>
       </c>
       <c r="G43" t="str">
         <v/>
@@ -5068,10 +5225,10 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>49999</v>
+        <v>44001</v>
       </c>
       <c r="B44" t="str">
-        <v>Other Income</v>
+        <v>Cashback &amp; Rewards</v>
       </c>
       <c r="C44" t="str">
         <v>Income</v>
@@ -5080,7 +5237,7 @@
         <v>Other Income</v>
       </c>
       <c r="E44" t="str">
-        <v>Miscellaneous</v>
+        <v>cashback,reward</v>
       </c>
       <c r="F44" t="str">
         <v/>
@@ -5091,22 +5248,22 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>51001</v>
+        <v>49999</v>
       </c>
       <c r="B45" t="str">
-        <v>Rent / Housing</v>
+        <v>Other Income</v>
       </c>
       <c r="C45" t="str">
-        <v>Expense</v>
+        <v>Income</v>
       </c>
       <c r="D45" t="str">
-        <v>Household</v>
+        <v>Other Income</v>
       </c>
       <c r="E45" t="str">
-        <v>Rent &amp; Maintenance</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="F45" t="str">
-        <v>rent,maintenance</v>
+        <v/>
       </c>
       <c r="G45" t="str">
         <v/>
@@ -5114,10 +5271,10 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>51002</v>
+        <v>51001</v>
       </c>
       <c r="B46" t="str">
-        <v>Utilities - Electricity &amp; Water</v>
+        <v>Rent / Housing</v>
       </c>
       <c r="C46" t="str">
         <v>Expense</v>
@@ -5126,10 +5283,10 @@
         <v>Household</v>
       </c>
       <c r="E46" t="str">
-        <v>Electricity / Water</v>
+        <v>Rent &amp; Maintenance</v>
       </c>
       <c r="F46" t="str">
-        <v>kseb,electricity,water bill</v>
+        <v>rent,maintenance</v>
       </c>
       <c r="G46" t="str">
         <v/>
@@ -5137,10 +5294,10 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>51003</v>
+        <v>51002</v>
       </c>
       <c r="B47" t="str">
-        <v>Utilities - Internet &amp; Mobile</v>
+        <v>Utilities - Electricity &amp; Water</v>
       </c>
       <c r="C47" t="str">
         <v>Expense</v>
@@ -5149,10 +5306,10 @@
         <v>Household</v>
       </c>
       <c r="E47" t="str">
-        <v>Recharge / Broadband</v>
+        <v>Electricity / Water</v>
       </c>
       <c r="F47" t="str">
-        <v>recharge,airtel,jio,bsnl,broadband,wifi</v>
+        <v>kseb,electricity,water bill</v>
       </c>
       <c r="G47" t="str">
         <v/>
@@ -5160,10 +5317,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>51004</v>
+        <v>51003</v>
       </c>
       <c r="B48" t="str">
-        <v>Gas / LPG</v>
+        <v>Utilities - Internet &amp; Mobile</v>
       </c>
       <c r="C48" t="str">
         <v>Expense</v>
@@ -5172,10 +5329,10 @@
         <v>Household</v>
       </c>
       <c r="E48" t="str">
-        <v>Cooking Gas</v>
+        <v>Recharge / Broadband</v>
       </c>
       <c r="F48" t="str">
-        <v>lpg,indane,gas</v>
+        <v>recharge,airtel,jio,bsnl,broadband,wifi</v>
       </c>
       <c r="G48" t="str">
         <v/>
@@ -5183,10 +5340,10 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>51005</v>
+        <v>51004</v>
       </c>
       <c r="B49" t="str">
-        <v>Household Appliances</v>
+        <v>Gas / LPG</v>
       </c>
       <c r="C49" t="str">
         <v>Expense</v>
@@ -5195,10 +5352,10 @@
         <v>Household</v>
       </c>
       <c r="E49" t="str">
-        <v>Appliances &amp; Repairs</v>
+        <v>Cooking Gas</v>
       </c>
       <c r="F49" t="str">
-        <v>washing machine,appliance,repair</v>
+        <v>lpg,indane,gas</v>
       </c>
       <c r="G49" t="str">
         <v/>
@@ -5206,22 +5363,22 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>52001</v>
+        <v>51005</v>
       </c>
       <c r="B50" t="str">
-        <v>Groceries</v>
+        <v>Household Appliances</v>
       </c>
       <c r="C50" t="str">
         <v>Expense</v>
       </c>
       <c r="D50" t="str">
-        <v>Food</v>
+        <v>Household</v>
       </c>
       <c r="E50" t="str">
-        <v>Provisions</v>
+        <v>Appliances &amp; Repairs</v>
       </c>
       <c r="F50" t="str">
-        <v>grocery,supermarket,mart,bigbasket,blinkit,zepto,dmart</v>
+        <v>washing machine,appliance,repair</v>
       </c>
       <c r="G50" t="str">
         <v/>
@@ -5229,10 +5386,10 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>52002</v>
+        <v>52001</v>
       </c>
       <c r="B51" t="str">
-        <v>Dining Out</v>
+        <v>Groceries</v>
       </c>
       <c r="C51" t="str">
         <v>Expense</v>
@@ -5241,10 +5398,10 @@
         <v>Food</v>
       </c>
       <c r="E51" t="str">
-        <v>Restaurants &amp; Delivery</v>
+        <v>Provisions</v>
       </c>
       <c r="F51" t="str">
-        <v>swiggy,zomato,restaurant,hotel,cafe</v>
+        <v>grocery,supermarket,mart,bigbasket,blinkit,zepto,dmart</v>
       </c>
       <c r="G51" t="str">
         <v/>
@@ -5252,10 +5409,10 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>52003</v>
+        <v>52002</v>
       </c>
       <c r="B52" t="str">
-        <v>Snacks &amp; Beverages</v>
+        <v>Dining Out</v>
       </c>
       <c r="C52" t="str">
         <v>Expense</v>
@@ -5264,10 +5421,10 @@
         <v>Food</v>
       </c>
       <c r="E52" t="str">
-        <v>snacks,tea,coffee</v>
+        <v>Restaurants &amp; Delivery</v>
       </c>
       <c r="F52" t="str">
-        <v/>
+        <v>swiggy,zomato,restaurant,hotel,cafe</v>
       </c>
       <c r="G52" t="str">
         <v/>
@@ -5275,22 +5432,22 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>53001</v>
+        <v>52003</v>
       </c>
       <c r="B53" t="str">
-        <v>Transport &amp; Fuel</v>
+        <v>Snacks &amp; Beverages</v>
       </c>
       <c r="C53" t="str">
         <v>Expense</v>
       </c>
       <c r="D53" t="str">
-        <v>Transport</v>
+        <v>Food</v>
       </c>
       <c r="E53" t="str">
-        <v>Fuel / Taxi / Toll</v>
+        <v>snacks,tea,coffee</v>
       </c>
       <c r="F53" t="str">
-        <v>uber,ola,rapido,petrol,fuel,hpcl,bpcl,fastag</v>
+        <v/>
       </c>
       <c r="G53" t="str">
         <v/>
@@ -5298,10 +5455,10 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>53002</v>
+        <v>53001</v>
       </c>
       <c r="B54" t="str">
-        <v>Travel</v>
+        <v>Transport &amp; Fuel</v>
       </c>
       <c r="C54" t="str">
         <v>Expense</v>
@@ -5310,10 +5467,10 @@
         <v>Transport</v>
       </c>
       <c r="E54" t="str">
-        <v>Trips &amp; Tickets</v>
+        <v>Fuel / Taxi / Toll</v>
       </c>
       <c r="F54" t="str">
-        <v>irctc,makemytrip,redbus,indigo</v>
+        <v>uber,ola,rapido,petrol,fuel,hpcl,bpcl,fastag</v>
       </c>
       <c r="G54" t="str">
         <v/>
@@ -5321,10 +5478,10 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>53003</v>
+        <v>53002</v>
       </c>
       <c r="B55" t="str">
-        <v>Vehicle Maintenance</v>
+        <v>Travel</v>
       </c>
       <c r="C55" t="str">
         <v>Expense</v>
@@ -5333,10 +5490,10 @@
         <v>Transport</v>
       </c>
       <c r="E55" t="str">
-        <v>service,repair</v>
+        <v>Trips &amp; Tickets</v>
       </c>
       <c r="F55" t="str">
-        <v/>
+        <v>irctc,makemytrip,redbus,indigo</v>
       </c>
       <c r="G55" t="str">
         <v/>
@@ -5344,22 +5501,22 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>54001</v>
+        <v>53003</v>
       </c>
       <c r="B56" t="str">
-        <v>Family Support</v>
+        <v>Vehicle Maintenance</v>
       </c>
       <c r="C56" t="str">
         <v>Expense</v>
       </c>
       <c r="D56" t="str">
-        <v>Family &amp; Personal</v>
+        <v>Transport</v>
       </c>
       <c r="E56" t="str">
-        <v>Family / Amma</v>
+        <v>service,repair</v>
       </c>
       <c r="F56" t="str">
-        <v>amma,family</v>
+        <v/>
       </c>
       <c r="G56" t="str">
         <v/>
@@ -5367,10 +5524,10 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>54002</v>
+        <v>54001</v>
       </c>
       <c r="B57" t="str">
-        <v>Health &amp; Medical</v>
+        <v>Family Support</v>
       </c>
       <c r="C57" t="str">
         <v>Expense</v>
@@ -5379,10 +5536,10 @@
         <v>Family &amp; Personal</v>
       </c>
       <c r="E57" t="str">
-        <v>Pharmacy / Hospital</v>
+        <v>Family / Amma</v>
       </c>
       <c r="F57" t="str">
-        <v>pharmacy,medical,hospital,clinic</v>
+        <v>amma,family</v>
       </c>
       <c r="G57" t="str">
         <v/>
@@ -5390,10 +5547,10 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>54003</v>
+        <v>54002</v>
       </c>
       <c r="B58" t="str">
-        <v>Education</v>
+        <v>Health &amp; Medical</v>
       </c>
       <c r="C58" t="str">
         <v>Expense</v>
@@ -5402,10 +5559,10 @@
         <v>Family &amp; Personal</v>
       </c>
       <c r="E58" t="str">
-        <v>Fees &amp; Courses</v>
+        <v>Pharmacy / Hospital</v>
       </c>
       <c r="F58" t="str">
-        <v>school,college,course,tuition</v>
+        <v>pharmacy,medical,hospital,clinic</v>
       </c>
       <c r="G58" t="str">
         <v/>
@@ -5413,10 +5570,10 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>54004</v>
+        <v>54003</v>
       </c>
       <c r="B59" t="str">
-        <v>Shopping</v>
+        <v>Education</v>
       </c>
       <c r="C59" t="str">
         <v>Expense</v>
@@ -5425,10 +5582,10 @@
         <v>Family &amp; Personal</v>
       </c>
       <c r="E59" t="str">
-        <v>Online &amp; Retail</v>
+        <v>Fees &amp; Courses</v>
       </c>
       <c r="F59" t="str">
-        <v>amazon,flipkart,myntra,ajio</v>
+        <v>school,college,course,tuition</v>
       </c>
       <c r="G59" t="str">
         <v/>
@@ -5436,10 +5593,10 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>54005</v>
+        <v>54004</v>
       </c>
       <c r="B60" t="str">
-        <v>Gifts &amp; Functions</v>
+        <v>Shopping</v>
       </c>
       <c r="C60" t="str">
         <v>Expense</v>
@@ -5448,10 +5605,10 @@
         <v>Family &amp; Personal</v>
       </c>
       <c r="E60" t="str">
-        <v>Guests &amp; Gifts</v>
+        <v>Online &amp; Retail</v>
       </c>
       <c r="F60" t="str">
-        <v>guest,marriage,function</v>
+        <v>amazon,flipkart,myntra,ajio</v>
       </c>
       <c r="G60" t="str">
         <v/>
@@ -5459,10 +5616,10 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>54006</v>
+        <v>54005</v>
       </c>
       <c r="B61" t="str">
-        <v>Entertainment &amp; Subscriptions</v>
+        <v>Gifts &amp; Functions</v>
       </c>
       <c r="C61" t="str">
         <v>Expense</v>
@@ -5471,10 +5628,10 @@
         <v>Family &amp; Personal</v>
       </c>
       <c r="E61" t="str">
-        <v>netflix,spotify,prime</v>
+        <v>Guests &amp; Gifts</v>
       </c>
       <c r="F61" t="str">
-        <v/>
+        <v>guest,marriage,function</v>
       </c>
       <c r="G61" t="str">
         <v/>
@@ -5482,10 +5639,10 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>54007</v>
+        <v>54006</v>
       </c>
       <c r="B62" t="str">
-        <v>Personal Care</v>
+        <v>Entertainment &amp; Subscriptions</v>
       </c>
       <c r="C62" t="str">
         <v>Expense</v>
@@ -5494,7 +5651,7 @@
         <v>Family &amp; Personal</v>
       </c>
       <c r="E62" t="str">
-        <v>salon,grooming</v>
+        <v>netflix,spotify,prime</v>
       </c>
       <c r="F62" t="str">
         <v/>
@@ -5505,22 +5662,22 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>55001</v>
+        <v>54007</v>
       </c>
       <c r="B63" t="str">
-        <v>Loan EMI / Repayment</v>
+        <v>Personal Care</v>
       </c>
       <c r="C63" t="str">
         <v>Expense</v>
       </c>
       <c r="D63" t="str">
-        <v>Financial</v>
+        <v>Family &amp; Personal</v>
       </c>
       <c r="E63" t="str">
-        <v>EMIs</v>
+        <v>salon,grooming</v>
       </c>
       <c r="F63" t="str">
-        <v>emi,loan repay</v>
+        <v/>
       </c>
       <c r="G63" t="str">
         <v/>
@@ -5528,10 +5685,10 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>55002</v>
+        <v>55001</v>
       </c>
       <c r="B64" t="str">
-        <v>Credit Card Payment</v>
+        <v>Loan EMI / Repayment</v>
       </c>
       <c r="C64" t="str">
         <v>Expense</v>
@@ -5540,10 +5697,10 @@
         <v>Financial</v>
       </c>
       <c r="E64" t="str">
-        <v>Card Bills</v>
+        <v>EMIs</v>
       </c>
       <c r="F64" t="str">
-        <v>cc payment,card payment</v>
+        <v>emi,loan repay</v>
       </c>
       <c r="G64" t="str">
         <v/>
@@ -5551,10 +5708,10 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>55003</v>
+        <v>55002</v>
       </c>
       <c r="B65" t="str">
-        <v>Investment Contribution</v>
+        <v>Credit Card Payment</v>
       </c>
       <c r="C65" t="str">
         <v>Expense</v>
@@ -5563,10 +5720,10 @@
         <v>Financial</v>
       </c>
       <c r="E65" t="str">
-        <v>SIP / Deposits</v>
+        <v>Card Bills</v>
       </c>
       <c r="F65" t="str">
-        <v>sip</v>
+        <v>cc payment,card payment</v>
       </c>
       <c r="G65" t="str">
         <v/>
@@ -5574,10 +5731,10 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>55004</v>
+        <v>55003</v>
       </c>
       <c r="B66" t="str">
-        <v>Debt Given (Lent Out)</v>
+        <v>Investment Contribution</v>
       </c>
       <c r="C66" t="str">
         <v>Expense</v>
@@ -5586,10 +5743,10 @@
         <v>Financial</v>
       </c>
       <c r="E66" t="str">
-        <v>Money Lent</v>
+        <v>SIP / Deposits</v>
       </c>
       <c r="F66" t="str">
-        <v>lent to</v>
+        <v>sip</v>
       </c>
       <c r="G66" t="str">
         <v/>
@@ -5597,10 +5754,10 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>55005</v>
+        <v>55004</v>
       </c>
       <c r="B67" t="str">
-        <v>Taxes &amp; GST</v>
+        <v>Debt Given (Lent Out)</v>
       </c>
       <c r="C67" t="str">
         <v>Expense</v>
@@ -5609,10 +5766,10 @@
         <v>Financial</v>
       </c>
       <c r="E67" t="str">
-        <v>GST / Filing</v>
+        <v>Money Lent</v>
       </c>
       <c r="F67" t="str">
-        <v>gst,filing fee,tax</v>
+        <v>lent to</v>
       </c>
       <c r="G67" t="str">
         <v/>
@@ -5620,10 +5777,10 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>55006</v>
+        <v>55005</v>
       </c>
       <c r="B68" t="str">
-        <v>Insurance</v>
+        <v>Taxes &amp; GST</v>
       </c>
       <c r="C68" t="str">
         <v>Expense</v>
@@ -5632,10 +5789,10 @@
         <v>Financial</v>
       </c>
       <c r="E68" t="str">
-        <v>Premiums</v>
+        <v>GST / Filing</v>
       </c>
       <c r="F68" t="str">
-        <v>insurance,lic,premium</v>
+        <v>gst,filing fee,tax</v>
       </c>
       <c r="G68" t="str">
         <v/>
@@ -5643,10 +5800,10 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>55007</v>
+        <v>55006</v>
       </c>
       <c r="B69" t="str">
-        <v>Bank Charges &amp; Fees</v>
+        <v>Insurance</v>
       </c>
       <c r="C69" t="str">
         <v>Expense</v>
@@ -5655,10 +5812,10 @@
         <v>Financial</v>
       </c>
       <c r="E69" t="str">
-        <v>charges,fee</v>
+        <v>Premiums</v>
       </c>
       <c r="F69" t="str">
-        <v/>
+        <v>insurance,lic,premium</v>
       </c>
       <c r="G69" t="str">
         <v/>
@@ -5666,10 +5823,10 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>55008</v>
+        <v>55007</v>
       </c>
       <c r="B70" t="str">
-        <v>Interest Expense</v>
+        <v>Bank Charges &amp; Fees</v>
       </c>
       <c r="C70" t="str">
         <v>Expense</v>
@@ -5678,7 +5835,7 @@
         <v>Financial</v>
       </c>
       <c r="E70" t="str">
-        <v>interest</v>
+        <v>charges,fee</v>
       </c>
       <c r="F70" t="str">
         <v/>
@@ -5689,30 +5846,53 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>59999</v>
+        <v>55008</v>
       </c>
       <c r="B71" t="str">
-        <v>Other Expenses</v>
+        <v>Interest Expense</v>
       </c>
       <c r="C71" t="str">
         <v>Expense</v>
       </c>
       <c r="D71" t="str">
+        <v>Financial</v>
+      </c>
+      <c r="E71" t="str">
+        <v>interest</v>
+      </c>
+      <c r="F71" t="str">
+        <v/>
+      </c>
+      <c r="G71" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>59999</v>
+      </c>
+      <c r="B72" t="str">
+        <v>Other Expenses</v>
+      </c>
+      <c r="C72" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D72" t="str">
         <v>Other</v>
       </c>
-      <c r="E71" t="str">
+      <c r="E72" t="str">
         <v>Miscellaneous</v>
       </c>
-      <c r="F71" t="str">
-        <v/>
-      </c>
-      <c r="G71" t="str">
+      <c r="F72" t="str">
+        <v/>
+      </c>
+      <c r="G72" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G71"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G72"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6086,7 +6266,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L37"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -7404,16 +7584,54 @@
         <v>Yes</v>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>TXN-10034</v>
+      </c>
+      <c r="B37" t="str">
+        <v>2026-08-21</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Event settle</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Capitalise event: My Home Construction</v>
+      </c>
+      <c r="F37">
+        <v>165000</v>
+      </c>
+      <c r="G37" t="str">
+        <v/>
+      </c>
+      <c r="H37" t="str">
+        <v/>
+      </c>
+      <c r="I37" t="str">
+        <v>Event settle: EVT-01</v>
+      </c>
+      <c r="J37" t="str">
+        <v/>
+      </c>
+      <c r="K37">
+        <v>2</v>
+      </c>
+      <c r="L37" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L37"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L71"/>
+  <dimension ref="A1:L73"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -10061,9 +10279,85 @@
         <v>ACC-04</v>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>TXN-10034-L1</v>
+      </c>
+      <c r="B72" t="str">
+        <v>TXN-10034</v>
+      </c>
+      <c r="C72">
+        <v>1</v>
+      </c>
+      <c r="D72">
+        <v>165000</v>
+      </c>
+      <c r="E72" t="str">
+        <v>Dr</v>
+      </c>
+      <c r="F72" t="str">
+        <v>14002</v>
+      </c>
+      <c r="G72" t="str">
+        <v>Property / Land</v>
+      </c>
+      <c r="H72" t="str">
+        <v>Asset</v>
+      </c>
+      <c r="I72" t="str">
+        <v>Fixed Assets</v>
+      </c>
+      <c r="J72" t="str">
+        <v>Ledger</v>
+      </c>
+      <c r="K72" t="str">
+        <v>Fixed Asset</v>
+      </c>
+      <c r="L72" t="str">
+        <v>FA-01</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>TXN-10034-L2</v>
+      </c>
+      <c r="B73" t="str">
+        <v>TXN-10034</v>
+      </c>
+      <c r="C73">
+        <v>2</v>
+      </c>
+      <c r="D73">
+        <v>-165000</v>
+      </c>
+      <c r="E73" t="str">
+        <v>Cr</v>
+      </c>
+      <c r="F73" t="str">
+        <v>29001</v>
+      </c>
+      <c r="G73" t="str">
+        <v>Event WIP Clearing</v>
+      </c>
+      <c r="H73" t="str">
+        <v>Liability</v>
+      </c>
+      <c r="I73" t="str">
+        <v>Clearing</v>
+      </c>
+      <c r="J73" t="str">
+        <v>Ledger</v>
+      </c>
+      <c r="K73" t="str">
+        <v/>
+      </c>
+      <c r="L73" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L71"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L73"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -11445,7 +11739,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -11526,9 +11820,38 @@
         <v>Paid to vendor</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>TXN-10034-L1</v>
+      </c>
+      <c r="B5" t="str">
+        <v>FA-01</v>
+      </c>
+      <c r="C5" t="str">
+        <v>TXN-10034</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5" t="str">
+        <v>2026-08-21</v>
+      </c>
+      <c r="F5">
+        <v>165000</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Dr</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Property / Land</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Capitalise event: My Home Construction</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-21T20:53:18.027Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -414,7 +414,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O33"/>
+  <dimension ref="A1:O34"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1900,9 +1900,56 @@
         <v>EVT-01</v>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>TXN-10031</v>
+      </c>
+      <c r="B34" t="str">
+        <v>2026-08-07</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Commitment</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Interest Expense</v>
+      </c>
+      <c r="F34" t="str">
+        <v/>
+      </c>
+      <c r="G34">
+        <v>400</v>
+      </c>
+      <c r="H34" t="str">
+        <v/>
+      </c>
+      <c r="I34" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="J34" t="str">
+        <v>Commitment: CM-01</v>
+      </c>
+      <c r="K34" t="str">
+        <v/>
+      </c>
+      <c r="L34" t="str">
+        <v/>
+      </c>
+      <c r="M34" t="str">
+        <v>[{"kind":"Commitment","acct":"55008","sub":"cm:CM-01","cat":"","dr":400,"cr":0},{"kind":"Bank","acct":"23002","sub":"bank:ICICI Amazon Card","cat":"","dr":0,"cr":400}]</v>
+      </c>
+      <c r="N34" t="str">
+        <v/>
+      </c>
+      <c r="O34" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O34"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2259,10 +2306,10 @@
         <v>3373</v>
       </c>
       <c r="G9">
-        <v>46029</v>
+        <v>46429</v>
       </c>
       <c r="H9">
-        <v>42656</v>
+        <v>43056</v>
       </c>
       <c r="I9" t="str">
         <v/>
@@ -3617,7 +3664,7 @@
         <v>Monthly</v>
       </c>
       <c r="E4" t="str">
-        <v>2026-08-25</v>
+        <v>2026-09-25</v>
       </c>
       <c r="F4">
         <v>399</v>
@@ -5960,7 +6007,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L34"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -7164,16 +7211,54 @@
         <v>Yes</v>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>TXN-10031</v>
+      </c>
+      <c r="B34" t="str">
+        <v>2026-08-07</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Commitment</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Interest Expense</v>
+      </c>
+      <c r="F34">
+        <v>400</v>
+      </c>
+      <c r="G34" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="H34" t="str">
+        <v/>
+      </c>
+      <c r="I34" t="str">
+        <v>Commitment: CM-01</v>
+      </c>
+      <c r="J34" t="str">
+        <v/>
+      </c>
+      <c r="K34">
+        <v>2</v>
+      </c>
+      <c r="L34" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L34"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L65"/>
+  <dimension ref="A1:L67"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -9593,9 +9678,85 @@
         <v>ACC-03</v>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>TXN-10031-L1</v>
+      </c>
+      <c r="B66" t="str">
+        <v>TXN-10031</v>
+      </c>
+      <c r="C66">
+        <v>1</v>
+      </c>
+      <c r="D66">
+        <v>400</v>
+      </c>
+      <c r="E66" t="str">
+        <v>Dr</v>
+      </c>
+      <c r="F66" t="str">
+        <v>55008</v>
+      </c>
+      <c r="G66" t="str">
+        <v>Interest Expense</v>
+      </c>
+      <c r="H66" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="I66" t="str">
+        <v>Financial</v>
+      </c>
+      <c r="J66" t="str">
+        <v>Commitment</v>
+      </c>
+      <c r="K66" t="str">
+        <v/>
+      </c>
+      <c r="L66" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>TXN-10031-L2</v>
+      </c>
+      <c r="B67" t="str">
+        <v>TXN-10031</v>
+      </c>
+      <c r="C67">
+        <v>2</v>
+      </c>
+      <c r="D67">
+        <v>-400</v>
+      </c>
+      <c r="E67" t="str">
+        <v>Cr</v>
+      </c>
+      <c r="F67" t="str">
+        <v>23002</v>
+      </c>
+      <c r="G67" t="str">
+        <v>ICICI Amazon Card</v>
+      </c>
+      <c r="H67" t="str">
+        <v>Liability</v>
+      </c>
+      <c r="I67" t="str">
+        <v>Credit Cards</v>
+      </c>
+      <c r="J67" t="str">
+        <v>Bank</v>
+      </c>
+      <c r="K67" t="str">
+        <v>Card</v>
+      </c>
+      <c r="L67" t="str">
+        <v>CARD-01</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L65"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L67"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -10446,7 +10607,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -10643,9 +10804,38 @@
         <v>Bought gadget - split with Baby</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>TXN-10031-L2</v>
+      </c>
+      <c r="B9" t="str">
+        <v>CARD-01</v>
+      </c>
+      <c r="C9" t="str">
+        <v>TXN-10031</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9" t="str">
+        <v>2026-08-07</v>
+      </c>
+      <c r="F9">
+        <v>-400</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Cr</v>
+      </c>
+      <c r="H9" t="str">
+        <v>ICICI Amazon Card</v>
+      </c>
+      <c r="I9" t="str">
+        <v>Interest Expense</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I9"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-21T21:11:07.807Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -414,7 +414,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O34"/>
+  <dimension ref="A1:O35"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1947,9 +1947,56 @@
         <v/>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>TXN-10032</v>
+      </c>
+      <c r="B35" t="str">
+        <v>2026-08-22</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Commitment</v>
+      </c>
+      <c r="E35" t="str">
+        <v>CM</v>
+      </c>
+      <c r="F35" t="str">
+        <v/>
+      </c>
+      <c r="G35">
+        <v>100</v>
+      </c>
+      <c r="H35" t="str">
+        <v/>
+      </c>
+      <c r="I35" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="J35" t="str">
+        <v>Commitment: CM-02</v>
+      </c>
+      <c r="K35" t="str">
+        <v/>
+      </c>
+      <c r="L35" t="str">
+        <v/>
+      </c>
+      <c r="M35" t="str">
+        <v>[{"kind":"Commitment","acct":"CM","sub":"cm:CM-02","cat":"","dr":100,"cr":0},{"kind":"Bank","acct":"11002","sub":"bank:HDFC-Aluva","cat":"","dr":0,"cr":100}]</v>
+      </c>
+      <c r="N35" t="str">
+        <v/>
+      </c>
+      <c r="O35" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O35"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2106,10 +2153,10 @@
         <v>0</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H5">
-        <v>20000</v>
+        <v>19900</v>
       </c>
       <c r="I5" t="str">
         <v/>
@@ -3720,10 +3767,10 @@
         <v/>
       </c>
       <c r="J5" t="str">
-        <v/>
-      </c>
-      <c r="K5" t="str">
-        <v/>
+        <v>2026-08-22</v>
+      </c>
+      <c r="K5">
+        <v>100</v>
       </c>
       <c r="L5" t="str">
         <v>Open</v>
@@ -6007,7 +6054,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L35"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -7249,16 +7296,54 @@
         <v>Yes</v>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>TXN-10032</v>
+      </c>
+      <c r="B35" t="str">
+        <v>2026-08-22</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Commitment</v>
+      </c>
+      <c r="E35" t="str">
+        <v>CM</v>
+      </c>
+      <c r="F35">
+        <v>100</v>
+      </c>
+      <c r="G35" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="H35" t="str">
+        <v/>
+      </c>
+      <c r="I35" t="str">
+        <v>Commitment: CM-02</v>
+      </c>
+      <c r="J35" t="str">
+        <v/>
+      </c>
+      <c r="K35">
+        <v>2</v>
+      </c>
+      <c r="L35" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L35"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L67"/>
+  <dimension ref="A1:L69"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -9754,16 +9839,92 @@
         <v>CARD-01</v>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>TXN-10032-L1</v>
+      </c>
+      <c r="B68" t="str">
+        <v>TXN-10032</v>
+      </c>
+      <c r="C68">
+        <v>1</v>
+      </c>
+      <c r="D68">
+        <v>100</v>
+      </c>
+      <c r="E68" t="str">
+        <v>Dr</v>
+      </c>
+      <c r="F68" t="str">
+        <v>CM</v>
+      </c>
+      <c r="G68" t="str">
+        <v>House cleaning</v>
+      </c>
+      <c r="H68" t="str">
+        <v/>
+      </c>
+      <c r="I68" t="str">
+        <v/>
+      </c>
+      <c r="J68" t="str">
+        <v>Commitment</v>
+      </c>
+      <c r="K68" t="str">
+        <v/>
+      </c>
+      <c r="L68" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>TXN-10032-L2</v>
+      </c>
+      <c r="B69" t="str">
+        <v>TXN-10032</v>
+      </c>
+      <c r="C69">
+        <v>2</v>
+      </c>
+      <c r="D69">
+        <v>-100</v>
+      </c>
+      <c r="E69" t="str">
+        <v>Cr</v>
+      </c>
+      <c r="F69" t="str">
+        <v>11002</v>
+      </c>
+      <c r="G69" t="str">
+        <v>HDFC-Aluva Bank</v>
+      </c>
+      <c r="H69" t="str">
+        <v>Asset</v>
+      </c>
+      <c r="I69" t="str">
+        <v>Cash &amp; Bank</v>
+      </c>
+      <c r="J69" t="str">
+        <v>Bank</v>
+      </c>
+      <c r="K69" t="str">
+        <v>Bank</v>
+      </c>
+      <c r="L69" t="str">
+        <v>ACC-02</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L67"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L69"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I31"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -10598,9 +10759,38 @@
         <v>Expense for the well</v>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>TXN-10032-L2</v>
+      </c>
+      <c r="B31" t="str">
+        <v>ACC-02</v>
+      </c>
+      <c r="C31" t="str">
+        <v>TXN-10032</v>
+      </c>
+      <c r="D31">
+        <v>2</v>
+      </c>
+      <c r="E31" t="str">
+        <v>2026-08-22</v>
+      </c>
+      <c r="F31">
+        <v>-100</v>
+      </c>
+      <c r="G31" t="str">
+        <v>Cr</v>
+      </c>
+      <c r="H31" t="str">
+        <v>HDFC-Aluva Bank</v>
+      </c>
+      <c r="I31" t="str">
+        <v>CM</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I30"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I31"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-21T21:11:42.650Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -414,7 +414,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O35"/>
+  <dimension ref="A1:O36"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1994,9 +1994,56 @@
         <v/>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>TXN-10033</v>
+      </c>
+      <c r="B36" t="str">
+        <v>2026-08-21</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Commitment</v>
+      </c>
+      <c r="E36" t="str">
+        <v>CM</v>
+      </c>
+      <c r="F36" t="str">
+        <v/>
+      </c>
+      <c r="G36">
+        <v>500</v>
+      </c>
+      <c r="H36" t="str">
+        <v/>
+      </c>
+      <c r="I36" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="J36" t="str">
+        <v>Commitment: CM-02</v>
+      </c>
+      <c r="K36" t="str">
+        <v/>
+      </c>
+      <c r="L36" t="str">
+        <v/>
+      </c>
+      <c r="M36" t="str">
+        <v>[{"kind":"Commitment","acct":"CM","sub":"cm:CM-02","cat":"","dr":500,"cr":0},{"kind":"Bank","acct":"11002","sub":"bank:HDFC-Aluva","cat":"","dr":0,"cr":500}]</v>
+      </c>
+      <c r="N36" t="str">
+        <v/>
+      </c>
+      <c r="O36" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O36"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2153,10 +2200,10 @@
         <v>0</v>
       </c>
       <c r="G5">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="H5">
-        <v>19900</v>
+        <v>19400</v>
       </c>
       <c r="I5" t="str">
         <v/>
@@ -3752,7 +3799,7 @@
         <v>Weekly</v>
       </c>
       <c r="E5" t="str">
-        <v>2026-08-23</v>
+        <v>2026-08-30</v>
       </c>
       <c r="F5">
         <v>500</v>
@@ -3767,10 +3814,10 @@
         <v/>
       </c>
       <c r="J5" t="str">
-        <v>2026-08-22</v>
+        <v>2026-08-21</v>
       </c>
       <c r="K5">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="L5" t="str">
         <v>Open</v>
@@ -6054,7 +6101,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L36"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -7334,16 +7381,54 @@
         <v>Yes</v>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>TXN-10033</v>
+      </c>
+      <c r="B36" t="str">
+        <v>2026-08-21</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Commitment</v>
+      </c>
+      <c r="E36" t="str">
+        <v>CM</v>
+      </c>
+      <c r="F36">
+        <v>500</v>
+      </c>
+      <c r="G36" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="H36" t="str">
+        <v/>
+      </c>
+      <c r="I36" t="str">
+        <v>Commitment: CM-02</v>
+      </c>
+      <c r="J36" t="str">
+        <v/>
+      </c>
+      <c r="K36">
+        <v>2</v>
+      </c>
+      <c r="L36" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L36"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L69"/>
+  <dimension ref="A1:L71"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -9915,16 +10000,92 @@
         <v>ACC-02</v>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>TXN-10033-L1</v>
+      </c>
+      <c r="B70" t="str">
+        <v>TXN-10033</v>
+      </c>
+      <c r="C70">
+        <v>1</v>
+      </c>
+      <c r="D70">
+        <v>500</v>
+      </c>
+      <c r="E70" t="str">
+        <v>Dr</v>
+      </c>
+      <c r="F70" t="str">
+        <v>CM</v>
+      </c>
+      <c r="G70" t="str">
+        <v>House cleaning</v>
+      </c>
+      <c r="H70" t="str">
+        <v/>
+      </c>
+      <c r="I70" t="str">
+        <v/>
+      </c>
+      <c r="J70" t="str">
+        <v>Commitment</v>
+      </c>
+      <c r="K70" t="str">
+        <v/>
+      </c>
+      <c r="L70" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>TXN-10033-L2</v>
+      </c>
+      <c r="B71" t="str">
+        <v>TXN-10033</v>
+      </c>
+      <c r="C71">
+        <v>2</v>
+      </c>
+      <c r="D71">
+        <v>-500</v>
+      </c>
+      <c r="E71" t="str">
+        <v>Cr</v>
+      </c>
+      <c r="F71" t="str">
+        <v>11002</v>
+      </c>
+      <c r="G71" t="str">
+        <v>HDFC-Aluva Bank</v>
+      </c>
+      <c r="H71" t="str">
+        <v>Asset</v>
+      </c>
+      <c r="I71" t="str">
+        <v>Cash &amp; Bank</v>
+      </c>
+      <c r="J71" t="str">
+        <v>Bank</v>
+      </c>
+      <c r="K71" t="str">
+        <v>Bank</v>
+      </c>
+      <c r="L71" t="str">
+        <v>ACC-02</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L69"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L71"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I32"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -10788,9 +10949,38 @@
         <v>CM</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>TXN-10033-L2</v>
+      </c>
+      <c r="B32" t="str">
+        <v>ACC-02</v>
+      </c>
+      <c r="C32" t="str">
+        <v>TXN-10033</v>
+      </c>
+      <c r="D32">
+        <v>2</v>
+      </c>
+      <c r="E32" t="str">
+        <v>2026-08-21</v>
+      </c>
+      <c r="F32">
+        <v>-500</v>
+      </c>
+      <c r="G32" t="str">
+        <v>Cr</v>
+      </c>
+      <c r="H32" t="str">
+        <v>HDFC-Aluva Bank</v>
+      </c>
+      <c r="I32" t="str">
+        <v>CM</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I32"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-21T21:39:41.645Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -3676,7 +3676,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:J8"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -3687,10 +3687,7 @@
     <col min="7" max="7" width="9.83203125" customWidth="1"/>
     <col min="8" max="8" width="14.83203125" customWidth="1"/>
     <col min="9" max="9" width="16.83203125" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
-    <col min="12" max="12" width="13.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3700,7 +3697,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Recurring financial tasks and reminders — recharges, cleaning, maintenance, subscriptions — with next-due tracking. Financial ones post a voucher on pay. Records last paid date &amp; amount; can be closed as one-off.</v>
+        <v>Recurring financial tasks and reminders — recharges, cleaning, maintenance, subscriptions — with next-due tracking. Financial ones post a voucher on pay.</v>
       </c>
     </row>
     <row r="3">
@@ -3732,15 +3729,6 @@
         <v>Main Account</v>
       </c>
       <c r="J3" t="str">
-        <v>Last Paid</v>
-      </c>
-      <c r="K3" t="str">
-        <v>Last Amount</v>
-      </c>
-      <c r="L3" t="str">
-        <v>Record Status</v>
-      </c>
-      <c r="M3" t="str">
         <v>Note</v>
       </c>
     </row>
@@ -3773,15 +3761,6 @@
         <v>55008</v>
       </c>
       <c r="J4" t="str">
-        <v>2026-08-05</v>
-      </c>
-      <c r="K4">
-        <v>399</v>
-      </c>
-      <c r="L4" t="str">
-        <v>Open</v>
-      </c>
-      <c r="M4" t="str">
         <v>98xxx</v>
       </c>
     </row>
@@ -3814,15 +3793,6 @@
         <v/>
       </c>
       <c r="J5" t="str">
-        <v>2026-08-21</v>
-      </c>
-      <c r="K5">
-        <v>500</v>
-      </c>
-      <c r="L5" t="str">
-        <v>Open</v>
-      </c>
-      <c r="M5" t="str">
         <v>Ramesh</v>
       </c>
     </row>
@@ -3857,15 +3827,6 @@
       <c r="J6" t="str">
         <v/>
       </c>
-      <c r="K6" t="str">
-        <v/>
-      </c>
-      <c r="L6" t="str">
-        <v>Open</v>
-      </c>
-      <c r="M6" t="str">
-        <v/>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -3881,7 +3842,7 @@
         <v>Yearly</v>
       </c>
       <c r="E7" t="str">
-        <v/>
+        <v>2026-08-21</v>
       </c>
       <c r="F7">
         <v>25000</v>
@@ -3896,15 +3857,6 @@
         <v/>
       </c>
       <c r="J7" t="str">
-        <v>2026-07-20</v>
-      </c>
-      <c r="K7">
-        <v>25000</v>
-      </c>
-      <c r="L7" t="str">
-        <v>Closed</v>
-      </c>
-      <c r="M7" t="str">
         <v>Full exterior</v>
       </c>
     </row>
@@ -3939,26 +3891,17 @@
       <c r="J8" t="str">
         <v/>
       </c>
-      <c r="K8" t="str">
-        <v/>
-      </c>
-      <c r="L8" t="str">
-        <v>Open</v>
-      </c>
-      <c r="M8" t="str">
-        <v/>
-      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J8"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:N5"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -3971,8 +3914,9 @@
     <col min="9" max="9" width="11.83203125" customWidth="1"/>
     <col min="10" max="10" width="14.83203125" customWidth="1"/>
     <col min="11" max="11" width="18.83203125" customWidth="1"/>
-    <col min="12" max="12" width="20.83203125" customWidth="1"/>
-    <col min="13" max="13" width="10.83203125" customWidth="1"/>
+    <col min="12" max="12" width="13.83203125" customWidth="1"/>
+    <col min="13" max="13" width="13.83203125" customWidth="1"/>
+    <col min="14" max="14" width="13.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3982,7 +3926,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Accumulate costs against a project. Net accrued = debits minus credits on the event account. On completion the net total capitalises into the main account.</v>
+        <v>Accumulate costs &amp; income against a project. On completion the net total capitalises into the main account.</v>
       </c>
     </row>
     <row r="3">
@@ -4020,10 +3964,13 @@
         <v>Settlement Ref</v>
       </c>
       <c r="L3" t="str">
-        <v>Net Accrued (debit-credit)</v>
+        <v>Spent</v>
       </c>
       <c r="M3" t="str">
-        <v>Txn Count</v>
+        <v>Received</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Net Accrued</v>
       </c>
     </row>
     <row r="4">
@@ -4064,7 +4011,10 @@
         <v>285000</v>
       </c>
       <c r="M4">
-        <v>4</v>
+        <v>120000</v>
+      </c>
+      <c r="N4">
+        <v>165000</v>
       </c>
     </row>
     <row r="5">
@@ -4105,12 +4055,15 @@
         <v>150000</v>
       </c>
       <c r="M5">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="N5">
+        <v>150000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6081,7 +6034,7 @@
         <v>Theme</v>
       </c>
       <c r="B6" t="str">
-        <v>light</v>
+        <v>dark</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-08-21T21:46:47.170Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -414,7 +414,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O36"/>
+  <dimension ref="A1:O37"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2041,9 +2041,56 @@
         <v/>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>TXN-10034</v>
+      </c>
+      <c r="B37" t="str">
+        <v>2026-08-22</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Event</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Property / Land</v>
+      </c>
+      <c r="F37" t="str">
+        <v>Test</v>
+      </c>
+      <c r="G37">
+        <v>35000</v>
+      </c>
+      <c r="H37" t="str">
+        <v/>
+      </c>
+      <c r="I37" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="J37" t="str">
+        <v>Event type: Electrical</v>
+      </c>
+      <c r="K37" t="str">
+        <v/>
+      </c>
+      <c r="L37" t="str">
+        <v/>
+      </c>
+      <c r="M37" t="str">
+        <v>[{"kind":"Event","acct":"14002","sub":"ev:EVT-01","cat":"Electrical","dr":35000,"cr":0},{"kind":"Bank","acct":"11002","sub":"bank:HDFC-Aluva","cat":"","dr":0,"cr":35000}]</v>
+      </c>
+      <c r="N37" t="str">
+        <v/>
+      </c>
+      <c r="O37" t="str">
+        <v>EVT-01</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O37"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2200,10 +2247,10 @@
         <v>0</v>
       </c>
       <c r="G5">
-        <v>600</v>
+        <v>35600</v>
       </c>
       <c r="H5">
-        <v>19400</v>
+        <v>-15600</v>
       </c>
       <c r="I5" t="str">
         <v/>
@@ -3676,7 +3723,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:M8"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -3687,7 +3734,10 @@
     <col min="7" max="7" width="9.83203125" customWidth="1"/>
     <col min="8" max="8" width="14.83203125" customWidth="1"/>
     <col min="9" max="9" width="16.83203125" customWidth="1"/>
-    <col min="10" max="10" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
+    <col min="11" max="11" width="12.83203125" customWidth="1"/>
+    <col min="12" max="12" width="13.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3697,7 +3747,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Recurring financial tasks and reminders — recharges, cleaning, maintenance, subscriptions — with next-due tracking. Financial ones post a voucher on pay.</v>
+        <v>Recurring financial tasks and reminders — recharges, cleaning, maintenance, subscriptions — with next-due tracking. Financial ones post a voucher on pay. Records last paid date &amp; amount; can be closed as one-off.</v>
       </c>
     </row>
     <row r="3">
@@ -3729,6 +3779,15 @@
         <v>Main Account</v>
       </c>
       <c r="J3" t="str">
+        <v>Last Paid</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Last Amount</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Record Status</v>
+      </c>
+      <c r="M3" t="str">
         <v>Note</v>
       </c>
     </row>
@@ -3761,6 +3820,15 @@
         <v>55008</v>
       </c>
       <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v>Open</v>
+      </c>
+      <c r="M4" t="str">
         <v>98xxx</v>
       </c>
     </row>
@@ -3793,6 +3861,15 @@
         <v/>
       </c>
       <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v>Open</v>
+      </c>
+      <c r="M5" t="str">
         <v>Ramesh</v>
       </c>
     </row>
@@ -3827,6 +3904,15 @@
       <c r="J6" t="str">
         <v/>
       </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v>Open</v>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -3857,6 +3943,15 @@
         <v/>
       </c>
       <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v>Open</v>
+      </c>
+      <c r="M7" t="str">
         <v>Full exterior</v>
       </c>
     </row>
@@ -3891,17 +3986,26 @@
       <c r="J8" t="str">
         <v/>
       </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v>Open</v>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M8"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:M5"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -3914,9 +4018,8 @@
     <col min="9" max="9" width="11.83203125" customWidth="1"/>
     <col min="10" max="10" width="14.83203125" customWidth="1"/>
     <col min="11" max="11" width="18.83203125" customWidth="1"/>
-    <col min="12" max="12" width="13.83203125" customWidth="1"/>
-    <col min="13" max="13" width="13.83203125" customWidth="1"/>
-    <col min="14" max="14" width="13.83203125" customWidth="1"/>
+    <col min="12" max="12" width="20.83203125" customWidth="1"/>
+    <col min="13" max="13" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3926,7 +4029,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Accumulate costs &amp; income against a project. On completion the net total capitalises into the main account.</v>
+        <v>Accumulate costs against a project. Net accrued = debits minus credits on the event account. On completion the net total capitalises into the main account.</v>
       </c>
     </row>
     <row r="3">
@@ -3964,13 +4067,10 @@
         <v>Settlement Ref</v>
       </c>
       <c r="L3" t="str">
-        <v>Spent</v>
+        <v>Net Accrued (debit-credit)</v>
       </c>
       <c r="M3" t="str">
-        <v>Received</v>
-      </c>
-      <c r="N3" t="str">
-        <v>Net Accrued</v>
+        <v>Txn Count</v>
       </c>
     </row>
     <row r="4">
@@ -4008,13 +4108,10 @@
         <v/>
       </c>
       <c r="L4">
-        <v>285000</v>
+        <v>320000</v>
       </c>
       <c r="M4">
-        <v>120000</v>
-      </c>
-      <c r="N4">
-        <v>165000</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -4055,15 +4152,12 @@
         <v>150000</v>
       </c>
       <c r="M5">
-        <v>0</v>
-      </c>
-      <c r="N5">
-        <v>150000</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6054,7 +6148,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L37"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -7372,16 +7466,54 @@
         <v>Yes</v>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>TXN-10034</v>
+      </c>
+      <c r="B37" t="str">
+        <v>2026-08-22</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Event</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Test</v>
+      </c>
+      <c r="F37">
+        <v>35000</v>
+      </c>
+      <c r="G37" t="str">
+        <v>Direct Credit</v>
+      </c>
+      <c r="H37" t="str">
+        <v>EVT-01</v>
+      </c>
+      <c r="I37" t="str">
+        <v>Event type: Electrical</v>
+      </c>
+      <c r="J37" t="str">
+        <v/>
+      </c>
+      <c r="K37">
+        <v>2</v>
+      </c>
+      <c r="L37" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L37"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L71"/>
+  <dimension ref="A1:L73"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -10029,16 +10161,92 @@
         <v>ACC-02</v>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>TXN-10034-L1</v>
+      </c>
+      <c r="B72" t="str">
+        <v>TXN-10034</v>
+      </c>
+      <c r="C72">
+        <v>1</v>
+      </c>
+      <c r="D72">
+        <v>35000</v>
+      </c>
+      <c r="E72" t="str">
+        <v>Dr</v>
+      </c>
+      <c r="F72" t="str">
+        <v>14002</v>
+      </c>
+      <c r="G72" t="str">
+        <v>Property / Land</v>
+      </c>
+      <c r="H72" t="str">
+        <v>Asset</v>
+      </c>
+      <c r="I72" t="str">
+        <v>Fixed Assets</v>
+      </c>
+      <c r="J72" t="str">
+        <v>Event</v>
+      </c>
+      <c r="K72" t="str">
+        <v>Fixed Asset</v>
+      </c>
+      <c r="L72" t="str">
+        <v>FA-01</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>TXN-10034-L2</v>
+      </c>
+      <c r="B73" t="str">
+        <v>TXN-10034</v>
+      </c>
+      <c r="C73">
+        <v>2</v>
+      </c>
+      <c r="D73">
+        <v>-35000</v>
+      </c>
+      <c r="E73" t="str">
+        <v>Cr</v>
+      </c>
+      <c r="F73" t="str">
+        <v>11002</v>
+      </c>
+      <c r="G73" t="str">
+        <v>HDFC-Aluva Bank</v>
+      </c>
+      <c r="H73" t="str">
+        <v>Asset</v>
+      </c>
+      <c r="I73" t="str">
+        <v>Cash &amp; Bank</v>
+      </c>
+      <c r="J73" t="str">
+        <v>Bank</v>
+      </c>
+      <c r="K73" t="str">
+        <v>Bank</v>
+      </c>
+      <c r="L73" t="str">
+        <v>ACC-02</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L71"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L73"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I33"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -10931,9 +11139,38 @@
         <v>CM</v>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>TXN-10034-L2</v>
+      </c>
+      <c r="B33" t="str">
+        <v>ACC-02</v>
+      </c>
+      <c r="C33" t="str">
+        <v>TXN-10034</v>
+      </c>
+      <c r="D33">
+        <v>2</v>
+      </c>
+      <c r="E33" t="str">
+        <v>2026-08-22</v>
+      </c>
+      <c r="F33">
+        <v>-35000</v>
+      </c>
+      <c r="G33" t="str">
+        <v>Cr</v>
+      </c>
+      <c r="H33" t="str">
+        <v>HDFC-Aluva Bank</v>
+      </c>
+      <c r="I33" t="str">
+        <v>Test</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I33"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -11413,7 +11650,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -11494,16 +11731,45 @@
         <v>Expense for the well</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>TXN-10034-L1</v>
+      </c>
+      <c r="B5" t="str">
+        <v>FA-01</v>
+      </c>
+      <c r="C5" t="str">
+        <v>TXN-10034</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5" t="str">
+        <v>2026-08-22</v>
+      </c>
+      <c r="F5">
+        <v>35000</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Dr</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Property / Land</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Test</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -11681,9 +11947,35 @@
         <v>Expense for the well</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>TXN-10034-E</v>
+      </c>
+      <c r="B9" t="str">
+        <v>EVT-01</v>
+      </c>
+      <c r="C9" t="str">
+        <v>TXN-10034</v>
+      </c>
+      <c r="D9" t="str">
+        <v>2026-08-22</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Voucher</v>
+      </c>
+      <c r="F9">
+        <v>35000</v>
+      </c>
+      <c r="G9" t="str">
+        <v>debit</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Test</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>